<commit_message>
docs: define los ítems del pedido y actualiza la planificación al acuerdo de Firestore
</commit_message>
<xml_diff>
--- a/docs/SanMarkFood-Planificacion.xlsx
+++ b/docs/SanMarkFood-Planificacion.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>Ecosistema de 2 apps (Comensal y Restaurante) con backend propio compartido, para el descubrimiento, reserva y pedido de comida en restaurantes cercanos a San Marcos.</t>
+          <t>Ecosistema de 2 apps (Comensal y Restaurante) que comparten un backend en Firebase (Firestore y Cloud Functions), para el descubrimiento, reserva y pedido de comida en restaurantes cercanos a San Marcos.</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="H102" s="12" t="inlineStr">
         <is>
-          <t>Ktor (backend propio, agregación); MPAndroidChart o Vico (gráficos)</t>
+          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de locales y pedidos); Cloud Functions</t>
         </is>
       </c>
       <c r="I102" s="7" t="inlineStr">
@@ -3279,7 +3279,7 @@
       <c r="E103" s="8" t="n"/>
       <c r="F103" s="12" t="inlineStr">
         <is>
-          <t>El dashboard consume la agregación a través del backend propio (Ktor), no accede directamente a Firestore</t>
+          <t>El dashboard obtiene las métricas con consultas de agregación de Firestore (count, sum), sin backend propio; lo que no se pueda agregar así lo calcula una Cloud Function</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">

</xml_diff>

<commit_message>
[SCRUM-40] refactor: alinea el comensal con el restaurante y actualiza la planificación del Sprint 2
</commit_message>
<xml_diff>
--- a/docs/SanMarkFood-Planificacion.xlsx
+++ b/docs/SanMarkFood-Planificacion.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="FASES" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PLANIFICACION" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FASES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLANIFICACION" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -150,29 +150,29 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -545,14 +545,14 @@
   <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" s="14">
+    <row r="1" ht="22" customHeight="1" s="12">
       <c r="A1" s="17" t="inlineStr">
         <is>
           <t>FASES DE DESARROLLO</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" s="14"/>
+    <row r="2" ht="22" customHeight="1" s="12"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I2"/>
@@ -570,20 +570,20 @@
   <dimension ref="A1:K116"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="4" customWidth="1" style="14" min="1" max="1"/>
-    <col width="7" customWidth="1" style="14" min="2" max="2"/>
-    <col width="24" customWidth="1" style="14" min="3" max="3"/>
-    <col width="14" customWidth="1" style="14" min="4" max="4"/>
-    <col width="32" customWidth="1" style="14" min="5" max="5"/>
-    <col width="38" customWidth="1" style="14" min="6" max="6"/>
-    <col width="13" customWidth="1" style="14" min="7" max="7"/>
-    <col width="30" customWidth="1" style="14" min="8" max="8"/>
-    <col width="11" customWidth="1" style="14" min="9" max="10"/>
-    <col width="14" customWidth="1" style="14" min="11" max="11"/>
+    <col width="4" customWidth="1" style="12" min="1" max="1"/>
+    <col width="7" customWidth="1" style="12" min="2" max="2"/>
+    <col width="24" customWidth="1" style="12" min="3" max="3"/>
+    <col width="14" customWidth="1" style="12" min="4" max="4"/>
+    <col width="32" customWidth="1" style="12" min="5" max="5"/>
+    <col width="38" customWidth="1" style="12" min="6" max="6"/>
+    <col width="13" customWidth="1" style="12" min="7" max="7"/>
+    <col width="30" customWidth="1" style="12" min="8" max="8"/>
+    <col width="11" customWidth="1" style="12" min="9" max="10"/>
+    <col width="14" customWidth="1" style="12" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" s="14">
-      <c r="A1" s="16" t="inlineStr">
+    <row r="1" ht="24" customHeight="1" s="12">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>PLANIFICACIÓN DEL PROYECTO — San Mark Food</t>
         </is>
@@ -601,19 +601,19 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" s="14">
+    <row r="3" hidden="1" ht="30" customHeight="1" s="12">
       <c r="C3" s="1" t="inlineStr">
         <is>
           <t>DESCRIPCIÓN:</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>Ecosistema de 2 apps (Comensal y Restaurante) que comparten un backend en Firebase (Firestore y Cloud Functions), para el descubrimiento, reserva y pedido de comida en restaurantes cercanos a San Marcos.</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="1" s="12">
       <c r="C4" s="1" t="inlineStr">
         <is>
           <t>RESPONSABLES DEL PROYECTO</t>
@@ -626,7 +626,7 @@
       </c>
     </row>
     <row r="5"/>
-    <row r="6" ht="30" customHeight="1" s="14">
+    <row r="6" ht="30" customHeight="1" s="12">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Product Backlog</t>
@@ -683,75 +683,75 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1" s="14">
-      <c r="A7" s="15" t="inlineStr">
+    <row r="7" ht="45" customHeight="1" s="12">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Product Backlog</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Base, Autenticación y Gestión de Restaurante:
 Registro del restaurante, su perfil y su menú digital, incluyendo la digitalización de la carta física con IA.</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Restaurante</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>HU01 - Registro e inicio de sesión (Restaurante)
 Como restaurante, quiero registrarme e iniciar sesión, para acceder al panel de gestión de mi negocio.</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Formulario de registro con email y contraseña</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>Firebase Authentication; Jetpack Compose; ViewModel + StateFlow</t>
         </is>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>Semana 4</t>
         </is>
       </c>
-      <c r="J7" s="11" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>Semana 5</t>
         </is>
       </c>
-      <c r="K7" s="11" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>Jose Chuque</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" s="14">
+    <row r="8" ht="36" customHeight="1" s="12">
       <c r="A8" s="8" t="n"/>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="8" t="n"/>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="n"/>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>Verificación de correo electrónico antes de habilitar la cuenta</t>
         </is>
       </c>
-      <c r="G8" s="11" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -761,18 +761,18 @@
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="8" t="n"/>
     </row>
-    <row r="9" ht="36" customHeight="1" s="14">
+    <row r="9" ht="36" customHeight="1" s="12">
       <c r="A9" s="8" t="n"/>
       <c r="B9" s="8" t="n"/>
       <c r="C9" s="8" t="n"/>
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>Inicio de sesión persistente entre sesiones</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -782,18 +782,18 @@
       <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
     </row>
-    <row r="10" ht="36" customHeight="1" s="14">
+    <row r="10" ht="36" customHeight="1" s="12">
       <c r="A10" s="8" t="n"/>
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="8" t="n"/>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>Recuperación de contraseña vía correo electrónico</t>
         </is>
       </c>
-      <c r="G10" s="11" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -803,18 +803,18 @@
       <c r="J10" s="8" t="n"/>
       <c r="K10" s="8" t="n"/>
     </row>
-    <row r="11" ht="36" customHeight="1" s="14">
+    <row r="11" ht="36" customHeight="1" s="12">
       <c r="A11" s="8" t="n"/>
       <c r="B11" s="8" t="n"/>
       <c r="C11" s="8" t="n"/>
       <c r="D11" s="8" t="n"/>
       <c r="E11" s="9" t="n"/>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Campo de rol de la cuenta (restaurante, comensal o administrador), asignado en el servidor y no editable por el usuario</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -824,60 +824,60 @@
       <c r="J11" s="9" t="n"/>
       <c r="K11" s="9" t="n"/>
     </row>
-    <row r="12" ht="45" customHeight="1" s="14">
+    <row r="12" ht="45" customHeight="1" s="12">
       <c r="A12" s="8" t="n"/>
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="8" t="n"/>
       <c r="D12" s="8" t="n"/>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>HU02 - Registro y gestión de perfil de restaurante
 Como restaurante, quiero registrar los datos de mi local (nombre, dirección, horario, categoría), para que los comensales puedan encontrarme y conocer mi información básica.</t>
         </is>
       </c>
-      <c r="F12" s="10" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>Formulario de registro de local (nombre, dirección, categoría, teléfono); cada cuenta corresponde a un solo local</t>
         </is>
       </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Firestore (perfil del restaurante); Firebase Storage + Coil (fotos); Material Design 3</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>Semana 5</t>
         </is>
       </c>
-      <c r="J12" s="11" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>Semana 6</t>
         </is>
       </c>
-      <c r="K12" s="11" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>Jose Chuque</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1" s="14">
+    <row r="13" ht="36" customHeight="1" s="12">
       <c r="A13" s="8" t="n"/>
       <c r="B13" s="8" t="n"/>
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="8" t="n"/>
       <c r="E13" s="8" t="n"/>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>Configuración de horario de atención por día de la semana</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -887,18 +887,18 @@
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
     </row>
-    <row r="14" ht="36" customHeight="1" s="14">
+    <row r="14" ht="36" customHeight="1" s="12">
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="8" t="n"/>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
       <c r="E14" s="8" t="n"/>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>Subida de foto de portada y logo del local</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -908,18 +908,18 @@
       <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
     </row>
-    <row r="15" ht="36" customHeight="1" s="14">
+    <row r="15" ht="36" customHeight="1" s="12">
       <c r="A15" s="8" t="n"/>
       <c r="B15" s="8" t="n"/>
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="8" t="n"/>
       <c r="E15" s="8" t="n"/>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>Edición de los datos del perfil en cualquier momento</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -929,18 +929,18 @@
       <c r="J15" s="8" t="n"/>
       <c r="K15" s="8" t="n"/>
     </row>
-    <row r="16" ht="36" customHeight="1" s="14">
+    <row r="16" ht="36" customHeight="1" s="12">
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="8" t="n"/>
       <c r="C16" s="8" t="n"/>
       <c r="D16" s="8" t="n"/>
       <c r="E16" s="8" t="n"/>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>Estado del perfil: pendiente de aprobación, aprobado o rechazado, visible para el restaurante; mientras está pendiente puede preparar perfil, horario, fotos y carta, pero no es visible para los comensales ni recibe pedidos ni reservas</t>
         </is>
       </c>
-      <c r="G16" s="11" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -950,18 +950,18 @@
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
     </row>
-    <row r="17" ht="36" customHeight="1" s="14">
+    <row r="17" ht="36" customHeight="1" s="12">
       <c r="A17" s="8" t="n"/>
       <c r="B17" s="8" t="n"/>
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>Opción de pausar temporalmente la recepción de pedidos (marcar el local como cerrado)</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -971,18 +971,18 @@
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
     </row>
-    <row r="18" ht="36" customHeight="1" s="14">
+    <row r="18" ht="36" customHeight="1" s="12">
       <c r="A18" s="8" t="n"/>
       <c r="B18" s="8" t="n"/>
       <c r="C18" s="8" t="n"/>
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="9" t="n"/>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>Si el registro es rechazado, el local ve el motivo, corrige su perfil y lo reenvía a revisión (vuelve a pendiente)</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -992,60 +992,60 @@
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="9" t="n"/>
     </row>
-    <row r="19" ht="45" customHeight="1" s="14">
+    <row r="19" ht="45" customHeight="1" s="12">
       <c r="A19" s="8" t="n"/>
       <c r="B19" s="8" t="n"/>
       <c r="C19" s="8" t="n"/>
       <c r="D19" s="8" t="n"/>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>HU03 - Gestión de menú digital
 Como restaurante, quiero crear y editar mi menú digital con platos, precios y categorías, para mostrar mi oferta a los comensales.</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>Alta de plato (nombre, descripción, precio, categoría, foto)</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
         <is>
           <t>Firestore (colección de menú); Firebase Storage (fotos de platos); MVVM</t>
         </is>
       </c>
-      <c r="I19" s="11" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>Semana 6</t>
         </is>
       </c>
-      <c r="J19" s="11" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>Semana 7</t>
         </is>
       </c>
-      <c r="K19" s="11" t="inlineStr">
+      <c r="K19" s="7" t="inlineStr">
         <is>
           <t>Jose Chuque</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1" s="14">
+    <row r="20" ht="36" customHeight="1" s="12">
       <c r="A20" s="8" t="n"/>
       <c r="B20" s="8" t="n"/>
       <c r="C20" s="8" t="n"/>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>Edición y eliminación de platos existentes</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1055,18 +1055,18 @@
       <c r="J20" s="8" t="n"/>
       <c r="K20" s="8" t="n"/>
     </row>
-    <row r="21" ht="36" customHeight="1" s="14">
+    <row r="21" ht="36" customHeight="1" s="12">
       <c r="A21" s="8" t="n"/>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="n"/>
       <c r="E21" s="8" t="n"/>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>Organización de platos por categoría</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1076,18 +1076,18 @@
       <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
     </row>
-    <row r="22" ht="36" customHeight="1" s="14">
+    <row r="22" ht="36" customHeight="1" s="12">
       <c r="A22" s="8" t="n"/>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
       <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
-      <c r="F22" s="10" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>Marcar disponibilidad de un plato o de una opción del menú del día (disponible / agotado)</t>
         </is>
       </c>
-      <c r="G22" s="11" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1097,18 +1097,18 @@
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
     </row>
-    <row r="23" ht="36" customHeight="1" s="14">
+    <row r="23" ht="36" customHeight="1" s="12">
       <c r="A23" s="8" t="n"/>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
         <is>
           <t>Publicación diaria del menú del día (fecha, precio, opciones de entrada y de segundo, refresco y postre incluidos, y hora hasta la que se sirve, por defecto 15:00), separado de la carta fija</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1118,18 +1118,18 @@
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
     </row>
-    <row r="24" ht="36" customHeight="1" s="14">
+    <row r="24" ht="36" customHeight="1" s="12">
       <c r="A24" s="8" t="n"/>
       <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="9" t="n"/>
-      <c r="F24" s="10" t="inlineStr">
+      <c r="F24" s="11" t="inlineStr">
         <is>
           <t>El menú del día se arma desde una foto de la pizarra, copiando el de ayer o desde cero; vale solo para ese día, se puede editar tras publicarlo (los pedidos hechos conservan su precio) y terminar antes de la hora de fin</t>
         </is>
       </c>
-      <c r="G24" s="11" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1139,60 +1139,60 @@
       <c r="J24" s="9" t="n"/>
       <c r="K24" s="9" t="n"/>
     </row>
-    <row r="25" ht="45" customHeight="1" s="14">
+    <row r="25" ht="45" customHeight="1" s="12">
       <c r="A25" s="8" t="n"/>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>HU04 - Digitalización de carta física con IA
 Como restaurante, quiero tomar una foto de mi carta física impresa y que la app extraiga automáticamente los platos y precios, para digitalizar mi menú sin escribirlo manualmente.</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>Captura de foto de la carta física o de la pizarra del menú del día con la cámara del dispositivo</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H25" s="10" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>CameraX; ML Kit Text Recognition + API de un LLM (estructuración); Retrofit + corrutinas</t>
         </is>
       </c>
-      <c r="I25" s="11" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>Semana 7</t>
         </is>
       </c>
-      <c r="J25" s="11" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
         <is>
           <t>Semana 8</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
+      <c r="K25" s="7" t="inlineStr">
         <is>
           <t>Jose Chuque</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="36" customHeight="1" s="14">
+    <row r="26" ht="36" customHeight="1" s="12">
       <c r="A26" s="8" t="n"/>
       <c r="B26" s="8" t="n"/>
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="8" t="n"/>
       <c r="E26" s="8" t="n"/>
-      <c r="F26" s="10" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>Reconocimiento con IA (OCR + LLM) de platos y precios de la carta, y de las opciones de entrada y segundo del menú del día</t>
         </is>
       </c>
-      <c r="G26" s="11" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1202,18 +1202,16 @@
       <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
     </row>
-    <row r="27" ht="36" customHeight="1" s="14">
+    <row r="27" ht="36" customHeight="1" s="12">
       <c r="A27" s="8" t="n"/>
       <c r="B27" s="8" t="n"/>
       <c r="C27" s="9" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="9" t="n"/>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>Revisión y confirmación manual antes de publicar los platos extraídos</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="inlineStr">
+      <c r="F27" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1223,69 +1221,69 @@
       <c r="J27" s="9" t="n"/>
       <c r="K27" s="9" t="n"/>
     </row>
-    <row r="28" ht="45" customHeight="1" s="14">
+    <row r="28" ht="45" customHeight="1" s="12">
       <c r="A28" s="8" t="n"/>
       <c r="B28" s="8" t="n"/>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>Acceso y Aprobación de Restaurantes (Administrador):
 Inicio de sesión del administrador dentro de la App Restaurante, y aprobación de nuevos restaurantes antes de su publicación.</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>HU23 - Acceso de administrador
 Como administrador, quiero iniciar sesión con mis credenciales, para acceder a la sección de administración dentro de la App Restaurante.</t>
         </is>
       </c>
-      <c r="F28" s="10" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>Inicio de sesión con email y contraseña en la misma pantalla que los restaurantes; las cuentas de administrador se crean fuera de la app, sin registro público</t>
         </is>
       </c>
-      <c r="G28" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H28" s="10" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>Firebase Authentication (rol administrador); Jetpack Compose; ViewModel + StateFlow</t>
         </is>
       </c>
-      <c r="I28" s="11" t="inlineStr">
+      <c r="I28" s="7" t="inlineStr">
         <is>
           <t>Semana 4</t>
         </is>
       </c>
-      <c r="J28" s="11" t="inlineStr">
+      <c r="J28" s="7" t="inlineStr">
         <is>
           <t>Semana 5</t>
         </is>
       </c>
-      <c r="K28" s="11" t="inlineStr">
+      <c r="K28" s="7" t="inlineStr">
         <is>
           <t>Jose Chuque</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1" s="14">
+    <row r="29" ht="36" customHeight="1" s="12">
       <c r="A29" s="8" t="n"/>
       <c r="B29" s="8" t="n"/>
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="9" t="n"/>
-      <c r="F29" s="10" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>El sistema reconoce el rol administrador y muestra la sección de administración en vez del panel normal de restaurante</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1295,60 +1293,60 @@
       <c r="J29" s="9" t="n"/>
       <c r="K29" s="9" t="n"/>
     </row>
-    <row r="30" ht="45" customHeight="1" s="14">
+    <row r="30" ht="45" customHeight="1" s="12">
       <c r="A30" s="8" t="n"/>
       <c r="B30" s="8" t="n"/>
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="8" t="n"/>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>HU24 - Aprobación de restaurantes
 Como administrador, quiero revisar y aprobar o rechazar el registro de un nuevo restaurante, para evitar negocios falsos o duplicados antes de que sean visibles para los comensales.</t>
         </is>
       </c>
-      <c r="F30" s="10" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
         <is>
           <t>Listado de restaurantes con perfil pendiente de aprobación, con los reenvíos marcados y el motivo del rechazo anterior</t>
         </is>
       </c>
-      <c r="G30" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H30" s="10" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
         <is>
           <t>Firestore (listener de restaurantes pendientes); Firebase Cloud Messaging</t>
         </is>
       </c>
-      <c r="I30" s="11" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>Semana 5</t>
         </is>
       </c>
-      <c r="J30" s="11" t="inlineStr">
+      <c r="J30" s="7" t="inlineStr">
         <is>
           <t>Semana 6</t>
         </is>
       </c>
-      <c r="K30" s="11" t="inlineStr">
+      <c r="K30" s="7" t="inlineStr">
         <is>
           <t>Jose Chuque</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1" s="14">
+    <row r="31" ht="36" customHeight="1" s="12">
       <c r="A31" s="8" t="n"/>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="8" t="n"/>
       <c r="E31" s="8" t="n"/>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>Aprobar o rechazar un restaurante nuevo; el rechazo exige un motivo de una lista (datos incompletos, dirección no verificable, local duplicado) u «Otro» con texto</t>
         </is>
       </c>
-      <c r="G31" s="11" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1358,18 +1356,18 @@
       <c r="J31" s="8" t="n"/>
       <c r="K31" s="8" t="n"/>
     </row>
-    <row r="32" ht="36" customHeight="1" s="14">
+    <row r="32" ht="36" customHeight="1" s="12">
       <c r="A32" s="8" t="n"/>
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="9" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="9" t="n"/>
-      <c r="F32" s="10" t="inlineStr">
+      <c r="F32" s="11" t="inlineStr">
         <is>
           <t>Notificación al restaurante con el resultado de la revisión</t>
         </is>
       </c>
-      <c r="G32" s="11" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1379,69 +1377,69 @@
       <c r="J32" s="9" t="n"/>
       <c r="K32" s="9" t="n"/>
     </row>
-    <row r="33" ht="45" customHeight="1" s="14">
+    <row r="33" ht="45" customHeight="1" s="12">
       <c r="A33" s="8" t="n"/>
       <c r="B33" s="8" t="n"/>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Base, Autenticación, Descubrimiento y Perfil del Comensal:
 Registro del comensal, gestión de su perfil, y primera versión de la búsqueda de restaurantes cercanos.</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Comensal</t>
         </is>
       </c>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
         <is>
           <t>HU05 - Registro e inicio de sesión (Comensal)
 Como comensal, quiero registrarme e iniciar sesión, para acceder a la app y guardar mi actividad (pedidos, reservas, reseñas).</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>Formulario de registro con email y contraseña</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H33" s="10" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
         <is>
           <t>Firebase Authentication; Jetpack Compose; ViewModel + StateFlow</t>
         </is>
       </c>
-      <c r="I33" s="11" t="inlineStr">
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>Semana 4</t>
         </is>
       </c>
-      <c r="J33" s="11" t="inlineStr">
+      <c r="J33" s="7" t="inlineStr">
         <is>
           <t>Semana 5</t>
         </is>
       </c>
-      <c r="K33" s="11" t="inlineStr">
+      <c r="K33" s="7" t="inlineStr">
         <is>
           <t>Camila Bada</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="36" customHeight="1" s="14">
+    <row r="34" ht="36" customHeight="1" s="12">
       <c r="A34" s="8" t="n"/>
       <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="n"/>
       <c r="E34" s="8" t="n"/>
-      <c r="F34" s="10" t="inlineStr">
+      <c r="F34" s="11" t="inlineStr">
         <is>
           <t>Verificación de correo electrónico antes de habilitar la cuenta</t>
         </is>
       </c>
-      <c r="G34" s="11" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1451,18 +1449,18 @@
       <c r="J34" s="8" t="n"/>
       <c r="K34" s="8" t="n"/>
     </row>
-    <row r="35" ht="36" customHeight="1" s="14">
+    <row r="35" ht="36" customHeight="1" s="12">
       <c r="A35" s="8" t="n"/>
       <c r="B35" s="8" t="n"/>
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="n"/>
       <c r="E35" s="8" t="n"/>
-      <c r="F35" s="10" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>Inicio de sesión persistente entre sesiones</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1472,18 +1470,18 @@
       <c r="J35" s="8" t="n"/>
       <c r="K35" s="8" t="n"/>
     </row>
-    <row r="36" ht="36" customHeight="1" s="14">
+    <row r="36" ht="36" customHeight="1" s="12">
       <c r="A36" s="8" t="n"/>
       <c r="B36" s="8" t="n"/>
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="8" t="n"/>
       <c r="E36" s="8" t="n"/>
-      <c r="F36" s="10" t="inlineStr">
+      <c r="F36" s="11" t="inlineStr">
         <is>
           <t>Recuperación de contraseña vía correo electrónico</t>
         </is>
       </c>
-      <c r="G36" s="11" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1493,18 +1491,18 @@
       <c r="J36" s="8" t="n"/>
       <c r="K36" s="8" t="n"/>
     </row>
-    <row r="37" ht="36" customHeight="1" s="14">
+    <row r="37" ht="36" customHeight="1" s="12">
       <c r="A37" s="8" t="n"/>
       <c r="B37" s="8" t="n"/>
       <c r="C37" s="8" t="n"/>
       <c r="D37" s="8" t="n"/>
       <c r="E37" s="9" t="n"/>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>Exploración sin cuenta: mapa, menús y reseñas son visibles sin iniciar sesión; pedir, reservar y usar el asistente exigen sesión, y al iniciarla se vuelve a la pantalla de origen conservando el carrito</t>
         </is>
       </c>
-      <c r="G37" s="11" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1514,60 +1512,60 @@
       <c r="J37" s="9" t="n"/>
       <c r="K37" s="9" t="n"/>
     </row>
-    <row r="38" ht="45" customHeight="1" s="14">
+    <row r="38" ht="45" customHeight="1" s="12">
       <c r="A38" s="8" t="n"/>
       <c r="B38" s="8" t="n"/>
       <c r="C38" s="8" t="n"/>
       <c r="D38" s="8" t="n"/>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>HU19 - Gestión de perfil del comensal
 Como comensal, quiero gestionar mi perfil (nombre, foto, teléfono, direcciones frecuentes), para mantener mis datos actualizados y agilizar mis pedidos y reservas.</t>
         </is>
       </c>
-      <c r="F38" s="10" t="inlineStr">
+      <c r="F38" s="11" t="inlineStr">
         <is>
           <t>Edición de nombre, foto y teléfono</t>
         </is>
       </c>
-      <c r="G38" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H38" s="10" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
         <is>
           <t>Firestore (perfil del comensal); Firebase Storage + Coil (foto); Jetpack Compose</t>
         </is>
       </c>
-      <c r="I38" s="11" t="inlineStr">
+      <c r="I38" s="7" t="inlineStr">
         <is>
           <t>Semana 5</t>
         </is>
       </c>
-      <c r="J38" s="11" t="inlineStr">
+      <c r="J38" s="7" t="inlineStr">
         <is>
           <t>Semana 6</t>
         </is>
       </c>
-      <c r="K38" s="11" t="inlineStr">
+      <c r="K38" s="7" t="inlineStr">
         <is>
           <t>Camila Bada</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="36" customHeight="1" s="14">
+    <row r="39" ht="36" customHeight="1" s="12">
       <c r="A39" s="8" t="n"/>
       <c r="B39" s="8" t="n"/>
       <c r="C39" s="8" t="n"/>
       <c r="D39" s="8" t="n"/>
       <c r="E39" s="8" t="n"/>
-      <c r="F39" s="10" t="inlineStr">
+      <c r="F39" s="11" t="inlineStr">
         <is>
           <t>Registro de una o más direcciones frecuentes para delivery</t>
         </is>
       </c>
-      <c r="G39" s="11" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1577,18 +1575,18 @@
       <c r="J39" s="8" t="n"/>
       <c r="K39" s="8" t="n"/>
     </row>
-    <row r="40" ht="36" customHeight="1" s="14">
+    <row r="40" ht="36" customHeight="1" s="12">
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="8" t="n"/>
       <c r="C40" s="8" t="n"/>
       <c r="D40" s="8" t="n"/>
       <c r="E40" s="8" t="n"/>
-      <c r="F40" s="10" t="inlineStr">
+      <c r="F40" s="11" t="inlineStr">
         <is>
           <t>Los cambios se reflejan de inmediato en pedidos y reservas futuras</t>
         </is>
       </c>
-      <c r="G40" s="11" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1598,18 +1596,18 @@
       <c r="J40" s="8" t="n"/>
       <c r="K40" s="8" t="n"/>
     </row>
-    <row r="41" ht="36" customHeight="1" s="14">
+    <row r="41" ht="36" customHeight="1" s="12">
       <c r="A41" s="8" t="n"/>
       <c r="B41" s="8" t="n"/>
       <c r="C41" s="8" t="n"/>
       <c r="D41" s="8" t="n"/>
       <c r="E41" s="8" t="n"/>
-      <c r="F41" s="10" t="inlineStr">
+      <c r="F41" s="11" t="inlineStr">
         <is>
           <t>Preferencias de notificaciones: el comensal puede desactivar los avisos de reservas y de respuestas a sus reseñas; los avisos de estado de un pedido en curso no se pueden desactivar</t>
         </is>
       </c>
-      <c r="G41" s="11" t="inlineStr">
+      <c r="G41" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1619,18 +1617,18 @@
       <c r="J41" s="8" t="n"/>
       <c r="K41" s="8" t="n"/>
     </row>
-    <row r="42" ht="36" customHeight="1" s="14">
+    <row r="42" ht="36" customHeight="1" s="12">
       <c r="A42" s="8" t="n"/>
       <c r="B42" s="8" t="n"/>
       <c r="C42" s="8" t="n"/>
       <c r="D42" s="8" t="n"/>
       <c r="E42" s="9" t="n"/>
-      <c r="F42" s="10" t="inlineStr">
+      <c r="F42" s="11" t="inlineStr">
         <is>
           <t>La app sigue el modo claro u oscuro del sistema, con la paleta de San Mark Food en ambos temas (incluido el estilo del mapa)</t>
         </is>
       </c>
-      <c r="G42" s="11" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1640,60 +1638,60 @@
       <c r="J42" s="9" t="n"/>
       <c r="K42" s="9" t="n"/>
     </row>
-    <row r="43" ht="45" customHeight="1" s="14">
+    <row r="43" ht="45" customHeight="1" s="12">
       <c r="A43" s="8" t="n"/>
       <c r="B43" s="8" t="n"/>
       <c r="C43" s="8" t="n"/>
       <c r="D43" s="8" t="n"/>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="E43" s="11" t="inlineStr">
         <is>
           <t>HU06 - Búsqueda y descubrimiento de restaurantes cercanos
 Como comensal, quiero ver los restaurantes cercanos a mi ubicación con filtros por categoría y precio, para decidir dónde comer.</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
+      <c r="F43" s="11" t="inlineStr">
         <is>
           <t>Listado de restaurantes ordenado por cercanía a la ubicación del usuario</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H43" s="10" t="inlineStr">
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
         <is>
           <t>FusedLocationProviderClient (GPS); Retrofit + corrutinas (Google Places/Maps API); Maps SDK</t>
         </is>
       </c>
-      <c r="I43" s="11" t="inlineStr">
+      <c r="I43" s="7" t="inlineStr">
         <is>
           <t>Semana 6</t>
         </is>
       </c>
-      <c r="J43" s="11" t="inlineStr">
+      <c r="J43" s="7" t="inlineStr">
         <is>
           <t>Semana 7</t>
         </is>
       </c>
-      <c r="K43" s="11" t="inlineStr">
+      <c r="K43" s="7" t="inlineStr">
         <is>
           <t>Camila Bada</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="36" customHeight="1" s="14">
+    <row r="44" ht="36" customHeight="1" s="12">
       <c r="A44" s="8" t="n"/>
       <c r="B44" s="8" t="n"/>
       <c r="C44" s="8" t="n"/>
       <c r="D44" s="8" t="n"/>
       <c r="E44" s="8" t="n"/>
-      <c r="F44" s="10" t="inlineStr">
+      <c r="F44" s="11" t="inlineStr">
         <is>
           <t>Filtro por categoría, rango de precio y calificación</t>
         </is>
       </c>
-      <c r="G44" s="11" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1703,18 +1701,18 @@
       <c r="J44" s="8" t="n"/>
       <c r="K44" s="8" t="n"/>
     </row>
-    <row r="45" ht="36" customHeight="1" s="14">
+    <row r="45" ht="36" customHeight="1" s="12">
       <c r="A45" s="8" t="n"/>
       <c r="B45" s="8" t="n"/>
       <c r="C45" s="8" t="n"/>
       <c r="D45" s="8" t="n"/>
       <c r="E45" s="8" t="n"/>
-      <c r="F45" s="10" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
         <is>
           <t>Vista de detalle de restaurante con menú, horario y ubicación en mapa</t>
         </is>
       </c>
-      <c r="G45" s="11" t="inlineStr">
+      <c r="G45" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1724,18 +1722,18 @@
       <c r="J45" s="8" t="n"/>
       <c r="K45" s="8" t="n"/>
     </row>
-    <row r="46" ht="36" customHeight="1" s="14">
+    <row r="46" ht="36" customHeight="1" s="12">
       <c r="A46" s="8" t="n"/>
       <c r="B46" s="8" t="n"/>
       <c r="C46" s="8" t="n"/>
       <c r="D46" s="8" t="n"/>
       <c r="E46" s="8" t="n"/>
-      <c r="F46" s="10" t="inlineStr">
+      <c r="F46" s="11" t="inlineStr">
         <is>
           <t>El listado solo incluye restaurantes aprobados por el administrador</t>
         </is>
       </c>
-      <c r="G46" s="11" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1745,18 +1743,18 @@
       <c r="J46" s="8" t="n"/>
       <c r="K46" s="8" t="n"/>
     </row>
-    <row r="47" ht="36" customHeight="1" s="14">
+    <row r="47" ht="36" customHeight="1" s="12">
       <c r="A47" s="8" t="n"/>
       <c r="B47" s="9" t="n"/>
       <c r="C47" s="9" t="n"/>
       <c r="D47" s="9" t="n"/>
       <c r="E47" s="9" t="n"/>
-      <c r="F47" s="10" t="inlineStr">
+      <c r="F47" s="11" t="inlineStr">
         <is>
           <t>Vista principal con mapa y lista deslizable sincronizados; cada pin muestra el precio del menú del día (o «Carta» / «Cerrado»)</t>
         </is>
       </c>
-      <c r="G47" s="11" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1766,71 +1764,71 @@
       <c r="J47" s="9" t="n"/>
       <c r="K47" s="9" t="n"/>
     </row>
-    <row r="48" ht="45" customHeight="1" s="14">
+    <row r="48" ht="45" customHeight="1" s="12">
       <c r="A48" s="8" t="n"/>
-      <c r="B48" s="7" t="n">
+      <c r="B48" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C48" s="10" t="inlineStr">
         <is>
           <t>Backend Propio y Pedidos:
 Backend compartido por ambas apps, y el proceso de pedido completo: armado, pago, seguimiento y atención del lado del restaurante.</t>
         </is>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D48" s="10" t="inlineStr">
         <is>
           <t>Backend / Comensal / Restaurante</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="14" t="inlineStr">
         <is>
           <t>HU07 - Backend propio para pedidos y reservas
 Como equipo, necesitamos un backend propio que centralice la lógica de pedidos y reservas, para procesarlos de forma confiable y consistente entre ambas apps.</t>
         </is>
       </c>
-      <c r="F48" s="12" t="inlineStr">
-        <is>
-          <t>API REST con Ktor para creación y consulta de pedidos y reservas</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H48" s="12" t="inlineStr">
-        <is>
-          <t>Ktor; Exposed (ORM); PostgreSQL/H2; Retrofit + corrutinas desde ambas apps</t>
-        </is>
-      </c>
-      <c r="I48" s="7" t="inlineStr">
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>Cloud Functions HTTPS para crear y consultar pedidos y reservas, llamadas desde ambas apps con Retrofit</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H48" s="14" t="inlineStr">
+        <is>
+          <t>Cloud Functions for Firebase (HTTPS y programadas); Firestore; Retrofit + corrutinas desde ambas apps</t>
+        </is>
+      </c>
+      <c r="I48" s="10" t="inlineStr">
         <is>
           <t>Semana 9</t>
         </is>
       </c>
-      <c r="J48" s="7" t="inlineStr">
+      <c r="J48" s="10" t="inlineStr">
         <is>
           <t>Semana 10</t>
         </is>
       </c>
-      <c r="K48" s="7" t="inlineStr">
+      <c r="K48" s="10" t="inlineStr">
         <is>
           <t>Rodrigo Puente</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="36" customHeight="1" s="14">
+    <row r="49" ht="36" customHeight="1" s="12">
       <c r="A49" s="8" t="n"/>
       <c r="B49" s="8" t="n"/>
       <c r="C49" s="8" t="n"/>
       <c r="D49" s="8" t="n"/>
       <c r="E49" s="8" t="n"/>
-      <c r="F49" s="12" t="inlineStr">
-        <is>
-          <t>Persistencia de datos con Exposed ORM sobre una base de datos relacional</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>Persistencia de pedidos y reservas en Firestore, con reglas que solo permiten crearlos y cambiarlos desde las Cloud Functions</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1840,18 +1838,18 @@
       <c r="J49" s="8" t="n"/>
       <c r="K49" s="8" t="n"/>
     </row>
-    <row r="50" ht="36" customHeight="1" s="14">
+    <row r="50" ht="36" customHeight="1" s="12">
       <c r="A50" s="8" t="n"/>
       <c r="B50" s="8" t="n"/>
       <c r="C50" s="8" t="n"/>
       <c r="D50" s="8" t="n"/>
       <c r="E50" s="9" t="n"/>
-      <c r="F50" s="12" t="inlineStr">
-        <is>
-          <t>Despliegue del backend en un servicio en la nube accesible desde ambas apps</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>Despliegue de las Cloud Functions en Firebase (plan Blaze), accesibles desde ambas apps</t>
+        </is>
+      </c>
+      <c r="G50" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1861,60 +1859,60 @@
       <c r="J50" s="9" t="n"/>
       <c r="K50" s="9" t="n"/>
     </row>
-    <row r="51" ht="45" customHeight="1" s="14">
+    <row r="51" ht="45" customHeight="1" s="12">
       <c r="A51" s="8" t="n"/>
       <c r="B51" s="8" t="n"/>
       <c r="C51" s="8" t="n"/>
       <c r="D51" s="8" t="n"/>
-      <c r="E51" s="12" t="inlineStr">
+      <c r="E51" s="14" t="inlineStr">
         <is>
           <t>HU08 - Pedido con pago y calificación (Comensal)
 Como comensal, quiero armar un pedido, confirmarlo con mi huella o rostro antes de pagar, ver su estado en tiempo real y calificarlo al finalizar, para pedir con seguridad y ayudar a otros usuarios con mi opinión.</t>
         </is>
       </c>
-      <c r="F51" s="12" t="inlineStr">
+      <c r="F51" s="14" t="inlineStr">
         <is>
           <t>Armado de pedido desde el menú con carrito de compras; el carrito admite platos de un solo local y, al agregar de otro, se pide confirmar si se vacía el pedido actual</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H51" s="12" t="inlineStr">
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H51" s="14" t="inlineStr">
         <is>
           <t>BiometricPrompt (androidx.biometric); Firestore (estado en tiempo real); Room (carrito local); Retrofit (backend propio)</t>
         </is>
       </c>
-      <c r="I51" s="7" t="inlineStr">
+      <c r="I51" s="10" t="inlineStr">
         <is>
           <t>Semana 10</t>
         </is>
       </c>
-      <c r="J51" s="7" t="inlineStr">
+      <c r="J51" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="K51" s="7" t="inlineStr">
-        <is>
-          <t>Rodrigo Puente</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="36" customHeight="1" s="14">
+      <c r="K51" s="10" t="inlineStr">
+        <is>
+          <t>Camila Bada</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="36" customHeight="1" s="12">
       <c r="A52" s="8" t="n"/>
       <c r="B52" s="8" t="n"/>
       <c r="C52" s="8" t="n"/>
       <c r="D52" s="8" t="n"/>
       <c r="E52" s="8" t="n"/>
-      <c r="F52" s="12" t="inlineStr">
+      <c r="F52" s="14" t="inlineStr">
         <is>
           <t>Selección de modalidad (recojo o delivery) y método de pago</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G52" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1924,18 +1922,18 @@
       <c r="J52" s="8" t="n"/>
       <c r="K52" s="8" t="n"/>
     </row>
-    <row r="53" ht="36" customHeight="1" s="14">
+    <row r="53" ht="36" customHeight="1" s="12">
       <c r="A53" s="8" t="n"/>
       <c r="B53" s="8" t="n"/>
       <c r="C53" s="8" t="n"/>
       <c r="D53" s="8" t="n"/>
       <c r="E53" s="8" t="n"/>
-      <c r="F53" s="12" t="inlineStr">
+      <c r="F53" s="14" t="inlineStr">
         <is>
           <t>Confirmación biométrica (huella o rostro) antes de procesar el pago con billetera o tarjeta; el pago en efectivo se confirma sin biometría</t>
         </is>
       </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="G53" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1945,18 +1943,18 @@
       <c r="J53" s="8" t="n"/>
       <c r="K53" s="8" t="n"/>
     </row>
-    <row r="54" ht="36" customHeight="1" s="14">
+    <row r="54" ht="36" customHeight="1" s="12">
       <c r="A54" s="8" t="n"/>
       <c r="B54" s="8" t="n"/>
       <c r="C54" s="8" t="n"/>
       <c r="D54" s="8" t="n"/>
       <c r="E54" s="8" t="n"/>
-      <c r="F54" s="12" t="inlineStr">
+      <c r="F54" s="14" t="inlineStr">
         <is>
           <t>Seguimiento del estado del pedido en tiempo real</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G54" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1966,18 +1964,18 @@
       <c r="J54" s="8" t="n"/>
       <c r="K54" s="8" t="n"/>
     </row>
-    <row r="55" ht="36" customHeight="1" s="14">
+    <row r="55" ht="36" customHeight="1" s="12">
       <c r="A55" s="8" t="n"/>
       <c r="B55" s="8" t="n"/>
       <c r="C55" s="8" t="n"/>
       <c r="D55" s="8" t="n"/>
       <c r="E55" s="8" t="n"/>
-      <c r="F55" s="12" t="inlineStr">
+      <c r="F55" s="14" t="inlineStr">
         <is>
           <t>Calificación por pedido al finalizar: estrellas y comentario para el local, y «me gustó / no me gustó» opcional por cada plato</t>
         </is>
       </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="G55" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -1987,18 +1985,18 @@
       <c r="J55" s="8" t="n"/>
       <c r="K55" s="8" t="n"/>
     </row>
-    <row r="56" ht="36" customHeight="1" s="14">
+    <row r="56" ht="36" customHeight="1" s="12">
       <c r="A56" s="8" t="n"/>
       <c r="B56" s="8" t="n"/>
       <c r="C56" s="8" t="n"/>
       <c r="D56" s="8" t="n"/>
       <c r="E56" s="8" t="n"/>
-      <c r="F56" s="12" t="inlineStr">
+      <c r="F56" s="14" t="inlineStr">
         <is>
           <t>Cancelación del pedido por el comensal, siempre que el restaurante aún no lo haya aceptado</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G56" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2008,18 +2006,18 @@
       <c r="J56" s="8" t="n"/>
       <c r="K56" s="8" t="n"/>
     </row>
-    <row r="57" ht="36" customHeight="1" s="14">
+    <row r="57" ht="36" customHeight="1" s="12">
       <c r="A57" s="8" t="n"/>
       <c r="B57" s="8" t="n"/>
       <c r="C57" s="8" t="n"/>
       <c r="D57" s="8" t="n"/>
       <c r="E57" s="8" t="n"/>
-      <c r="F57" s="12" t="inlineStr">
+      <c r="F57" s="14" t="inlineStr">
         <is>
           <t>Armado del menú del día eligiendo 1 entrada y 1 segundo (refresco y postre incluidos); las opciones agotadas no se pueden elegir</t>
         </is>
       </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="G57" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2029,18 +2027,18 @@
       <c r="J57" s="8" t="n"/>
       <c r="K57" s="8" t="n"/>
     </row>
-    <row r="58" ht="36" customHeight="1" s="14">
+    <row r="58" ht="36" customHeight="1" s="12">
       <c r="A58" s="8" t="n"/>
       <c r="B58" s="8" t="n"/>
       <c r="C58" s="8" t="n"/>
       <c r="D58" s="8" t="n"/>
       <c r="E58" s="8" t="n"/>
-      <c r="F58" s="12" t="inlineStr">
+      <c r="F58" s="14" t="inlineStr">
         <is>
           <t>Estado «Rechazado» en el seguimiento: muestra el motivo del restaurante (o el rechazo automático a los 10 min) e informa la reversión del pago simulado</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G58" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2050,18 +2048,18 @@
       <c r="J58" s="8" t="n"/>
       <c r="K58" s="8" t="n"/>
     </row>
-    <row r="59" ht="36" customHeight="1" s="14">
+    <row r="59" ht="36" customHeight="1" s="12">
       <c r="A59" s="8" t="n"/>
       <c r="B59" s="8" t="n"/>
       <c r="C59" s="8" t="n"/>
       <c r="D59" s="8" t="n"/>
       <c r="E59" s="9" t="n"/>
-      <c r="F59" s="12" t="inlineStr">
+      <c r="F59" s="14" t="inlineStr">
         <is>
           <t>El menú del día solo se puede pedir hasta la hora de fin publicada o hasta que se agoten sus entradas o segundos; si vence con el menú en el pedido, se avisa al confirmar y se retira del pedido</t>
         </is>
       </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="G59" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2071,60 +2069,60 @@
       <c r="J59" s="9" t="n"/>
       <c r="K59" s="9" t="n"/>
     </row>
-    <row r="60" ht="45" customHeight="1" s="14">
+    <row r="60" ht="45" customHeight="1" s="12">
       <c r="A60" s="8" t="n"/>
       <c r="B60" s="8" t="n"/>
       <c r="C60" s="8" t="n"/>
       <c r="D60" s="8" t="n"/>
-      <c r="E60" s="12" t="inlineStr">
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t>HU09 - Gestión de pedidos entrantes (Restaurante)
 Como restaurante, quiero ver los pedidos entrantes y actualizar su estado, para que el comensal sepa cuándo estará listo su pedido.</t>
         </is>
       </c>
-      <c r="F60" s="12" t="inlineStr">
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>Listado de pedidos entrantes ordenado por hora de llegada</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H60" s="12" t="inlineStr">
+      <c r="G60" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H60" s="14" t="inlineStr">
         <is>
           <t>Firestore (listener en tiempo real); WorkManager (sincronización en background); Firebase Cloud Messaging</t>
         </is>
       </c>
-      <c r="I60" s="7" t="inlineStr">
+      <c r="I60" s="10" t="inlineStr">
         <is>
           <t>Semana 10</t>
         </is>
       </c>
-      <c r="J60" s="7" t="inlineStr">
+      <c r="J60" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="K60" s="7" t="inlineStr">
-        <is>
-          <t>Rodrigo Puente</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="36" customHeight="1" s="14">
+      <c r="K60" s="10" t="inlineStr">
+        <is>
+          <t>Jose Chuque</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="36" customHeight="1" s="12">
       <c r="A61" s="8" t="n"/>
       <c r="B61" s="8" t="n"/>
       <c r="C61" s="8" t="n"/>
       <c r="D61" s="8" t="n"/>
       <c r="E61" s="8" t="n"/>
-      <c r="F61" s="12" t="inlineStr">
+      <c r="F61" s="14" t="inlineStr">
         <is>
           <t>Cambio de estado del pedido (recibido, preparando, listo/en camino, entregado)</t>
         </is>
       </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="G61" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2134,18 +2132,18 @@
       <c r="J61" s="8" t="n"/>
       <c r="K61" s="8" t="n"/>
     </row>
-    <row r="62" ht="36" customHeight="1" s="14">
+    <row r="62" ht="36" customHeight="1" s="12">
       <c r="A62" s="8" t="n"/>
       <c r="B62" s="8" t="n"/>
       <c r="C62" s="8" t="n"/>
       <c r="D62" s="8" t="n"/>
       <c r="E62" s="8" t="n"/>
-      <c r="F62" s="12" t="inlineStr">
+      <c r="F62" s="14" t="inlineStr">
         <is>
           <t>Notificación push al comensal cuando cambia el estado</t>
         </is>
       </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="G62" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2155,18 +2153,18 @@
       <c r="J62" s="8" t="n"/>
       <c r="K62" s="8" t="n"/>
     </row>
-    <row r="63" ht="36" customHeight="1" s="14">
+    <row r="63" ht="36" customHeight="1" s="12">
       <c r="A63" s="8" t="n"/>
       <c r="B63" s="8" t="n"/>
       <c r="C63" s="8" t="n"/>
       <c r="D63" s="8" t="n"/>
       <c r="E63" s="8" t="n"/>
-      <c r="F63" s="12" t="inlineStr">
+      <c r="F63" s="14" t="inlineStr">
         <is>
           <t>Rechazo de un pedido entrante con motivo obligatorio (plato agotado, cocina saturada, local por cerrar u otro)</t>
         </is>
       </c>
-      <c r="G63" s="7" t="inlineStr">
+      <c r="G63" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2176,18 +2174,18 @@
       <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="n"/>
     </row>
-    <row r="64" ht="36" customHeight="1" s="14">
+    <row r="64" ht="36" customHeight="1" s="12">
       <c r="A64" s="8" t="n"/>
       <c r="B64" s="8" t="n"/>
       <c r="C64" s="8" t="n"/>
       <c r="D64" s="8" t="n"/>
       <c r="E64" s="8" t="n"/>
-      <c r="F64" s="12" t="inlineStr">
+      <c r="F64" s="14" t="inlineStr">
         <is>
           <t>Rechazo automático del pedido si el restaurante no lo acepta en 10 minutos, con aviso push al comensal</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G64" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2197,18 +2195,18 @@
       <c r="J64" s="8" t="n"/>
       <c r="K64" s="8" t="n"/>
     </row>
-    <row r="65" ht="36" customHeight="1" s="14">
+    <row r="65" ht="36" customHeight="1" s="12">
       <c r="A65" s="8" t="n"/>
       <c r="B65" s="8" t="n"/>
       <c r="C65" s="8" t="n"/>
       <c r="D65" s="8" t="n"/>
       <c r="E65" s="8" t="n"/>
-      <c r="F65" s="12" t="inlineStr">
+      <c r="F65" s="14" t="inlineStr">
         <is>
           <t>Aviso de pedido nuevo con notificación de alta prioridad y sonido que se repite hasta abrirlo, y cuenta regresiva de los 10 min en la app</t>
         </is>
       </c>
-      <c r="G65" s="7" t="inlineStr">
+      <c r="G65" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2218,18 +2216,18 @@
       <c r="J65" s="8" t="n"/>
       <c r="K65" s="8" t="n"/>
     </row>
-    <row r="66" ht="36" customHeight="1" s="14">
+    <row r="66" ht="36" customHeight="1" s="12">
       <c r="A66" s="8" t="n"/>
       <c r="B66" s="8" t="n"/>
       <c r="C66" s="8" t="n"/>
       <c r="D66" s="8" t="n"/>
       <c r="E66" s="8" t="n"/>
-      <c r="F66" s="12" t="inlineStr">
+      <c r="F66" s="14" t="inlineStr">
         <is>
           <t>Al aceptar un pedido, el local elige el tiempo estimado (10, 15, 20 o 30 min), con el que se calcula la hora que ve el comensal</t>
         </is>
       </c>
-      <c r="G66" s="7" t="inlineStr">
+      <c r="G66" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2239,18 +2237,18 @@
       <c r="J66" s="8" t="n"/>
       <c r="K66" s="8" t="n"/>
     </row>
-    <row r="67" ht="36" customHeight="1" s="14">
+    <row r="67" ht="36" customHeight="1" s="12">
       <c r="A67" s="8" t="n"/>
       <c r="B67" s="8" t="n"/>
       <c r="C67" s="9" t="n"/>
       <c r="D67" s="9" t="n"/>
       <c r="E67" s="9" t="n"/>
-      <c r="F67" s="12" t="inlineStr">
+      <c r="F67" s="14" t="inlineStr">
         <is>
           <t>Entrega de pedidos de recojo escribiendo el código de 4 dígitos del comensal; sin código se puede marcar entregado con confirmación</t>
         </is>
       </c>
-      <c r="G67" s="7" t="inlineStr">
+      <c r="G67" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2260,69 +2258,69 @@
       <c r="J67" s="9" t="n"/>
       <c r="K67" s="9" t="n"/>
     </row>
-    <row r="68" ht="45" customHeight="1" s="14">
+    <row r="68" ht="45" customHeight="1" s="12">
       <c r="A68" s="8" t="n"/>
       <c r="B68" s="8" t="n"/>
-      <c r="C68" s="7" t="inlineStr">
+      <c r="C68" s="10" t="inlineStr">
         <is>
           <t>Reservas:
 Solicitud de reserva por el comensal y su gestión por parte del restaurante.</t>
         </is>
       </c>
-      <c r="D68" s="7" t="inlineStr">
+      <c r="D68" s="10" t="inlineStr">
         <is>
           <t>Comensal / Restaurante</t>
         </is>
       </c>
-      <c r="E68" s="12" t="inlineStr">
+      <c r="E68" s="14" t="inlineStr">
         <is>
           <t>HU10 - Reserva de mesa (Comensal)
 Como comensal, quiero reservar una mesa en un restaurante para una fecha y hora determinada, para asegurar mi lugar antes de llegar.</t>
         </is>
       </c>
-      <c r="F68" s="12" t="inlineStr">
+      <c r="F68" s="14" t="inlineStr">
         <is>
           <t>Selección de fecha, hora y número de comensales: entre 2 h y 7 días de anticipación, horarios cada 30 min dentro del horario del local, de 1 a 10 comensales y máximo 2 reservas activas por comensal</t>
         </is>
       </c>
-      <c r="G68" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H68" s="12" t="inlineStr">
+      <c r="G68" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H68" s="14" t="inlineStr">
         <is>
           <t>WorkManager (recordatorios); Firebase Cloud Messaging; Firestore</t>
         </is>
       </c>
-      <c r="I68" s="7" t="inlineStr">
+      <c r="I68" s="10" t="inlineStr">
         <is>
           <t>Semana 9</t>
         </is>
       </c>
-      <c r="J68" s="7" t="inlineStr">
+      <c r="J68" s="10" t="inlineStr">
         <is>
           <t>Semana 10</t>
         </is>
       </c>
-      <c r="K68" s="7" t="inlineStr">
+      <c r="K68" s="10" t="inlineStr">
         <is>
           <t>Camila Bada</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="36" customHeight="1" s="14">
+    <row r="69" ht="36" customHeight="1" s="12">
       <c r="A69" s="8" t="n"/>
       <c r="B69" s="8" t="n"/>
       <c r="C69" s="8" t="n"/>
       <c r="D69" s="8" t="n"/>
       <c r="E69" s="8" t="n"/>
-      <c r="F69" s="12" t="inlineStr">
+      <c r="F69" s="14" t="inlineStr">
         <is>
           <t>Recordatorio de la reserva antes de la hora programada, con anticipación elegible (30 min, 1 h o 2 h)</t>
         </is>
       </c>
-      <c r="G69" s="7" t="inlineStr">
+      <c r="G69" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2332,18 +2330,18 @@
       <c r="J69" s="8" t="n"/>
       <c r="K69" s="8" t="n"/>
     </row>
-    <row r="70" ht="36" customHeight="1" s="14">
+    <row r="70" ht="36" customHeight="1" s="12">
       <c r="A70" s="8" t="n"/>
       <c r="B70" s="8" t="n"/>
       <c r="C70" s="8" t="n"/>
       <c r="D70" s="8" t="n"/>
       <c r="E70" s="8" t="n"/>
-      <c r="F70" s="12" t="inlineStr">
+      <c r="F70" s="14" t="inlineStr">
         <is>
           <t>Cancelación de la reserva desde la app</t>
         </is>
       </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="G70" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2353,18 +2351,18 @@
       <c r="J70" s="8" t="n"/>
       <c r="K70" s="8" t="n"/>
     </row>
-    <row r="71" ht="36" customHeight="1" s="14">
+    <row r="71" ht="36" customHeight="1" s="12">
       <c r="A71" s="8" t="n"/>
       <c r="B71" s="8" t="n"/>
       <c r="C71" s="8" t="n"/>
       <c r="D71" s="8" t="n"/>
       <c r="E71" s="9" t="n"/>
-      <c r="F71" s="12" t="inlineStr">
+      <c r="F71" s="14" t="inlineStr">
         <is>
           <t>Modificar la fecha u hora de una reserva ya creada, sin cancelarla; el cambio libera el horario anterior y la reserva vuelve a quedar pendiente de confirmación</t>
         </is>
       </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="G71" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2374,60 +2372,60 @@
       <c r="J71" s="9" t="n"/>
       <c r="K71" s="9" t="n"/>
     </row>
-    <row r="72" ht="45" customHeight="1" s="14">
+    <row r="72" ht="45" customHeight="1" s="12">
       <c r="A72" s="8" t="n"/>
       <c r="B72" s="8" t="n"/>
       <c r="C72" s="8" t="n"/>
       <c r="D72" s="8" t="n"/>
-      <c r="E72" s="12" t="inlineStr">
+      <c r="E72" s="14" t="inlineStr">
         <is>
           <t>HU12 - Gestión de reservas entrantes (Restaurante)
 Como restaurante, quiero ver las reservas entrantes y confirmarlas o rechazarlas, para organizar la disponibilidad de mesas de mi local.</t>
         </is>
       </c>
-      <c r="F72" s="12" t="inlineStr">
+      <c r="F72" s="14" t="inlineStr">
         <is>
           <t>Listado de reservas del día ordenado por hora</t>
         </is>
       </c>
-      <c r="G72" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H72" s="12" t="inlineStr">
+      <c r="G72" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H72" s="14" t="inlineStr">
         <is>
           <t>Firestore (listener en tiempo real); Firebase Cloud Messaging</t>
         </is>
       </c>
-      <c r="I72" s="7" t="inlineStr">
+      <c r="I72" s="10" t="inlineStr">
         <is>
           <t>Semana 9</t>
         </is>
       </c>
-      <c r="J72" s="7" t="inlineStr">
+      <c r="J72" s="10" t="inlineStr">
         <is>
           <t>Semana 10</t>
         </is>
       </c>
-      <c r="K72" s="7" t="inlineStr">
-        <is>
-          <t>Camila Bada</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="36" customHeight="1" s="14">
+      <c r="K72" s="10" t="inlineStr">
+        <is>
+          <t>Jose Chuque</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="36" customHeight="1" s="12">
       <c r="A73" s="8" t="n"/>
       <c r="B73" s="8" t="n"/>
       <c r="C73" s="8" t="n"/>
       <c r="D73" s="8" t="n"/>
       <c r="E73" s="8" t="n"/>
-      <c r="F73" s="12" t="inlineStr">
+      <c r="F73" s="14" t="inlineStr">
         <is>
           <t>Confirmación o rechazo de una reserva entrante; el rechazo exige un motivo de una lista (sin mesas a esa hora, local cerrado ese día, grupo demasiado grande) u «Otro» con texto</t>
         </is>
       </c>
-      <c r="G73" s="7" t="inlineStr">
+      <c r="G73" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2437,18 +2435,18 @@
       <c r="J73" s="8" t="n"/>
       <c r="K73" s="8" t="n"/>
     </row>
-    <row r="74" ht="36" customHeight="1" s="14">
+    <row r="74" ht="36" customHeight="1" s="12">
       <c r="A74" s="8" t="n"/>
       <c r="B74" s="8" t="n"/>
       <c r="C74" s="8" t="n"/>
       <c r="D74" s="8" t="n"/>
       <c r="E74" s="8" t="n"/>
-      <c r="F74" s="12" t="inlineStr">
+      <c r="F74" s="14" t="inlineStr">
         <is>
           <t>Notificación push al comensal con la respuesta y, si se rechazó, el motivo</t>
         </is>
       </c>
-      <c r="G74" s="7" t="inlineStr">
+      <c r="G74" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2458,18 +2456,18 @@
       <c r="J74" s="8" t="n"/>
       <c r="K74" s="8" t="n"/>
     </row>
-    <row r="75" ht="36" customHeight="1" s="14">
+    <row r="75" ht="36" customHeight="1" s="12">
       <c r="A75" s="8" t="n"/>
       <c r="B75" s="8" t="n"/>
       <c r="C75" s="8" t="n"/>
       <c r="D75" s="8" t="n"/>
       <c r="E75" s="8" t="n"/>
-      <c r="F75" s="12" t="inlineStr">
+      <c r="F75" s="14" t="inlineStr">
         <is>
           <t>Rechazo automático de la reserva si el restaurante no responde hasta 60 min antes de la hora reservada, con aviso push al comensal</t>
         </is>
       </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="G75" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2479,18 +2477,18 @@
       <c r="J75" s="8" t="n"/>
       <c r="K75" s="8" t="n"/>
     </row>
-    <row r="76" ht="36" customHeight="1" s="14">
+    <row r="76" ht="36" customHeight="1" s="12">
       <c r="A76" s="8" t="n"/>
       <c r="B76" s="8" t="n"/>
       <c r="C76" s="9" t="n"/>
       <c r="D76" s="9" t="n"/>
       <c r="E76" s="9" t="n"/>
-      <c r="F76" s="12" t="inlineStr">
+      <c r="F76" s="14" t="inlineStr">
         <is>
           <t>Cupo de reservas por franja de 30 min (número de comensales) configurable por el local; las franjas llenas, sumando reservas pendientes y confirmadas, no se pueden reservar</t>
         </is>
       </c>
-      <c r="G76" s="7" t="inlineStr">
+      <c r="G76" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2500,69 +2498,69 @@
       <c r="J76" s="9" t="n"/>
       <c r="K76" s="9" t="n"/>
     </row>
-    <row r="77" ht="45" customHeight="1" s="14">
+    <row r="77" ht="45" customHeight="1" s="12">
       <c r="A77" s="8" t="n"/>
       <c r="B77" s="8" t="n"/>
-      <c r="C77" s="7" t="inlineStr">
+      <c r="C77" s="10" t="inlineStr">
         <is>
           <t>Actividad del Comensal:
 Historial de pedidos y reservas pasadas, para consulta y repetición rápida.</t>
         </is>
       </c>
-      <c r="D77" s="7" t="inlineStr">
+      <c r="D77" s="10" t="inlineStr">
         <is>
           <t>Comensal</t>
         </is>
       </c>
-      <c r="E77" s="12" t="inlineStr">
+      <c r="E77" s="14" t="inlineStr">
         <is>
           <t>HU20 - Historial de pedidos y reservas
 Como comensal, quiero ver el historial de mis pedidos y reservas pasadas, para llevar un registro de mi actividad y repetir un pedido anterior fácilmente.</t>
         </is>
       </c>
-      <c r="F77" s="12" t="inlineStr">
+      <c r="F77" s="14" t="inlineStr">
         <is>
           <t>Listado de pedidos y reservas pasadas, ordenado por fecha</t>
         </is>
       </c>
-      <c r="G77" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H77" s="12" t="inlineStr">
+      <c r="G77" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H77" s="14" t="inlineStr">
         <is>
           <t>Firestore (historial); Retrofit + corrutinas (backend propio); Jetpack Compose</t>
         </is>
       </c>
-      <c r="I77" s="7" t="inlineStr">
+      <c r="I77" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="J77" s="7" t="inlineStr">
+      <c r="J77" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="K77" s="7" t="inlineStr">
+      <c r="K77" s="10" t="inlineStr">
         <is>
           <t>Camila Bada</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="36" customHeight="1" s="14">
+    <row r="78" ht="36" customHeight="1" s="12">
       <c r="A78" s="8" t="n"/>
       <c r="B78" s="8" t="n"/>
       <c r="C78" s="8" t="n"/>
       <c r="D78" s="8" t="n"/>
       <c r="E78" s="8" t="n"/>
-      <c r="F78" s="12" t="inlineStr">
+      <c r="F78" s="14" t="inlineStr">
         <is>
           <t>Detalle de cada pedido o reserva pasado (restaurante, ítems, estado final)</t>
         </is>
       </c>
-      <c r="G78" s="7" t="inlineStr">
+      <c r="G78" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2572,18 +2570,18 @@
       <c r="J78" s="8" t="n"/>
       <c r="K78" s="8" t="n"/>
     </row>
-    <row r="79" ht="36" customHeight="1" s="14">
+    <row r="79" ht="36" customHeight="1" s="12">
       <c r="A79" s="8" t="n"/>
       <c r="B79" s="8" t="n"/>
       <c r="C79" s="9" t="n"/>
       <c r="D79" s="9" t="n"/>
       <c r="E79" s="9" t="n"/>
-      <c r="F79" s="12" t="inlineStr">
+      <c r="F79" s="14" t="inlineStr">
         <is>
           <t>Opción de “repetir pedido” que precarga el carrito con los mismos ítems; si incluía menú del día, se eligen entrada y segundo del menú de hoy</t>
         </is>
       </c>
-      <c r="G79" s="7" t="inlineStr">
+      <c r="G79" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2593,69 +2591,69 @@
       <c r="J79" s="9" t="n"/>
       <c r="K79" s="9" t="n"/>
     </row>
-    <row r="80" ht="45" customHeight="1" s="14">
+    <row r="80" ht="45" customHeight="1" s="12">
       <c r="A80" s="8" t="n"/>
       <c r="B80" s="8" t="n"/>
-      <c r="C80" s="7" t="inlineStr">
+      <c r="C80" s="10" t="inlineStr">
         <is>
           <t>Chatbot y Reseñas con IA:
 Atención conversacional para el comensal, y el sistema completo de reseñas: resumen y alerta con IA, visualización de detalle, y respuesta del restaurante.</t>
         </is>
       </c>
-      <c r="D80" s="7" t="inlineStr">
+      <c r="D80" s="10" t="inlineStr">
         <is>
           <t>Comensal / Restaurante / Backend</t>
         </is>
       </c>
-      <c r="E80" s="12" t="inlineStr">
+      <c r="E80" s="14" t="inlineStr">
         <is>
           <t>HU11 - Chatbot de atención con entrada por voz
 Como comensal, quiero consultar a un chatbot (por texto o por voz) sobre horarios, disponibilidad o el estado de mi reserva/pedido, para resolver dudas rápidas sin llamar al restaurante.</t>
         </is>
       </c>
-      <c r="F80" s="12" t="inlineStr">
+      <c r="F80" s="14" t="inlineStr">
         <is>
           <t>Chat conversacional accesible desde la pantalla de un restaurante</t>
         </is>
       </c>
-      <c r="G80" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H80" s="12" t="inlineStr">
+      <c r="G80" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H80" s="14" t="inlineStr">
         <is>
           <t>SpeechRecognizer (entrada de voz); API de un LLM (vía Retrofit + corrutinas); Jetpack Compose</t>
         </is>
       </c>
-      <c r="I80" s="7" t="inlineStr">
+      <c r="I80" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="J80" s="7" t="inlineStr">
+      <c r="J80" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="K80" s="7" t="inlineStr">
-        <is>
-          <t>Camila Bada</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="36" customHeight="1" s="14">
+      <c r="K80" s="10" t="inlineStr">
+        <is>
+          <t>Jose Chuque</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="36" customHeight="1" s="12">
       <c r="A81" s="8" t="n"/>
       <c r="B81" s="8" t="n"/>
       <c r="C81" s="8" t="n"/>
       <c r="D81" s="8" t="n"/>
       <c r="E81" s="8" t="n"/>
-      <c r="F81" s="12" t="inlineStr">
+      <c r="F81" s="14" t="inlineStr">
         <is>
           <t>Entrada por voz mediante reconocimiento de habla, como alternativa al texto</t>
         </is>
       </c>
-      <c r="G81" s="7" t="inlineStr">
+      <c r="G81" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2665,18 +2663,18 @@
       <c r="J81" s="8" t="n"/>
       <c r="K81" s="8" t="n"/>
     </row>
-    <row r="82" ht="36" customHeight="1" s="14">
+    <row r="82" ht="36" customHeight="1" s="12">
       <c r="A82" s="8" t="n"/>
       <c r="B82" s="8" t="n"/>
       <c r="C82" s="8" t="n"/>
       <c r="D82" s="8" t="n"/>
       <c r="E82" s="8" t="n"/>
-      <c r="F82" s="12" t="inlineStr">
+      <c r="F82" s="14" t="inlineStr">
         <is>
           <t>Respuestas sobre horarios, menú y disponibilidad de ese restaurante</t>
         </is>
       </c>
-      <c r="G82" s="7" t="inlineStr">
+      <c r="G82" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2686,18 +2684,18 @@
       <c r="J82" s="8" t="n"/>
       <c r="K82" s="8" t="n"/>
     </row>
-    <row r="83" ht="36" customHeight="1" s="14">
+    <row r="83" ht="36" customHeight="1" s="12">
       <c r="A83" s="8" t="n"/>
       <c r="B83" s="8" t="n"/>
       <c r="C83" s="8" t="n"/>
       <c r="D83" s="8" t="n"/>
       <c r="E83" s="9" t="n"/>
-      <c r="F83" s="12" t="inlineStr">
+      <c r="F83" s="14" t="inlineStr">
         <is>
           <t>Consulta del estado de una reserva o pedido activo mediante el chat</t>
         </is>
       </c>
-      <c r="G83" s="7" t="inlineStr">
+      <c r="G83" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2707,60 +2705,60 @@
       <c r="J83" s="9" t="n"/>
       <c r="K83" s="9" t="n"/>
     </row>
-    <row r="84" ht="45" customHeight="1" s="14">
+    <row r="84" ht="45" customHeight="1" s="12">
       <c r="A84" s="8" t="n"/>
       <c r="B84" s="8" t="n"/>
       <c r="C84" s="8" t="n"/>
       <c r="D84" s="8" t="n"/>
-      <c r="E84" s="12" t="inlineStr">
+      <c r="E84" s="14" t="inlineStr">
         <is>
           <t>HU14 - Resumen de reseñas (Comensal)
 Como comensal, quiero ver un resumen breve de las opiniones de un restaurante, para decidir si me conviene sin leer cada reseña una por una.</t>
         </is>
       </c>
-      <c r="F84" s="12" t="inlineStr">
+      <c r="F84" s="14" t="inlineStr">
         <is>
           <t>Generación de un resumen de 2-3 líneas a partir de las reseñas recientes</t>
         </is>
       </c>
-      <c r="G84" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H84" s="12" t="inlineStr">
-        <is>
-          <t>API de un LLM (vía backend propio); Firestore (caché del resumen con timestamp)</t>
-        </is>
-      </c>
-      <c r="I84" s="7" t="inlineStr">
+      <c r="G84" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H84" s="14" t="inlineStr">
+        <is>
+          <t>Cloud Function programada (resumenResenas) que genera el resumen con Gemini; Firestore (caché del resumen con timestamp)</t>
+        </is>
+      </c>
+      <c r="I84" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="J84" s="7" t="inlineStr">
+      <c r="J84" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="K84" s="7" t="inlineStr">
+      <c r="K84" s="10" t="inlineStr">
         <is>
           <t>Rodrigo Puente</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="36" customHeight="1" s="14">
+    <row r="85" ht="36" customHeight="1" s="12">
       <c r="A85" s="8" t="n"/>
       <c r="B85" s="8" t="n"/>
       <c r="C85" s="8" t="n"/>
       <c r="D85" s="8" t="n"/>
       <c r="E85" s="9" t="n"/>
-      <c r="F85" s="12" t="inlineStr">
+      <c r="F85" s="14" t="inlineStr">
         <is>
           <t>Resumen cacheado y regenerado solo cada cierto tiempo, no en cada visita</t>
         </is>
       </c>
-      <c r="G85" s="7" t="inlineStr">
+      <c r="G85" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2770,60 +2768,60 @@
       <c r="J85" s="9" t="n"/>
       <c r="K85" s="9" t="n"/>
     </row>
-    <row r="86" ht="45" customHeight="1" s="14">
+    <row r="86" ht="45" customHeight="1" s="12">
       <c r="A86" s="8" t="n"/>
       <c r="B86" s="8" t="n"/>
       <c r="C86" s="8" t="n"/>
       <c r="D86" s="8" t="n"/>
-      <c r="E86" s="12" t="inlineStr">
+      <c r="E86" s="14" t="inlineStr">
         <is>
           <t>HU22 - Ver detalle de reseñas de un restaurante (Comensal)
 Como comensal, quiero ver el listado completo de reseñas de un restaurante (autor, calificación, comentario, fecha), para revisar el detalle si el resumen de IA no me es suficiente.</t>
         </is>
       </c>
-      <c r="F86" s="12" t="inlineStr">
+      <c r="F86" s="14" t="inlineStr">
         <is>
           <t>Listado de reseñas ordenado por fecha, con calificación y comentario</t>
         </is>
       </c>
-      <c r="G86" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H86" s="12" t="inlineStr">
+      <c r="G86" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H86" s="14" t="inlineStr">
         <is>
           <t>Firestore (colección de reseñas); Jetpack Compose</t>
         </is>
       </c>
-      <c r="I86" s="7" t="inlineStr">
+      <c r="I86" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="J86" s="7" t="inlineStr">
+      <c r="J86" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="K86" s="7" t="inlineStr">
-        <is>
-          <t>Rodrigo Puente</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="36" customHeight="1" s="14">
+      <c r="K86" s="10" t="inlineStr">
+        <is>
+          <t>Camila Bada</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="36" customHeight="1" s="12">
       <c r="A87" s="8" t="n"/>
       <c r="B87" s="8" t="n"/>
       <c r="C87" s="8" t="n"/>
       <c r="D87" s="8" t="n"/>
       <c r="E87" s="8" t="n"/>
-      <c r="F87" s="12" t="inlineStr">
+      <c r="F87" s="14" t="inlineStr">
         <is>
           <t>Filtro por calificación (1 a 5 estrellas)</t>
         </is>
       </c>
-      <c r="G87" s="7" t="inlineStr">
+      <c r="G87" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2833,18 +2831,18 @@
       <c r="J87" s="8" t="n"/>
       <c r="K87" s="8" t="n"/>
     </row>
-    <row r="88" ht="36" customHeight="1" s="14">
+    <row r="88" ht="36" customHeight="1" s="12">
       <c r="A88" s="8" t="n"/>
       <c r="B88" s="8" t="n"/>
       <c r="C88" s="8" t="n"/>
       <c r="D88" s="8" t="n"/>
       <c r="E88" s="8" t="n"/>
-      <c r="F88" s="12" t="inlineStr">
+      <c r="F88" s="14" t="inlineStr">
         <is>
           <t>Se muestra la respuesta del restaurante debajo de la reseña, si existe</t>
         </is>
       </c>
-      <c r="G88" s="7" t="inlineStr">
+      <c r="G88" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2854,18 +2852,18 @@
       <c r="J88" s="8" t="n"/>
       <c r="K88" s="8" t="n"/>
     </row>
-    <row r="89" ht="36" customHeight="1" s="14">
+    <row r="89" ht="36" customHeight="1" s="12">
       <c r="A89" s="8" t="n"/>
       <c r="B89" s="8" t="n"/>
       <c r="C89" s="8" t="n"/>
       <c r="D89" s="8" t="n"/>
       <c r="E89" s="9" t="n"/>
-      <c r="F89" s="12" t="inlineStr">
+      <c r="F89" s="14" t="inlineStr">
         <is>
           <t>Reportar una reseña ajena con motivo (ofensiva, falsa, spam u otro); cada comensal puede reportarla una sola vez y la reseña pasa a la cola de moderación de HU25</t>
         </is>
       </c>
-      <c r="G89" s="7" t="inlineStr">
+      <c r="G89" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2875,60 +2873,60 @@
       <c r="J89" s="9" t="n"/>
       <c r="K89" s="9" t="n"/>
     </row>
-    <row r="90" ht="45" customHeight="1" s="14">
+    <row r="90" ht="45" customHeight="1" s="12">
       <c r="A90" s="8" t="n"/>
       <c r="B90" s="8" t="n"/>
       <c r="C90" s="8" t="n"/>
       <c r="D90" s="8" t="n"/>
-      <c r="E90" s="12" t="inlineStr">
+      <c r="E90" s="14" t="inlineStr">
         <is>
           <t>HU15 - Alerta de reseñas negativas (Restaurante)
 Como restaurante, quiero recibir una alerta cuando llega una reseña negativa, para poder responder o corregir el problema a tiempo.</t>
         </is>
       </c>
-      <c r="F90" s="12" t="inlineStr">
+      <c r="F90" s="14" t="inlineStr">
         <is>
           <t>Clasificación automática del sentimiento de cada reseña nueva (positivo/negativo/neutro)</t>
         </is>
       </c>
-      <c r="G90" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H90" s="12" t="inlineStr">
+      <c r="G90" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H90" s="14" t="inlineStr">
         <is>
           <t>Cloud Functions for Firebase (trigger en Firestore); API de un LLM; Firebase Cloud Messaging</t>
         </is>
       </c>
-      <c r="I90" s="7" t="inlineStr">
+      <c r="I90" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="J90" s="7" t="inlineStr">
+      <c r="J90" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="K90" s="7" t="inlineStr">
+      <c r="K90" s="10" t="inlineStr">
         <is>
           <t>Rodrigo Puente</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="36" customHeight="1" s="14">
+    <row r="91" ht="36" customHeight="1" s="12">
       <c r="A91" s="8" t="n"/>
       <c r="B91" s="8" t="n"/>
       <c r="C91" s="8" t="n"/>
       <c r="D91" s="8" t="n"/>
       <c r="E91" s="8" t="n"/>
-      <c r="F91" s="12" t="inlineStr">
+      <c r="F91" s="14" t="inlineStr">
         <is>
           <t>Extracción del motivo principal cuando la reseña es negativa</t>
         </is>
       </c>
-      <c r="G91" s="7" t="inlineStr">
+      <c r="G91" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2938,18 +2936,18 @@
       <c r="J91" s="8" t="n"/>
       <c r="K91" s="8" t="n"/>
     </row>
-    <row r="92" ht="36" customHeight="1" s="14">
+    <row r="92" ht="36" customHeight="1" s="12">
       <c r="A92" s="8" t="n"/>
       <c r="B92" s="8" t="n"/>
       <c r="C92" s="8" t="n"/>
       <c r="D92" s="8" t="n"/>
       <c r="E92" s="9" t="n"/>
-      <c r="F92" s="12" t="inlineStr">
+      <c r="F92" s="14" t="inlineStr">
         <is>
           <t>Notificación push al restaurante ante una reseña clasificada como negativa</t>
         </is>
       </c>
-      <c r="G92" s="7" t="inlineStr">
+      <c r="G92" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -2959,60 +2957,60 @@
       <c r="J92" s="9" t="n"/>
       <c r="K92" s="9" t="n"/>
     </row>
-    <row r="93" ht="45" customHeight="1" s="14">
+    <row r="93" ht="45" customHeight="1" s="12">
       <c r="A93" s="8" t="n"/>
       <c r="B93" s="8" t="n"/>
       <c r="C93" s="8" t="n"/>
       <c r="D93" s="8" t="n"/>
-      <c r="E93" s="12" t="inlineStr">
+      <c r="E93" s="14" t="inlineStr">
         <is>
           <t>HU21 - Gestión y respuesta a reseñas (Restaurante)
 Como restaurante, quiero ver todas mis reseñas recibidas y responder a cualquiera de ellas, para mostrar que atiendo la retroalimentación de mis comensales, no solo las negativas.</t>
         </is>
       </c>
-      <c r="F93" s="12" t="inlineStr">
+      <c r="F93" s="14" t="inlineStr">
         <is>
           <t>Listado completo de reseñas recibidas, no solo las negativas</t>
         </is>
       </c>
-      <c r="G93" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H93" s="12" t="inlineStr">
+      <c r="G93" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H93" s="14" t="inlineStr">
         <is>
           <t>Firestore (subcolección de respuestas); Firebase Cloud Messaging</t>
         </is>
       </c>
-      <c r="I93" s="7" t="inlineStr">
+      <c r="I93" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="J93" s="7" t="inlineStr">
+      <c r="J93" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="K93" s="7" t="inlineStr">
+      <c r="K93" s="10" t="inlineStr">
         <is>
           <t>Jose Chuque</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="36" customHeight="1" s="14">
+    <row r="94" ht="36" customHeight="1" s="12">
       <c r="A94" s="8" t="n"/>
       <c r="B94" s="8" t="n"/>
       <c r="C94" s="8" t="n"/>
       <c r="D94" s="8" t="n"/>
       <c r="E94" s="8" t="n"/>
-      <c r="F94" s="12" t="inlineStr">
+      <c r="F94" s="14" t="inlineStr">
         <is>
           <t>Responder públicamente a cualquier reseña</t>
         </is>
       </c>
-      <c r="G94" s="7" t="inlineStr">
+      <c r="G94" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3022,18 +3020,18 @@
       <c r="J94" s="8" t="n"/>
       <c r="K94" s="8" t="n"/>
     </row>
-    <row r="95" ht="36" customHeight="1" s="14">
+    <row r="95" ht="36" customHeight="1" s="12">
       <c r="A95" s="8" t="n"/>
       <c r="B95" s="8" t="n"/>
       <c r="C95" s="9" t="n"/>
       <c r="D95" s="9" t="n"/>
       <c r="E95" s="9" t="n"/>
-      <c r="F95" s="12" t="inlineStr">
+      <c r="F95" s="14" t="inlineStr">
         <is>
           <t>Notificación al comensal cuando su reseña recibe respuesta</t>
         </is>
       </c>
-      <c r="G95" s="7" t="inlineStr">
+      <c r="G95" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3043,69 +3041,69 @@
       <c r="J95" s="9" t="n"/>
       <c r="K95" s="9" t="n"/>
     </row>
-    <row r="96" ht="45" customHeight="1" s="14">
+    <row r="96" ht="45" customHeight="1" s="12">
       <c r="A96" s="8" t="n"/>
       <c r="B96" s="8" t="n"/>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C96" s="10" t="inlineStr">
         <is>
           <t>Moderación de la Plataforma (Administrador):
 Revisión y moderación de las reseñas del sistema.</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D96" s="10" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E96" s="12" t="inlineStr">
+      <c r="E96" s="14" t="inlineStr">
         <is>
           <t>HU25 - Moderación de reseñas
 Como administrador, quiero revisar y eliminar una reseña reportada como abusiva o falsa, para mantener la confianza del sistema de reseñas.</t>
         </is>
       </c>
-      <c r="F96" s="12" t="inlineStr">
+      <c r="F96" s="14" t="inlineStr">
         <is>
           <t>Listado de reseñas reportadas o marcadas para revisión</t>
         </is>
       </c>
-      <c r="G96" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H96" s="12" t="inlineStr">
+      <c r="G96" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H96" s="14" t="inlineStr">
         <is>
           <t>Firestore (listener de reseñas reportadas); Cloud Functions for Firebase</t>
         </is>
       </c>
-      <c r="I96" s="7" t="inlineStr">
+      <c r="I96" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="J96" s="7" t="inlineStr">
+      <c r="J96" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="K96" s="7" t="inlineStr">
-        <is>
-          <t>Rodrigo Puente</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="36" customHeight="1" s="14">
+      <c r="K96" s="10" t="inlineStr">
+        <is>
+          <t>Camila Bada</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="36" customHeight="1" s="12">
       <c r="A97" s="8" t="n"/>
       <c r="B97" s="8" t="n"/>
       <c r="C97" s="8" t="n"/>
       <c r="D97" s="8" t="n"/>
       <c r="E97" s="8" t="n"/>
-      <c r="F97" s="12" t="inlineStr">
+      <c r="F97" s="14" t="inlineStr">
         <is>
           <t>Eliminar una reseña clasificada como abusiva o falsa</t>
         </is>
       </c>
-      <c r="G97" s="7" t="inlineStr">
+      <c r="G97" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3115,18 +3113,18 @@
       <c r="J97" s="8" t="n"/>
       <c r="K97" s="8" t="n"/>
     </row>
-    <row r="98" ht="36" customHeight="1" s="14">
+    <row r="98" ht="36" customHeight="1" s="12">
       <c r="A98" s="8" t="n"/>
       <c r="B98" s="8" t="n"/>
       <c r="C98" s="9" t="n"/>
       <c r="D98" s="9" t="n"/>
       <c r="E98" s="9" t="n"/>
-      <c r="F98" s="12" t="inlineStr">
+      <c r="F98" s="14" t="inlineStr">
         <is>
           <t>Registro de la acción de moderación realizada</t>
         </is>
       </c>
-      <c r="G98" s="7" t="inlineStr">
+      <c r="G98" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3136,69 +3134,69 @@
       <c r="J98" s="9" t="n"/>
       <c r="K98" s="9" t="n"/>
     </row>
-    <row r="99" ht="45" customHeight="1" s="14">
+    <row r="99" ht="45" customHeight="1" s="12">
       <c r="A99" s="8" t="n"/>
       <c r="B99" s="8" t="n"/>
-      <c r="C99" s="7" t="inlineStr">
+      <c r="C99" s="10" t="inlineStr">
         <is>
           <t>Dashboard de Restaurante y de Plataforma:
 Panel de indicadores del negocio para el restaurante, y panel agregado de la plataforma para el administrador.</t>
         </is>
       </c>
-      <c r="D99" s="7" t="inlineStr">
+      <c r="D99" s="10" t="inlineStr">
         <is>
           <t>Restaurante / Administrador</t>
         </is>
       </c>
-      <c r="E99" s="12" t="inlineStr">
+      <c r="E99" s="14" t="inlineStr">
         <is>
           <t>HU13 - Dashboard de restaurante
 Como restaurante, quiero ver un dashboard con mis ventas, platos más pedidos y calificación promedio, para entender cómo va mi negocio en la app.</t>
         </is>
       </c>
-      <c r="F99" s="12" t="inlineStr">
+      <c r="F99" s="14" t="inlineStr">
         <is>
           <t>Gráfico de ventas/pedidos por día o semana</t>
         </is>
       </c>
-      <c r="G99" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H99" s="12" t="inlineStr">
+      <c r="G99" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H99" s="14" t="inlineStr">
         <is>
           <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de pedidos y calificaciones)</t>
         </is>
       </c>
-      <c r="I99" s="7" t="inlineStr">
+      <c r="I99" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="J99" s="7" t="inlineStr">
+      <c r="J99" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="K99" s="7" t="inlineStr">
+      <c r="K99" s="10" t="inlineStr">
         <is>
           <t>Jose Chuque</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="36" customHeight="1" s="14">
+    <row r="100" ht="36" customHeight="1" s="12">
       <c r="A100" s="8" t="n"/>
       <c r="B100" s="8" t="n"/>
       <c r="C100" s="8" t="n"/>
       <c r="D100" s="8" t="n"/>
       <c r="E100" s="8" t="n"/>
-      <c r="F100" s="12" t="inlineStr">
+      <c r="F100" s="14" t="inlineStr">
         <is>
           <t>Ranking de platos más pedidos</t>
         </is>
       </c>
-      <c r="G100" s="7" t="inlineStr">
+      <c r="G100" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3208,18 +3206,18 @@
       <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="n"/>
     </row>
-    <row r="101" ht="36" customHeight="1" s="14">
+    <row r="101" ht="36" customHeight="1" s="12">
       <c r="A101" s="8" t="n"/>
       <c r="B101" s="8" t="n"/>
       <c r="C101" s="8" t="n"/>
       <c r="D101" s="8" t="n"/>
       <c r="E101" s="9" t="n"/>
-      <c r="F101" s="12" t="inlineStr">
+      <c r="F101" s="14" t="inlineStr">
         <is>
           <t>Calificación promedio y su evolución en el tiempo</t>
         </is>
       </c>
-      <c r="G101" s="7" t="inlineStr">
+      <c r="G101" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3229,60 +3227,60 @@
       <c r="J101" s="9" t="n"/>
       <c r="K101" s="9" t="n"/>
     </row>
-    <row r="102" ht="45" customHeight="1" s="14">
+    <row r="102" ht="45" customHeight="1" s="12">
       <c r="A102" s="8" t="n"/>
       <c r="B102" s="8" t="n"/>
       <c r="C102" s="8" t="n"/>
       <c r="D102" s="8" t="n"/>
-      <c r="E102" s="12" t="inlineStr">
+      <c r="E102" s="14" t="inlineStr">
         <is>
           <t>HU26 - Dashboard global (Administrador)
 Como administrador, quiero ver métricas agregadas de toda la plataforma (restaurantes activos, pedidos totales), para monitorear la salud del negocio.</t>
         </is>
       </c>
-      <c r="F102" s="12" t="inlineStr">
+      <c r="F102" s="14" t="inlineStr">
         <is>
           <t>Métricas agregadas de todos los restaurantes: restaurantes activos y pedidos totales</t>
         </is>
       </c>
-      <c r="G102" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H102" s="12" t="inlineStr">
+      <c r="G102" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H102" s="14" t="inlineStr">
         <is>
           <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de locales y pedidos); Cloud Functions</t>
         </is>
       </c>
-      <c r="I102" s="7" t="inlineStr">
+      <c r="I102" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="J102" s="7" t="inlineStr">
+      <c r="J102" s="10" t="inlineStr">
         <is>
           <t>Semana 12</t>
         </is>
       </c>
-      <c r="K102" s="7" t="inlineStr">
+      <c r="K102" s="10" t="inlineStr">
         <is>
           <t>Rodrigo Puente</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="36" customHeight="1" s="14">
+    <row r="103" ht="36" customHeight="1" s="12">
       <c r="A103" s="8" t="n"/>
       <c r="B103" s="8" t="n"/>
       <c r="C103" s="8" t="n"/>
       <c r="D103" s="8" t="n"/>
       <c r="E103" s="8" t="n"/>
-      <c r="F103" s="12" t="inlineStr">
+      <c r="F103" s="14" t="inlineStr">
         <is>
           <t>El dashboard obtiene las métricas con consultas de agregación de Firestore (count, sum), sin backend propio; lo que no se pueda agregar así lo calcula una Cloud Function</t>
         </is>
       </c>
-      <c r="G103" s="7" t="inlineStr">
+      <c r="G103" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3292,18 +3290,18 @@
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
     </row>
-    <row r="104" ht="36" customHeight="1" s="14">
+    <row r="104" ht="36" customHeight="1" s="12">
       <c r="A104" s="8" t="n"/>
       <c r="B104" s="9" t="n"/>
       <c r="C104" s="9" t="n"/>
       <c r="D104" s="9" t="n"/>
       <c r="E104" s="9" t="n"/>
-      <c r="F104" s="12" t="inlineStr">
+      <c r="F104" s="14" t="inlineStr">
         <is>
           <t>Gráfico de evolución de pedidos totales por semana</t>
         </is>
       </c>
-      <c r="G104" s="7" t="inlineStr">
+      <c r="G104" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3313,71 +3311,71 @@
       <c r="J104" s="9" t="n"/>
       <c r="K104" s="9" t="n"/>
     </row>
-    <row r="105" ht="45" customHeight="1" s="14">
+    <row r="105" ht="45" customHeight="1" s="12">
       <c r="A105" s="8" t="n"/>
-      <c r="B105" s="11" t="n">
+      <c r="B105" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C105" s="11" t="inlineStr">
+      <c r="C105" s="7" t="inlineStr">
         <is>
           <t>Seguridad, Pruebas y Despliegue:
 Asegurar, probar y publicar ambas aplicaciones.</t>
         </is>
       </c>
-      <c r="D105" s="11" t="inlineStr">
+      <c r="D105" s="7" t="inlineStr">
         <is>
           <t>Ambas</t>
         </is>
       </c>
-      <c r="E105" s="10" t="inlineStr">
+      <c r="E105" s="11" t="inlineStr">
         <is>
           <t>HU16 - Aseguramiento con OWASP Mobile
 Como equipo, queremos aplicar buenas prácticas de seguridad móvil OWASP, para proteger los datos de comensales y restaurantes en ambas apps.</t>
         </is>
       </c>
-      <c r="F105" s="10" t="inlineStr">
+      <c r="F105" s="11" t="inlineStr">
         <is>
           <t>Revisión de almacenamiento seguro de credenciales y tokens</t>
         </is>
       </c>
-      <c r="G105" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H105" s="10" t="inlineStr">
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H105" s="11" t="inlineStr">
         <is>
           <t>OWASP MASVS/MSTG (checklist); ProGuard/R8; EncryptedSharedPreferences</t>
         </is>
       </c>
-      <c r="I105" s="11" t="inlineStr">
+      <c r="I105" s="7" t="inlineStr">
         <is>
           <t>Semana 13</t>
         </is>
       </c>
-      <c r="J105" s="11" t="inlineStr">
+      <c r="J105" s="7" t="inlineStr">
         <is>
           <t>Semana 13</t>
         </is>
       </c>
-      <c r="K105" s="11" t="inlineStr">
-        <is>
-          <t>Jose Chuque</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="36" customHeight="1" s="14">
+      <c r="K105" s="7" t="inlineStr">
+        <is>
+          <t>Rodrigo Puente</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="36" customHeight="1" s="12">
       <c r="A106" s="8" t="n"/>
       <c r="B106" s="8" t="n"/>
       <c r="C106" s="8" t="n"/>
       <c r="D106" s="8" t="n"/>
       <c r="E106" s="8" t="n"/>
-      <c r="F106" s="10" t="inlineStr">
+      <c r="F106" s="11" t="inlineStr">
         <is>
           <t>Ofuscación de código y protección contra ingeniería inversa</t>
         </is>
       </c>
-      <c r="G106" s="11" t="inlineStr">
+      <c r="G106" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3387,18 +3385,18 @@
       <c r="J106" s="8" t="n"/>
       <c r="K106" s="8" t="n"/>
     </row>
-    <row r="107" ht="36" customHeight="1" s="14">
+    <row r="107" ht="36" customHeight="1" s="12">
       <c r="A107" s="8" t="n"/>
       <c r="B107" s="8" t="n"/>
       <c r="C107" s="8" t="n"/>
       <c r="D107" s="8" t="n"/>
       <c r="E107" s="8" t="n"/>
-      <c r="F107" s="10" t="inlineStr">
+      <c r="F107" s="11" t="inlineStr">
         <is>
           <t>Validación de comunicación segura (HTTPS/TLS) con el backend y Firebase</t>
         </is>
       </c>
-      <c r="G107" s="11" t="inlineStr">
+      <c r="G107" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3408,18 +3406,18 @@
       <c r="J107" s="8" t="n"/>
       <c r="K107" s="8" t="n"/>
     </row>
-    <row r="108" ht="36" customHeight="1" s="14">
+    <row r="108" ht="36" customHeight="1" s="12">
       <c r="A108" s="8" t="n"/>
       <c r="B108" s="8" t="n"/>
       <c r="C108" s="8" t="n"/>
       <c r="D108" s="8" t="n"/>
       <c r="E108" s="9" t="n"/>
-      <c r="F108" s="10" t="inlineStr">
+      <c r="F108" s="11" t="inlineStr">
         <is>
           <t>Validación de que solo el rol administrador puede acceder a los endpoints y reglas de agregación global</t>
         </is>
       </c>
-      <c r="G108" s="11" t="inlineStr">
+      <c r="G108" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3429,60 +3427,60 @@
       <c r="J108" s="9" t="n"/>
       <c r="K108" s="9" t="n"/>
     </row>
-    <row r="109" ht="45" customHeight="1" s="14">
+    <row r="109" ht="45" customHeight="1" s="12">
       <c r="A109" s="8" t="n"/>
       <c r="B109" s="8" t="n"/>
       <c r="C109" s="8" t="n"/>
       <c r="D109" s="8" t="n"/>
-      <c r="E109" s="10" t="inlineStr">
+      <c r="E109" s="11" t="inlineStr">
         <is>
           <t>HU17 - Pruebas y corrección de observaciones
 Como equipo, queremos probar ambas aplicaciones de forma integral y levantar las observaciones de los sprints anteriores, para asegurar la calidad antes del despliegue final.</t>
         </is>
       </c>
-      <c r="F109" s="10" t="inlineStr">
+      <c r="F109" s="11" t="inlineStr">
         <is>
           <t>Pruebas unitarias de ViewModels y casos de uso principales en ambas apps</t>
         </is>
       </c>
-      <c r="G109" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H109" s="10" t="inlineStr">
+      <c r="G109" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H109" s="11" t="inlineStr">
         <is>
           <t>JUnit; Espresso / Compose Testing; Firebase Test Lab</t>
         </is>
       </c>
-      <c r="I109" s="11" t="inlineStr">
+      <c r="I109" s="7" t="inlineStr">
         <is>
           <t>Semana 14</t>
         </is>
       </c>
-      <c r="J109" s="11" t="inlineStr">
+      <c r="J109" s="7" t="inlineStr">
         <is>
           <t>Semana 14</t>
         </is>
       </c>
-      <c r="K109" s="11" t="inlineStr">
-        <is>
-          <t>Camila Bada</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="36" customHeight="1" s="14">
+      <c r="K109" s="7" t="inlineStr">
+        <is>
+          <t>Rodrigo Puente</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="36" customHeight="1" s="12">
       <c r="A110" s="8" t="n"/>
       <c r="B110" s="8" t="n"/>
       <c r="C110" s="8" t="n"/>
       <c r="D110" s="8" t="n"/>
       <c r="E110" s="8" t="n"/>
-      <c r="F110" s="10" t="inlineStr">
+      <c r="F110" s="11" t="inlineStr">
         <is>
           <t>Pruebas de UI de los flujos críticos (registro, pedido, reserva)</t>
         </is>
       </c>
-      <c r="G110" s="11" t="inlineStr">
+      <c r="G110" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3492,18 +3490,18 @@
       <c r="J110" s="8" t="n"/>
       <c r="K110" s="8" t="n"/>
     </row>
-    <row r="111" ht="36" customHeight="1" s="14">
+    <row r="111" ht="36" customHeight="1" s="12">
       <c r="A111" s="8" t="n"/>
       <c r="B111" s="8" t="n"/>
       <c r="C111" s="8" t="n"/>
       <c r="D111" s="8" t="n"/>
       <c r="E111" s="8" t="n"/>
-      <c r="F111" s="10" t="inlineStr">
+      <c r="F111" s="11" t="inlineStr">
         <is>
           <t>Ejecución en Firebase Test Lab en distintos dispositivos</t>
         </is>
       </c>
-      <c r="G111" s="11" t="inlineStr">
+      <c r="G111" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3513,18 +3511,18 @@
       <c r="J111" s="8" t="n"/>
       <c r="K111" s="8" t="n"/>
     </row>
-    <row r="112" ht="36" customHeight="1" s="14">
+    <row r="112" ht="36" customHeight="1" s="12">
       <c r="A112" s="8" t="n"/>
       <c r="B112" s="8" t="n"/>
       <c r="C112" s="8" t="n"/>
       <c r="D112" s="8" t="n"/>
       <c r="E112" s="9" t="n"/>
-      <c r="F112" s="10" t="inlineStr">
+      <c r="F112" s="11" t="inlineStr">
         <is>
           <t>Corrección de observaciones formuladas en la sustentación del 2do Sprint</t>
         </is>
       </c>
-      <c r="G112" s="11" t="inlineStr">
+      <c r="G112" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3534,60 +3532,60 @@
       <c r="J112" s="9" t="n"/>
       <c r="K112" s="9" t="n"/>
     </row>
-    <row r="113" ht="45" customHeight="1" s="14">
+    <row r="113" ht="45" customHeight="1" s="12">
       <c r="A113" s="8" t="n"/>
       <c r="B113" s="8" t="n"/>
       <c r="C113" s="8" t="n"/>
       <c r="D113" s="8" t="n"/>
-      <c r="E113" s="10" t="inlineStr">
+      <c r="E113" s="11" t="inlineStr">
         <is>
           <t>HU18 - Despliegue en Google Play Store (2 apps)
 Como equipo, queremos publicar ambas aplicaciones en Google Play Store, para que estén disponibles públicamente al finalizar el curso.</t>
         </is>
       </c>
-      <c r="F113" s="10" t="inlineStr">
+      <c r="F113" s="11" t="inlineStr">
         <is>
           <t>Generación del bundle firmado (AAB) de cada app</t>
         </is>
       </c>
-      <c r="G113" s="11" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H113" s="10" t="inlineStr">
+      <c r="G113" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H113" s="11" t="inlineStr">
         <is>
           <t>Play App Signing; Google Play Console; Firebase App Distribution</t>
         </is>
       </c>
-      <c r="I113" s="11" t="inlineStr">
+      <c r="I113" s="7" t="inlineStr">
         <is>
           <t>Semana 15</t>
         </is>
       </c>
-      <c r="J113" s="11" t="inlineStr">
+      <c r="J113" s="7" t="inlineStr">
         <is>
           <t>Semana 15</t>
         </is>
       </c>
-      <c r="K113" s="11" t="inlineStr">
+      <c r="K113" s="7" t="inlineStr">
         <is>
           <t>Rodrigo Puente</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="36" customHeight="1" s="14">
+    <row r="114" ht="36" customHeight="1" s="12">
       <c r="A114" s="8" t="n"/>
       <c r="B114" s="8" t="n"/>
       <c r="C114" s="8" t="n"/>
       <c r="D114" s="8" t="n"/>
       <c r="E114" s="8" t="n"/>
-      <c r="F114" s="10" t="inlineStr">
+      <c r="F114" s="11" t="inlineStr">
         <is>
           <t>Configuración de la ficha de cada app en Play Console</t>
         </is>
       </c>
-      <c r="G114" s="11" t="inlineStr">
+      <c r="G114" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3597,18 +3595,18 @@
       <c r="J114" s="8" t="n"/>
       <c r="K114" s="8" t="n"/>
     </row>
-    <row r="115" ht="36" customHeight="1" s="14">
+    <row r="115" ht="36" customHeight="1" s="12">
       <c r="A115" s="8" t="n"/>
       <c r="B115" s="8" t="n"/>
       <c r="C115" s="8" t="n"/>
       <c r="D115" s="8" t="n"/>
       <c r="E115" s="8" t="n"/>
-      <c r="F115" s="10" t="inlineStr">
+      <c r="F115" s="11" t="inlineStr">
         <is>
           <t>Distribución beta previa con Firebase App Distribution</t>
         </is>
       </c>
-      <c r="G115" s="11" t="inlineStr">
+      <c r="G115" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3618,18 +3616,18 @@
       <c r="J115" s="8" t="n"/>
       <c r="K115" s="8" t="n"/>
     </row>
-    <row r="116" ht="36" customHeight="1" s="14">
+    <row r="116" ht="36" customHeight="1" s="12">
       <c r="A116" s="9" t="n"/>
       <c r="B116" s="9" t="n"/>
       <c r="C116" s="9" t="n"/>
       <c r="D116" s="9" t="n"/>
       <c r="E116" s="9" t="n"/>
-      <c r="F116" s="10" t="inlineStr">
+      <c r="F116" s="11" t="inlineStr">
         <is>
           <t>Publicación en producción de ambas apps en Google Play Store</t>
         </is>
       </c>
-      <c r="G116" s="11" t="inlineStr">
+      <c r="G116" s="7" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3641,146 +3639,133 @@
     </row>
   </sheetData>
   <mergeCells count="158">
-    <mergeCell ref="I12:I18"/>
     <mergeCell ref="K80:K83"/>
+    <mergeCell ref="K96:K98"/>
     <mergeCell ref="I48:I50"/>
     <mergeCell ref="K48:K50"/>
     <mergeCell ref="J25:J27"/>
     <mergeCell ref="H7:H11"/>
+    <mergeCell ref="D99:D104"/>
+    <mergeCell ref="J68:J71"/>
     <mergeCell ref="E7:E11"/>
     <mergeCell ref="J43:J47"/>
     <mergeCell ref="I38:I42"/>
     <mergeCell ref="E3:K3"/>
     <mergeCell ref="K38:K42"/>
+    <mergeCell ref="C48:C67"/>
+    <mergeCell ref="K105:K108"/>
+    <mergeCell ref="H33:H37"/>
     <mergeCell ref="D68:D76"/>
+    <mergeCell ref="J33:J37"/>
     <mergeCell ref="I90:I92"/>
     <mergeCell ref="J72:J76"/>
     <mergeCell ref="K33:K37"/>
     <mergeCell ref="H28:H29"/>
+    <mergeCell ref="E4:K4"/>
     <mergeCell ref="H19:H24"/>
     <mergeCell ref="E113:E116"/>
     <mergeCell ref="J109:J112"/>
+    <mergeCell ref="I84:I85"/>
     <mergeCell ref="I109:I112"/>
     <mergeCell ref="E99:E101"/>
+    <mergeCell ref="I60:I67"/>
+    <mergeCell ref="I19:I24"/>
+    <mergeCell ref="K19:K24"/>
     <mergeCell ref="E68:E71"/>
+    <mergeCell ref="I102:I104"/>
+    <mergeCell ref="K102:K104"/>
+    <mergeCell ref="C80:C95"/>
     <mergeCell ref="E30:E32"/>
+    <mergeCell ref="K51:K59"/>
     <mergeCell ref="D48:D67"/>
+    <mergeCell ref="E51:E59"/>
+    <mergeCell ref="E77:E79"/>
     <mergeCell ref="I86:I89"/>
     <mergeCell ref="K12:K18"/>
+    <mergeCell ref="H99:H101"/>
     <mergeCell ref="J90:J92"/>
+    <mergeCell ref="H68:H71"/>
+    <mergeCell ref="K7:K11"/>
     <mergeCell ref="C96:C98"/>
     <mergeCell ref="K109:K112"/>
     <mergeCell ref="C28:C32"/>
     <mergeCell ref="H109:H112"/>
+    <mergeCell ref="E80:E83"/>
     <mergeCell ref="E96:E98"/>
     <mergeCell ref="E60:E67"/>
+    <mergeCell ref="E48:E50"/>
     <mergeCell ref="E72:E76"/>
     <mergeCell ref="J113:J116"/>
+    <mergeCell ref="H25:H27"/>
+    <mergeCell ref="J51:J59"/>
+    <mergeCell ref="J77:J79"/>
     <mergeCell ref="J99:J101"/>
     <mergeCell ref="H86:H89"/>
     <mergeCell ref="H80:H83"/>
+    <mergeCell ref="D80:D95"/>
+    <mergeCell ref="K28:K29"/>
+    <mergeCell ref="C105:C116"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="I25:I27"/>
+    <mergeCell ref="I72:I76"/>
+    <mergeCell ref="K99:K101"/>
     <mergeCell ref="I105:I108"/>
+    <mergeCell ref="E90:E92"/>
+    <mergeCell ref="C7:C27"/>
+    <mergeCell ref="K68:K71"/>
     <mergeCell ref="I93:I95"/>
+    <mergeCell ref="H72:H76"/>
     <mergeCell ref="I43:I47"/>
     <mergeCell ref="K43:K47"/>
     <mergeCell ref="K77:K79"/>
+    <mergeCell ref="H96:H98"/>
     <mergeCell ref="I113:I116"/>
-    <mergeCell ref="H96:H98"/>
     <mergeCell ref="J7:J11"/>
     <mergeCell ref="H90:H92"/>
+    <mergeCell ref="I33:I37"/>
     <mergeCell ref="H77:H79"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="E84:E85"/>
     <mergeCell ref="B48:B104"/>
+    <mergeCell ref="J80:J83"/>
     <mergeCell ref="J96:J98"/>
     <mergeCell ref="J60:J67"/>
+    <mergeCell ref="J48:J50"/>
     <mergeCell ref="E28:E29"/>
+    <mergeCell ref="K25:K27"/>
     <mergeCell ref="E19:E24"/>
     <mergeCell ref="E102:E104"/>
+    <mergeCell ref="H84:H85"/>
     <mergeCell ref="I51:I59"/>
+    <mergeCell ref="K60:K67"/>
+    <mergeCell ref="E12:E18"/>
+    <mergeCell ref="E86:E89"/>
+    <mergeCell ref="C99:C104"/>
     <mergeCell ref="H43:H47"/>
+    <mergeCell ref="H60:H67"/>
+    <mergeCell ref="C68:C76"/>
+    <mergeCell ref="H102:H104"/>
+    <mergeCell ref="J102:J104"/>
     <mergeCell ref="I7:I11"/>
+    <mergeCell ref="D77:D79"/>
+    <mergeCell ref="E109:E112"/>
     <mergeCell ref="E38:E42"/>
     <mergeCell ref="I96:I98"/>
     <mergeCell ref="K90:K92"/>
+    <mergeCell ref="E2:K2"/>
     <mergeCell ref="B7:B47"/>
     <mergeCell ref="J84:J85"/>
+    <mergeCell ref="H113:H116"/>
+    <mergeCell ref="C33:C47"/>
     <mergeCell ref="H51:H59"/>
+    <mergeCell ref="A7:A116"/>
     <mergeCell ref="J28:J29"/>
     <mergeCell ref="D28:D32"/>
     <mergeCell ref="J19:J24"/>
     <mergeCell ref="C77:C79"/>
     <mergeCell ref="I28:I29"/>
+    <mergeCell ref="K84:K85"/>
     <mergeCell ref="K113:K116"/>
-    <mergeCell ref="I99:I101"/>
-    <mergeCell ref="I68:I71"/>
-    <mergeCell ref="I30:I32"/>
-    <mergeCell ref="K30:K32"/>
-    <mergeCell ref="K86:K89"/>
-    <mergeCell ref="H105:H108"/>
-    <mergeCell ref="H38:H42"/>
-    <mergeCell ref="E33:E37"/>
-    <mergeCell ref="J38:J42"/>
-    <mergeCell ref="H93:H95"/>
-    <mergeCell ref="J93:J95"/>
-    <mergeCell ref="K96:K98"/>
-    <mergeCell ref="D99:D104"/>
-    <mergeCell ref="J68:J71"/>
-    <mergeCell ref="C48:C67"/>
-    <mergeCell ref="K105:K108"/>
-    <mergeCell ref="H33:H37"/>
-    <mergeCell ref="J33:J37"/>
-    <mergeCell ref="E4:K4"/>
-    <mergeCell ref="I84:I85"/>
-    <mergeCell ref="I60:I67"/>
-    <mergeCell ref="I19:I24"/>
-    <mergeCell ref="K19:K24"/>
-    <mergeCell ref="I102:I104"/>
-    <mergeCell ref="C80:C95"/>
-    <mergeCell ref="K102:K104"/>
-    <mergeCell ref="K51:K59"/>
-    <mergeCell ref="E51:E59"/>
-    <mergeCell ref="E77:E79"/>
-    <mergeCell ref="H99:H101"/>
-    <mergeCell ref="H68:H71"/>
-    <mergeCell ref="K7:K11"/>
-    <mergeCell ref="E80:E83"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="H25:H27"/>
-    <mergeCell ref="J51:J59"/>
-    <mergeCell ref="J77:J79"/>
-    <mergeCell ref="D80:D95"/>
-    <mergeCell ref="K28:K29"/>
-    <mergeCell ref="C105:C116"/>
-    <mergeCell ref="I72:I76"/>
-    <mergeCell ref="K99:K101"/>
-    <mergeCell ref="C7:C27"/>
-    <mergeCell ref="E90:E92"/>
-    <mergeCell ref="K68:K71"/>
-    <mergeCell ref="H72:H76"/>
-    <mergeCell ref="I33:I37"/>
-    <mergeCell ref="I80:I83"/>
-    <mergeCell ref="J80:J83"/>
-    <mergeCell ref="J48:J50"/>
-    <mergeCell ref="K25:K27"/>
-    <mergeCell ref="H84:H85"/>
-    <mergeCell ref="K60:K67"/>
-    <mergeCell ref="E12:E18"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="C99:C104"/>
-    <mergeCell ref="H60:H67"/>
-    <mergeCell ref="C68:C76"/>
-    <mergeCell ref="H102:H104"/>
-    <mergeCell ref="J102:J104"/>
-    <mergeCell ref="D77:D79"/>
-    <mergeCell ref="E109:E112"/>
-    <mergeCell ref="E2:K2"/>
-    <mergeCell ref="H113:H116"/>
-    <mergeCell ref="C33:C47"/>
-    <mergeCell ref="A7:A116"/>
-    <mergeCell ref="K84:K85"/>
     <mergeCell ref="H48:H50"/>
     <mergeCell ref="E25:E27"/>
     <mergeCell ref="H30:H32"/>
@@ -3788,17 +3773,30 @@
     <mergeCell ref="J12:J18"/>
     <mergeCell ref="J86:J89"/>
     <mergeCell ref="E105:E108"/>
+    <mergeCell ref="I99:I101"/>
     <mergeCell ref="K93:K95"/>
+    <mergeCell ref="I68:I71"/>
     <mergeCell ref="E93:E95"/>
     <mergeCell ref="B105:B116"/>
     <mergeCell ref="E43:E47"/>
+    <mergeCell ref="I30:I32"/>
     <mergeCell ref="D105:D116"/>
+    <mergeCell ref="K30:K32"/>
+    <mergeCell ref="K86:K89"/>
     <mergeCell ref="I77:I79"/>
     <mergeCell ref="D96:D98"/>
+    <mergeCell ref="H105:H108"/>
+    <mergeCell ref="H38:H42"/>
+    <mergeCell ref="E33:E37"/>
+    <mergeCell ref="J38:J42"/>
     <mergeCell ref="D7:D27"/>
     <mergeCell ref="D33:D47"/>
+    <mergeCell ref="H93:H95"/>
+    <mergeCell ref="J93:J95"/>
     <mergeCell ref="K72:K76"/>
+    <mergeCell ref="I12:I18"/>
     <mergeCell ref="J105:J108"/>
+    <mergeCell ref="I80:I83"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[SCRUM-39] docs: acuerdo de pedidos y reservas y plan del Sprint 2
</commit_message>
<xml_diff>
--- a/docs/SanMarkFood-Planificacion.xlsx
+++ b/docs/SanMarkFood-Planificacion.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" style="12" min="1" max="1"/>
@@ -625,7 +625,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="30" customHeight="1" s="12">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -1813,7 +1812,7 @@
       </c>
       <c r="K48" s="10" t="inlineStr">
         <is>
-          <t>Rodrigo Puente</t>
+          <t>Jose Chuque</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1842,7 @@
       <c r="B50" s="8" t="n"/>
       <c r="C50" s="8" t="n"/>
       <c r="D50" s="8" t="n"/>
-      <c r="E50" s="9" t="n"/>
+      <c r="E50" s="8" t="n"/>
       <c r="F50" s="14" t="inlineStr">
         <is>
           <t>Despliegue de las Cloud Functions en Firebase (plan Blaze), accesibles desde ambas apps</t>
@@ -1854,25 +1853,20 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H50" s="9" t="n"/>
-      <c r="I50" s="9" t="n"/>
-      <c r="J50" s="9" t="n"/>
-      <c r="K50" s="9" t="n"/>
-    </row>
-    <row r="51" ht="45" customHeight="1" s="12">
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="n"/>
+      <c r="K50" s="8" t="n"/>
+    </row>
+    <row r="51" ht="36" customHeight="1" s="12">
       <c r="A51" s="8" t="n"/>
       <c r="B51" s="8" t="n"/>
       <c r="C51" s="8" t="n"/>
       <c r="D51" s="8" t="n"/>
-      <c r="E51" s="14" t="inlineStr">
-        <is>
-          <t>HU08 - Pedido con pago y calificación (Comensal)
-Como comensal, quiero armar un pedido, confirmarlo con mi huella o rostro antes de pagar, ver su estado en tiempo real y calificarlo al finalizar, para pedir con seguridad y ayudar a otros usuarios con mi opinión.</t>
-        </is>
-      </c>
+      <c r="E51" s="8" t="n"/>
       <c r="F51" s="14" t="inlineStr">
         <is>
-          <t>Armado de pedido desde el menú con carrito de compras; el carrito admite platos de un solo local y, al agregar de otro, se pide confirmar si se vacía el pedido actual</t>
+          <t>Datos de ejemplo (pedidos, reservas y reseñas) cargados con un script, para que las apps se prueben sin esperar a las funciones</t>
         </is>
       </c>
       <c r="G51" s="10" t="inlineStr">
@@ -1880,26 +1874,10 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H51" s="14" t="inlineStr">
-        <is>
-          <t>BiometricPrompt (androidx.biometric); Firestore (estado en tiempo real); Room (carrito local); Retrofit (backend propio)</t>
-        </is>
-      </c>
-      <c r="I51" s="10" t="inlineStr">
-        <is>
-          <t>Semana 10</t>
-        </is>
-      </c>
-      <c r="J51" s="10" t="inlineStr">
-        <is>
-          <t>Semana 11</t>
-        </is>
-      </c>
-      <c r="K51" s="10" t="inlineStr">
-        <is>
-          <t>Camila Bada</t>
-        </is>
-      </c>
+      <c r="H51" s="8" t="n"/>
+      <c r="I51" s="8" t="n"/>
+      <c r="J51" s="8" t="n"/>
+      <c r="K51" s="8" t="n"/>
     </row>
     <row r="52" ht="36" customHeight="1" s="12">
       <c r="A52" s="8" t="n"/>
@@ -1909,7 +1887,7 @@
       <c r="E52" s="8" t="n"/>
       <c r="F52" s="14" t="inlineStr">
         <is>
-          <t>Selección de modalidad (recojo o delivery) y método de pago</t>
+          <t>La app del comensal guarda su token de avisos y muestra las notificaciones que envían las funciones</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr">
@@ -1927,10 +1905,10 @@
       <c r="B53" s="8" t="n"/>
       <c r="C53" s="8" t="n"/>
       <c r="D53" s="8" t="n"/>
-      <c r="E53" s="8" t="n"/>
+      <c r="E53" s="9" t="n"/>
       <c r="F53" s="14" t="inlineStr">
         <is>
-          <t>Confirmación biométrica (huella o rostro) antes de procesar el pago con billetera o tarjeta; el pago en efectivo se confirma sin biometría</t>
+          <t>Función resenas: guarda la calificación de un pedido entregado y actualiza la calificación promedio del local</t>
         </is>
       </c>
       <c r="G53" s="10" t="inlineStr">
@@ -1938,20 +1916,25 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H53" s="8" t="n"/>
-      <c r="I53" s="8" t="n"/>
-      <c r="J53" s="8" t="n"/>
-      <c r="K53" s="8" t="n"/>
-    </row>
-    <row r="54" ht="36" customHeight="1" s="12">
+      <c r="H53" s="9" t="n"/>
+      <c r="I53" s="9" t="n"/>
+      <c r="J53" s="9" t="n"/>
+      <c r="K53" s="9" t="n"/>
+    </row>
+    <row r="54" ht="45" customHeight="1" s="12">
       <c r="A54" s="8" t="n"/>
       <c r="B54" s="8" t="n"/>
       <c r="C54" s="8" t="n"/>
       <c r="D54" s="8" t="n"/>
-      <c r="E54" s="8" t="n"/>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>HU08 - Pedido con pago y calificación (Comensal)
+Como comensal, quiero armar un pedido, confirmarlo con mi huella o rostro antes de pagar, ver su estado en tiempo real y calificarlo al finalizar, para pedir con seguridad y ayudar a otros usuarios con mi opinión.</t>
+        </is>
+      </c>
       <c r="F54" s="14" t="inlineStr">
         <is>
-          <t>Seguimiento del estado del pedido en tiempo real</t>
+          <t>Armado de pedido desde el menú con carrito de compras; el carrito admite platos de un solo local y, al agregar de otro, se pide confirmar si se vacía el pedido actual</t>
         </is>
       </c>
       <c r="G54" s="10" t="inlineStr">
@@ -1959,10 +1942,26 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H54" s="8" t="n"/>
-      <c r="I54" s="8" t="n"/>
-      <c r="J54" s="8" t="n"/>
-      <c r="K54" s="8" t="n"/>
+      <c r="H54" s="14" t="inlineStr">
+        <is>
+          <t>BiometricPrompt (androidx.biometric); Firestore (estado en tiempo real); Room (carrito local); Retrofit (Cloud Functions y Geocoding API)</t>
+        </is>
+      </c>
+      <c r="I54" s="10" t="inlineStr">
+        <is>
+          <t>Semana 10</t>
+        </is>
+      </c>
+      <c r="J54" s="10" t="inlineStr">
+        <is>
+          <t>Semana 11</t>
+        </is>
+      </c>
+      <c r="K54" s="10" t="inlineStr">
+        <is>
+          <t>Camila Bada</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="36" customHeight="1" s="12">
       <c r="A55" s="8" t="n"/>
@@ -1972,7 +1971,7 @@
       <c r="E55" s="8" t="n"/>
       <c r="F55" s="14" t="inlineStr">
         <is>
-          <t>Calificación por pedido al finalizar: estrellas y comentario para el local, y «me gustó / no me gustó» opcional por cada plato</t>
+          <t>Selección de modalidad (recojo o delivery) y método de pago</t>
         </is>
       </c>
       <c r="G55" s="10" t="inlineStr">
@@ -1993,7 +1992,7 @@
       <c r="E56" s="8" t="n"/>
       <c r="F56" s="14" t="inlineStr">
         <is>
-          <t>Cancelación del pedido por el comensal, siempre que el restaurante aún no lo haya aceptado</t>
+          <t>Confirmación biométrica (huella o rostro) antes de procesar el pago con billetera o tarjeta; el pago en efectivo se confirma sin biometría</t>
         </is>
       </c>
       <c r="G56" s="10" t="inlineStr">
@@ -2014,7 +2013,7 @@
       <c r="E57" s="8" t="n"/>
       <c r="F57" s="14" t="inlineStr">
         <is>
-          <t>Armado del menú del día eligiendo 1 entrada y 1 segundo (refresco y postre incluidos); las opciones agotadas no se pueden elegir</t>
+          <t>Seguimiento del estado del pedido en tiempo real</t>
         </is>
       </c>
       <c r="G57" s="10" t="inlineStr">
@@ -2035,7 +2034,7 @@
       <c r="E58" s="8" t="n"/>
       <c r="F58" s="14" t="inlineStr">
         <is>
-          <t>Estado «Rechazado» en el seguimiento: muestra el motivo del restaurante (o el rechazo automático a los 10 min) e informa la reversión del pago simulado</t>
+          <t>Calificación por pedido al finalizar: estrellas y comentario para el local, y «me gustó / no me gustó» opcional por cada plato</t>
         </is>
       </c>
       <c r="G58" s="10" t="inlineStr">
@@ -2053,10 +2052,10 @@
       <c r="B59" s="8" t="n"/>
       <c r="C59" s="8" t="n"/>
       <c r="D59" s="8" t="n"/>
-      <c r="E59" s="9" t="n"/>
+      <c r="E59" s="8" t="n"/>
       <c r="F59" s="14" t="inlineStr">
         <is>
-          <t>El menú del día solo se puede pedir hasta la hora de fin publicada o hasta que se agoten sus entradas o segundos; si vence con el menú en el pedido, se avisa al confirmar y se retira del pedido</t>
+          <t>Cancelación del pedido por el comensal, siempre que el restaurante aún no lo haya aceptado</t>
         </is>
       </c>
       <c r="G59" s="10" t="inlineStr">
@@ -2064,25 +2063,20 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H59" s="9" t="n"/>
-      <c r="I59" s="9" t="n"/>
-      <c r="J59" s="9" t="n"/>
-      <c r="K59" s="9" t="n"/>
-    </row>
-    <row r="60" ht="45" customHeight="1" s="12">
+      <c r="H59" s="8" t="n"/>
+      <c r="I59" s="8" t="n"/>
+      <c r="J59" s="8" t="n"/>
+      <c r="K59" s="8" t="n"/>
+    </row>
+    <row r="60" ht="36" customHeight="1" s="12">
       <c r="A60" s="8" t="n"/>
       <c r="B60" s="8" t="n"/>
       <c r="C60" s="8" t="n"/>
       <c r="D60" s="8" t="n"/>
-      <c r="E60" s="14" t="inlineStr">
-        <is>
-          <t>HU09 - Gestión de pedidos entrantes (Restaurante)
-Como restaurante, quiero ver los pedidos entrantes y actualizar su estado, para que el comensal sepa cuándo estará listo su pedido.</t>
-        </is>
-      </c>
+      <c r="E60" s="8" t="n"/>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>Listado de pedidos entrantes ordenado por hora de llegada</t>
+          <t>Armado del menú del día eligiendo 1 entrada y 1 segundo (refresco y postre incluidos); las opciones agotadas no se pueden elegir</t>
         </is>
       </c>
       <c r="G60" s="10" t="inlineStr">
@@ -2090,26 +2084,10 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H60" s="14" t="inlineStr">
-        <is>
-          <t>Firestore (listener en tiempo real); WorkManager (sincronización en background); Firebase Cloud Messaging</t>
-        </is>
-      </c>
-      <c r="I60" s="10" t="inlineStr">
-        <is>
-          <t>Semana 10</t>
-        </is>
-      </c>
-      <c r="J60" s="10" t="inlineStr">
-        <is>
-          <t>Semana 11</t>
-        </is>
-      </c>
-      <c r="K60" s="10" t="inlineStr">
-        <is>
-          <t>Jose Chuque</t>
-        </is>
-      </c>
+      <c r="H60" s="8" t="n"/>
+      <c r="I60" s="8" t="n"/>
+      <c r="J60" s="8" t="n"/>
+      <c r="K60" s="8" t="n"/>
     </row>
     <row r="61" ht="36" customHeight="1" s="12">
       <c r="A61" s="8" t="n"/>
@@ -2119,7 +2097,7 @@
       <c r="E61" s="8" t="n"/>
       <c r="F61" s="14" t="inlineStr">
         <is>
-          <t>Cambio de estado del pedido (recibido, preparando, listo/en camino, entregado)</t>
+          <t>Estado «Rechazado» en el seguimiento: muestra el motivo del restaurante (o el rechazo automático a los 10 min) e informa la reversión del pago simulado</t>
         </is>
       </c>
       <c r="G61" s="10" t="inlineStr">
@@ -2140,7 +2118,7 @@
       <c r="E62" s="8" t="n"/>
       <c r="F62" s="14" t="inlineStr">
         <is>
-          <t>Notificación push al comensal cuando cambia el estado</t>
+          <t>El menú del día solo se puede pedir hasta la hora de fin publicada o hasta que se agoten sus entradas o segundos; si vence con el menú en el pedido, se avisa al confirmar y se retira del pedido</t>
         </is>
       </c>
       <c r="G62" s="10" t="inlineStr">
@@ -2158,10 +2136,10 @@
       <c r="B63" s="8" t="n"/>
       <c r="C63" s="8" t="n"/>
       <c r="D63" s="8" t="n"/>
-      <c r="E63" s="8" t="n"/>
+      <c r="E63" s="9" t="n"/>
       <c r="F63" s="14" t="inlineStr">
         <is>
-          <t>Rechazo de un pedido entrante con motivo obligatorio (plato agotado, cocina saturada, local por cerrar u otro)</t>
+          <t>La dirección de delivery se convierte en coordenadas con la Geocoding API de Google, consumida con Retrofit + corrutinas</t>
         </is>
       </c>
       <c r="G63" s="10" t="inlineStr">
@@ -2169,20 +2147,25 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H63" s="8" t="n"/>
-      <c r="I63" s="8" t="n"/>
-      <c r="J63" s="8" t="n"/>
-      <c r="K63" s="8" t="n"/>
-    </row>
-    <row r="64" ht="36" customHeight="1" s="12">
+      <c r="H63" s="9" t="n"/>
+      <c r="I63" s="9" t="n"/>
+      <c r="J63" s="9" t="n"/>
+      <c r="K63" s="9" t="n"/>
+    </row>
+    <row r="64" ht="45" customHeight="1" s="12">
       <c r="A64" s="8" t="n"/>
       <c r="B64" s="8" t="n"/>
       <c r="C64" s="8" t="n"/>
       <c r="D64" s="8" t="n"/>
-      <c r="E64" s="8" t="n"/>
+      <c r="E64" s="14" t="inlineStr">
+        <is>
+          <t>HU09 - Gestión de pedidos entrantes (Restaurante)
+Como restaurante, quiero ver los pedidos entrantes y actualizar su estado, para que el comensal sepa cuándo estará listo su pedido.</t>
+        </is>
+      </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>Rechazo automático del pedido si el restaurante no lo acepta en 10 minutos, con aviso push al comensal</t>
+          <t>Listado de pedidos entrantes ordenado por hora de llegada</t>
         </is>
       </c>
       <c r="G64" s="10" t="inlineStr">
@@ -2190,10 +2173,26 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H64" s="8" t="n"/>
-      <c r="I64" s="8" t="n"/>
-      <c r="J64" s="8" t="n"/>
-      <c r="K64" s="8" t="n"/>
+      <c r="H64" s="14" t="inlineStr">
+        <is>
+          <t>Firestore (listener en tiempo real); WorkManager (sincronización en background); Firebase Cloud Messaging</t>
+        </is>
+      </c>
+      <c r="I64" s="10" t="inlineStr">
+        <is>
+          <t>Semana 10</t>
+        </is>
+      </c>
+      <c r="J64" s="10" t="inlineStr">
+        <is>
+          <t>Semana 11</t>
+        </is>
+      </c>
+      <c r="K64" s="10" t="inlineStr">
+        <is>
+          <t>Jose Chuque</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="36" customHeight="1" s="12">
       <c r="A65" s="8" t="n"/>
@@ -2203,7 +2202,7 @@
       <c r="E65" s="8" t="n"/>
       <c r="F65" s="14" t="inlineStr">
         <is>
-          <t>Aviso de pedido nuevo con notificación de alta prioridad y sonido que se repite hasta abrirlo, y cuenta regresiva de los 10 min en la app</t>
+          <t>Cambio de estado del pedido (recibido, preparando, listo/en camino, entregado)</t>
         </is>
       </c>
       <c r="G65" s="10" t="inlineStr">
@@ -2224,7 +2223,7 @@
       <c r="E66" s="8" t="n"/>
       <c r="F66" s="14" t="inlineStr">
         <is>
-          <t>Al aceptar un pedido, el local elige el tiempo estimado (10, 15, 20 o 30 min), con el que se calcula la hora que ve el comensal</t>
+          <t>Notificación push al comensal cuando cambia el estado</t>
         </is>
       </c>
       <c r="G66" s="10" t="inlineStr">
@@ -2240,12 +2239,12 @@
     <row r="67" ht="36" customHeight="1" s="12">
       <c r="A67" s="8" t="n"/>
       <c r="B67" s="8" t="n"/>
-      <c r="C67" s="9" t="n"/>
-      <c r="D67" s="9" t="n"/>
-      <c r="E67" s="9" t="n"/>
+      <c r="C67" s="8" t="n"/>
+      <c r="D67" s="8" t="n"/>
+      <c r="E67" s="8" t="n"/>
       <c r="F67" s="14" t="inlineStr">
         <is>
-          <t>Entrega de pedidos de recojo escribiendo el código de 4 dígitos del comensal; sin código se puede marcar entregado con confirmación</t>
+          <t>Rechazo de un pedido entrante con motivo obligatorio (plato agotado, cocina saturada, local por cerrar u otro)</t>
         </is>
       </c>
       <c r="G67" s="10" t="inlineStr">
@@ -2253,34 +2252,20 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H67" s="9" t="n"/>
-      <c r="I67" s="9" t="n"/>
-      <c r="J67" s="9" t="n"/>
-      <c r="K67" s="9" t="n"/>
-    </row>
-    <row r="68" ht="45" customHeight="1" s="12">
+      <c r="H67" s="8" t="n"/>
+      <c r="I67" s="8" t="n"/>
+      <c r="J67" s="8" t="n"/>
+      <c r="K67" s="8" t="n"/>
+    </row>
+    <row r="68" ht="36" customHeight="1" s="12">
       <c r="A68" s="8" t="n"/>
       <c r="B68" s="8" t="n"/>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>Reservas:
-Solicitud de reserva por el comensal y su gestión por parte del restaurante.</t>
-        </is>
-      </c>
-      <c r="D68" s="10" t="inlineStr">
-        <is>
-          <t>Comensal / Restaurante</t>
-        </is>
-      </c>
-      <c r="E68" s="14" t="inlineStr">
-        <is>
-          <t>HU10 - Reserva de mesa (Comensal)
-Como comensal, quiero reservar una mesa en un restaurante para una fecha y hora determinada, para asegurar mi lugar antes de llegar.</t>
-        </is>
-      </c>
+      <c r="C68" s="8" t="n"/>
+      <c r="D68" s="8" t="n"/>
+      <c r="E68" s="8" t="n"/>
       <c r="F68" s="14" t="inlineStr">
         <is>
-          <t>Selección de fecha, hora y número de comensales: entre 2 h y 7 días de anticipación, horarios cada 30 min dentro del horario del local, de 1 a 10 comensales y máximo 2 reservas activas por comensal</t>
+          <t>Rechazo automático del pedido si el restaurante no lo acepta en 10 minutos, con aviso push al comensal</t>
         </is>
       </c>
       <c r="G68" s="10" t="inlineStr">
@@ -2288,26 +2273,10 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H68" s="14" t="inlineStr">
-        <is>
-          <t>WorkManager (recordatorios); Firebase Cloud Messaging; Firestore</t>
-        </is>
-      </c>
-      <c r="I68" s="10" t="inlineStr">
-        <is>
-          <t>Semana 9</t>
-        </is>
-      </c>
-      <c r="J68" s="10" t="inlineStr">
-        <is>
-          <t>Semana 10</t>
-        </is>
-      </c>
-      <c r="K68" s="10" t="inlineStr">
-        <is>
-          <t>Camila Bada</t>
-        </is>
-      </c>
+      <c r="H68" s="8" t="n"/>
+      <c r="I68" s="8" t="n"/>
+      <c r="J68" s="8" t="n"/>
+      <c r="K68" s="8" t="n"/>
     </row>
     <row r="69" ht="36" customHeight="1" s="12">
       <c r="A69" s="8" t="n"/>
@@ -2317,7 +2286,7 @@
       <c r="E69" s="8" t="n"/>
       <c r="F69" s="14" t="inlineStr">
         <is>
-          <t>Recordatorio de la reserva antes de la hora programada, con anticipación elegible (30 min, 1 h o 2 h)</t>
+          <t>Aviso de pedido nuevo con notificación de alta prioridad y sonido que se repite hasta abrirlo, y cuenta regresiva de los 10 min en la app</t>
         </is>
       </c>
       <c r="G69" s="10" t="inlineStr">
@@ -2338,7 +2307,7 @@
       <c r="E70" s="8" t="n"/>
       <c r="F70" s="14" t="inlineStr">
         <is>
-          <t>Cancelación de la reserva desde la app</t>
+          <t>Al aceptar un pedido, el local elige el tiempo estimado (10, 15, 20 o 30 min), con el que se calcula la hora que ve el comensal</t>
         </is>
       </c>
       <c r="G70" s="10" t="inlineStr">
@@ -2354,12 +2323,12 @@
     <row r="71" ht="36" customHeight="1" s="12">
       <c r="A71" s="8" t="n"/>
       <c r="B71" s="8" t="n"/>
-      <c r="C71" s="8" t="n"/>
-      <c r="D71" s="8" t="n"/>
+      <c r="C71" s="9" t="n"/>
+      <c r="D71" s="9" t="n"/>
       <c r="E71" s="9" t="n"/>
       <c r="F71" s="14" t="inlineStr">
         <is>
-          <t>Modificar la fecha u hora de una reserva ya creada, sin cancelarla; el cambio libera el horario anterior y la reserva vuelve a quedar pendiente de confirmación</t>
+          <t>Entrega de pedidos de recojo escribiendo el código de 4 dígitos del comensal; sin código se puede marcar entregado con confirmación</t>
         </is>
       </c>
       <c r="G71" s="10" t="inlineStr">
@@ -2375,17 +2344,26 @@
     <row r="72" ht="45" customHeight="1" s="12">
       <c r="A72" s="8" t="n"/>
       <c r="B72" s="8" t="n"/>
-      <c r="C72" s="8" t="n"/>
-      <c r="D72" s="8" t="n"/>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>Reservas:
+Solicitud de reserva por el comensal y su gestión por parte del restaurante.</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>Comensal / Restaurante</t>
+        </is>
+      </c>
       <c r="E72" s="14" t="inlineStr">
         <is>
-          <t>HU12 - Gestión de reservas entrantes (Restaurante)
-Como restaurante, quiero ver las reservas entrantes y confirmarlas o rechazarlas, para organizar la disponibilidad de mesas de mi local.</t>
+          <t>HU10 - Reserva de mesa (Comensal)
+Como comensal, quiero reservar una mesa en un restaurante para una fecha y hora determinada, para asegurar mi lugar antes de llegar.</t>
         </is>
       </c>
       <c r="F72" s="14" t="inlineStr">
         <is>
-          <t>Listado de reservas del día ordenado por hora</t>
+          <t>Selección de fecha, hora y número de comensales: entre 2 h y 7 días de anticipación, horarios cada 30 min dentro del horario del local, de 1 a 10 comensales y máximo 2 reservas activas por comensal</t>
         </is>
       </c>
       <c r="G72" s="10" t="inlineStr">
@@ -2395,7 +2373,7 @@
       </c>
       <c r="H72" s="14" t="inlineStr">
         <is>
-          <t>Firestore (listener en tiempo real); Firebase Cloud Messaging</t>
+          <t>WorkManager (recordatorios); Firebase Cloud Messaging; Firestore</t>
         </is>
       </c>
       <c r="I72" s="10" t="inlineStr">
@@ -2410,7 +2388,7 @@
       </c>
       <c r="K72" s="10" t="inlineStr">
         <is>
-          <t>Jose Chuque</t>
+          <t>Camila Bada</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2400,7 @@
       <c r="E73" s="8" t="n"/>
       <c r="F73" s="14" t="inlineStr">
         <is>
-          <t>Confirmación o rechazo de una reserva entrante; el rechazo exige un motivo de una lista (sin mesas a esa hora, local cerrado ese día, grupo demasiado grande) u «Otro» con texto</t>
+          <t>Recordatorio de la reserva antes de la hora programada, con anticipación elegible (30 min, 1 h o 2 h), programado con WorkManager</t>
         </is>
       </c>
       <c r="G73" s="10" t="inlineStr">
@@ -2443,7 +2421,7 @@
       <c r="E74" s="8" t="n"/>
       <c r="F74" s="14" t="inlineStr">
         <is>
-          <t>Notificación push al comensal con la respuesta y, si se rechazó, el motivo</t>
+          <t>Cancelación de la reserva desde la app</t>
         </is>
       </c>
       <c r="G74" s="10" t="inlineStr">
@@ -2461,10 +2439,10 @@
       <c r="B75" s="8" t="n"/>
       <c r="C75" s="8" t="n"/>
       <c r="D75" s="8" t="n"/>
-      <c r="E75" s="8" t="n"/>
+      <c r="E75" s="9" t="n"/>
       <c r="F75" s="14" t="inlineStr">
         <is>
-          <t>Rechazo automático de la reserva si el restaurante no responde hasta 60 min antes de la hora reservada, con aviso push al comensal</t>
+          <t>Modificar la fecha u hora de una reserva ya creada, sin cancelarla; el cambio libera el horario anterior y la reserva vuelve a quedar pendiente de confirmación</t>
         </is>
       </c>
       <c r="G75" s="10" t="inlineStr">
@@ -2472,20 +2450,25 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H75" s="8" t="n"/>
-      <c r="I75" s="8" t="n"/>
-      <c r="J75" s="8" t="n"/>
-      <c r="K75" s="8" t="n"/>
-    </row>
-    <row r="76" ht="36" customHeight="1" s="12">
+      <c r="H75" s="9" t="n"/>
+      <c r="I75" s="9" t="n"/>
+      <c r="J75" s="9" t="n"/>
+      <c r="K75" s="9" t="n"/>
+    </row>
+    <row r="76" ht="45" customHeight="1" s="12">
       <c r="A76" s="8" t="n"/>
       <c r="B76" s="8" t="n"/>
-      <c r="C76" s="9" t="n"/>
-      <c r="D76" s="9" t="n"/>
-      <c r="E76" s="9" t="n"/>
+      <c r="C76" s="8" t="n"/>
+      <c r="D76" s="8" t="n"/>
+      <c r="E76" s="14" t="inlineStr">
+        <is>
+          <t>HU12 - Gestión de reservas entrantes (Restaurante)
+Como restaurante, quiero ver las reservas entrantes y confirmarlas o rechazarlas, para organizar la disponibilidad de mesas de mi local.</t>
+        </is>
+      </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
-          <t>Cupo de reservas por franja de 30 min (número de comensales) configurable por el local; las franjas llenas, sumando reservas pendientes y confirmadas, no se pueden reservar</t>
+          <t>Listado de reservas del día ordenado por hora</t>
         </is>
       </c>
       <c r="G76" s="10" t="inlineStr">
@@ -2493,34 +2476,36 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H76" s="9" t="n"/>
-      <c r="I76" s="9" t="n"/>
-      <c r="J76" s="9" t="n"/>
-      <c r="K76" s="9" t="n"/>
-    </row>
-    <row r="77" ht="45" customHeight="1" s="12">
+      <c r="H76" s="14" t="inlineStr">
+        <is>
+          <t>Firestore (listener en tiempo real); Firebase Cloud Messaging</t>
+        </is>
+      </c>
+      <c r="I76" s="10" t="inlineStr">
+        <is>
+          <t>Semana 9</t>
+        </is>
+      </c>
+      <c r="J76" s="10" t="inlineStr">
+        <is>
+          <t>Semana 10</t>
+        </is>
+      </c>
+      <c r="K76" s="10" t="inlineStr">
+        <is>
+          <t>Jose Chuque</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="36" customHeight="1" s="12">
       <c r="A77" s="8" t="n"/>
       <c r="B77" s="8" t="n"/>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>Actividad del Comensal:
-Historial de pedidos y reservas pasadas, para consulta y repetición rápida.</t>
-        </is>
-      </c>
-      <c r="D77" s="10" t="inlineStr">
-        <is>
-          <t>Comensal</t>
-        </is>
-      </c>
-      <c r="E77" s="14" t="inlineStr">
-        <is>
-          <t>HU20 - Historial de pedidos y reservas
-Como comensal, quiero ver el historial de mis pedidos y reservas pasadas, para llevar un registro de mi actividad y repetir un pedido anterior fácilmente.</t>
-        </is>
-      </c>
+      <c r="C77" s="8" t="n"/>
+      <c r="D77" s="8" t="n"/>
+      <c r="E77" s="8" t="n"/>
       <c r="F77" s="14" t="inlineStr">
         <is>
-          <t>Listado de pedidos y reservas pasadas, ordenado por fecha</t>
+          <t>Confirmación o rechazo de una reserva entrante; el rechazo exige un motivo de una lista (sin mesas a esa hora, local cerrado ese día, grupo demasiado grande) u «Otro» con texto</t>
         </is>
       </c>
       <c r="G77" s="10" t="inlineStr">
@@ -2528,26 +2513,10 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H77" s="14" t="inlineStr">
-        <is>
-          <t>Firestore (historial); Retrofit + corrutinas (backend propio); Jetpack Compose</t>
-        </is>
-      </c>
-      <c r="I77" s="10" t="inlineStr">
-        <is>
-          <t>Semana 11</t>
-        </is>
-      </c>
-      <c r="J77" s="10" t="inlineStr">
-        <is>
-          <t>Semana 12</t>
-        </is>
-      </c>
-      <c r="K77" s="10" t="inlineStr">
-        <is>
-          <t>Camila Bada</t>
-        </is>
-      </c>
+      <c r="H77" s="8" t="n"/>
+      <c r="I77" s="8" t="n"/>
+      <c r="J77" s="8" t="n"/>
+      <c r="K77" s="8" t="n"/>
     </row>
     <row r="78" ht="36" customHeight="1" s="12">
       <c r="A78" s="8" t="n"/>
@@ -2557,7 +2526,7 @@
       <c r="E78" s="8" t="n"/>
       <c r="F78" s="14" t="inlineStr">
         <is>
-          <t>Detalle de cada pedido o reserva pasado (restaurante, ítems, estado final)</t>
+          <t>Notificación push al comensal con la respuesta y, si se rechazó, el motivo</t>
         </is>
       </c>
       <c r="G78" s="10" t="inlineStr">
@@ -2573,12 +2542,12 @@
     <row r="79" ht="36" customHeight="1" s="12">
       <c r="A79" s="8" t="n"/>
       <c r="B79" s="8" t="n"/>
-      <c r="C79" s="9" t="n"/>
-      <c r="D79" s="9" t="n"/>
-      <c r="E79" s="9" t="n"/>
+      <c r="C79" s="8" t="n"/>
+      <c r="D79" s="8" t="n"/>
+      <c r="E79" s="8" t="n"/>
       <c r="F79" s="14" t="inlineStr">
         <is>
-          <t>Opción de “repetir pedido” que precarga el carrito con los mismos ítems; si incluía menú del día, se eligen entrada y segundo del menú de hoy</t>
+          <t>Rechazo automático de la reserva si el restaurante no responde hasta 60 min antes de la hora reservada, con aviso push al comensal</t>
         </is>
       </c>
       <c r="G79" s="10" t="inlineStr">
@@ -2586,92 +2555,92 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H79" s="9" t="n"/>
-      <c r="I79" s="9" t="n"/>
-      <c r="J79" s="9" t="n"/>
-      <c r="K79" s="9" t="n"/>
-    </row>
-    <row r="80" ht="45" customHeight="1" s="12">
+      <c r="H79" s="8" t="n"/>
+      <c r="I79" s="8" t="n"/>
+      <c r="J79" s="8" t="n"/>
+      <c r="K79" s="8" t="n"/>
+    </row>
+    <row r="80" ht="36" customHeight="1" s="12">
       <c r="A80" s="8" t="n"/>
       <c r="B80" s="8" t="n"/>
-      <c r="C80" s="10" t="inlineStr">
+      <c r="C80" s="9" t="n"/>
+      <c r="D80" s="9" t="n"/>
+      <c r="E80" s="9" t="n"/>
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>Cupo de reservas por franja de 30 min (número de comensales) configurable por el local; las franjas llenas, sumando reservas pendientes y confirmadas, no se pueden reservar</t>
+        </is>
+      </c>
+      <c r="G80" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H80" s="9" t="n"/>
+      <c r="I80" s="9" t="n"/>
+      <c r="J80" s="9" t="n"/>
+      <c r="K80" s="9" t="n"/>
+    </row>
+    <row r="81" ht="45" customHeight="1" s="12">
+      <c r="A81" s="8" t="n"/>
+      <c r="B81" s="8" t="n"/>
+      <c r="C81" s="8" t="inlineStr">
         <is>
           <t>Chatbot y Reseñas con IA:
 Atención conversacional para el comensal, y el sistema completo de reseñas: resumen y alerta con IA, visualización de detalle, y respuesta del restaurante.</t>
         </is>
       </c>
-      <c r="D80" s="10" t="inlineStr">
+      <c r="D81" s="8" t="inlineStr">
         <is>
           <t>Comensal / Restaurante / Backend</t>
         </is>
       </c>
-      <c r="E80" s="14" t="inlineStr">
-        <is>
-          <t>HU11 - Chatbot de atención con entrada por voz
-Como comensal, quiero consultar a un chatbot (por texto o por voz) sobre horarios, disponibilidad o el estado de mi reserva/pedido, para resolver dudas rápidas sin llamar al restaurante.</t>
-        </is>
-      </c>
-      <c r="F80" s="14" t="inlineStr">
-        <is>
-          <t>Chat conversacional accesible desde la pantalla de un restaurante</t>
-        </is>
-      </c>
-      <c r="G80" s="10" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H80" s="14" t="inlineStr">
-        <is>
-          <t>SpeechRecognizer (entrada de voz); API de un LLM (vía Retrofit + corrutinas); Jetpack Compose</t>
-        </is>
-      </c>
-      <c r="I80" s="10" t="inlineStr">
+      <c r="E81" s="14" t="inlineStr">
+        <is>
+          <t>HU14 - Resumen de reseñas (Comensal)
+Como comensal, quiero ver un resumen breve de las opiniones de un restaurante, para decidir si me conviene sin leer cada reseña una por una.</t>
+        </is>
+      </c>
+      <c r="F81" s="14" t="inlineStr">
+        <is>
+          <t>Generación de un resumen de 2-3 líneas a partir de las reseñas recientes</t>
+        </is>
+      </c>
+      <c r="G81" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H81" s="14" t="inlineStr">
+        <is>
+          <t>Cloud Function programada (resumenResenas) que genera el resumen con Gemini; Firestore (caché del resumen con timestamp)</t>
+        </is>
+      </c>
+      <c r="I81" s="10" t="inlineStr">
         <is>
           <t>Semana 11</t>
         </is>
       </c>
-      <c r="J80" s="10" t="inlineStr">
-        <is>
-          <t>Semana 12</t>
-        </is>
-      </c>
-      <c r="K80" s="10" t="inlineStr">
-        <is>
-          <t>Jose Chuque</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="36" customHeight="1" s="12">
-      <c r="A81" s="8" t="n"/>
-      <c r="B81" s="8" t="n"/>
-      <c r="C81" s="8" t="n"/>
-      <c r="D81" s="8" t="n"/>
-      <c r="E81" s="8" t="n"/>
-      <c r="F81" s="14" t="inlineStr">
-        <is>
-          <t>Entrada por voz mediante reconocimiento de habla, como alternativa al texto</t>
-        </is>
-      </c>
-      <c r="G81" s="10" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H81" s="8" t="n"/>
-      <c r="I81" s="8" t="n"/>
-      <c r="J81" s="8" t="n"/>
-      <c r="K81" s="8" t="n"/>
+      <c r="J81" s="10" t="inlineStr">
+        <is>
+          <t>Semana 11</t>
+        </is>
+      </c>
+      <c r="K81" s="10" t="inlineStr">
+        <is>
+          <t>Rodrigo Puente</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="36" customHeight="1" s="12">
       <c r="A82" s="8" t="n"/>
       <c r="B82" s="8" t="n"/>
       <c r="C82" s="8" t="n"/>
       <c r="D82" s="8" t="n"/>
-      <c r="E82" s="8" t="n"/>
+      <c r="E82" s="9" t="n"/>
       <c r="F82" s="14" t="inlineStr">
         <is>
-          <t>Respuestas sobre horarios, menú y disponibilidad de ese restaurante</t>
+          <t>Resumen cacheado y regenerado solo cada cierto tiempo, no en cada visita</t>
         </is>
       </c>
       <c r="G82" s="10" t="inlineStr">
@@ -2679,20 +2648,25 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H82" s="8" t="n"/>
-      <c r="I82" s="8" t="n"/>
-      <c r="J82" s="8" t="n"/>
-      <c r="K82" s="8" t="n"/>
-    </row>
-    <row r="83" ht="36" customHeight="1" s="12">
+      <c r="H82" s="9" t="n"/>
+      <c r="I82" s="9" t="n"/>
+      <c r="J82" s="9" t="n"/>
+      <c r="K82" s="9" t="n"/>
+    </row>
+    <row r="83" ht="45" customHeight="1" s="12">
       <c r="A83" s="8" t="n"/>
       <c r="B83" s="8" t="n"/>
       <c r="C83" s="8" t="n"/>
       <c r="D83" s="8" t="n"/>
-      <c r="E83" s="9" t="n"/>
+      <c r="E83" s="14" t="inlineStr">
+        <is>
+          <t>HU15 - Alerta de reseñas negativas (Restaurante)
+Como restaurante, quiero recibir una alerta cuando llega una reseña negativa, para poder responder o corregir el problema a tiempo.</t>
+        </is>
+      </c>
       <c r="F83" s="14" t="inlineStr">
         <is>
-          <t>Consulta del estado de una reserva o pedido activo mediante el chat</t>
+          <t>Clasificación automática del sentimiento de cada reseña nueva (positivo/negativo/neutro)</t>
         </is>
       </c>
       <c r="G83" s="10" t="inlineStr">
@@ -2700,25 +2674,36 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H83" s="9" t="n"/>
-      <c r="I83" s="9" t="n"/>
-      <c r="J83" s="9" t="n"/>
-      <c r="K83" s="9" t="n"/>
-    </row>
-    <row r="84" ht="45" customHeight="1" s="12">
+      <c r="H83" s="14" t="inlineStr">
+        <is>
+          <t>Cloud Functions for Firebase (trigger en Firestore); Gemini (clasificación del sentimiento); Firebase Cloud Messaging</t>
+        </is>
+      </c>
+      <c r="I83" s="10" t="inlineStr">
+        <is>
+          <t>Semana 11</t>
+        </is>
+      </c>
+      <c r="J83" s="10" t="inlineStr">
+        <is>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="K83" s="10" t="inlineStr">
+        <is>
+          <t>Rodrigo Puente</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="36" customHeight="1" s="12">
       <c r="A84" s="8" t="n"/>
       <c r="B84" s="8" t="n"/>
       <c r="C84" s="8" t="n"/>
       <c r="D84" s="8" t="n"/>
-      <c r="E84" s="14" t="inlineStr">
-        <is>
-          <t>HU14 - Resumen de reseñas (Comensal)
-Como comensal, quiero ver un resumen breve de las opiniones de un restaurante, para decidir si me conviene sin leer cada reseña una por una.</t>
-        </is>
-      </c>
+      <c r="E84" s="8" t="n"/>
       <c r="F84" s="14" t="inlineStr">
         <is>
-          <t>Generación de un resumen de 2-3 líneas a partir de las reseñas recientes</t>
+          <t>Extracción del motivo principal cuando la reseña es negativa</t>
         </is>
       </c>
       <c r="G84" s="10" t="inlineStr">
@@ -2726,36 +2711,20 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H84" s="14" t="inlineStr">
-        <is>
-          <t>Cloud Function programada (resumenResenas) que genera el resumen con Gemini; Firestore (caché del resumen con timestamp)</t>
-        </is>
-      </c>
-      <c r="I84" s="10" t="inlineStr">
-        <is>
-          <t>Semana 11</t>
-        </is>
-      </c>
-      <c r="J84" s="10" t="inlineStr">
-        <is>
-          <t>Semana 11</t>
-        </is>
-      </c>
-      <c r="K84" s="10" t="inlineStr">
-        <is>
-          <t>Rodrigo Puente</t>
-        </is>
-      </c>
+      <c r="H84" s="8" t="n"/>
+      <c r="I84" s="8" t="n"/>
+      <c r="J84" s="8" t="n"/>
+      <c r="K84" s="8" t="n"/>
     </row>
     <row r="85" ht="36" customHeight="1" s="12">
       <c r="A85" s="8" t="n"/>
-      <c r="B85" s="8" t="n"/>
+      <c r="B85" s="9" t="n"/>
       <c r="C85" s="8" t="n"/>
       <c r="D85" s="8" t="n"/>
       <c r="E85" s="9" t="n"/>
       <c r="F85" s="14" t="inlineStr">
         <is>
-          <t>Resumen cacheado y regenerado solo cada cierto tiempo, no en cada visita</t>
+          <t>Notificación push al restaurante ante una reseña clasificada como negativa</t>
         </is>
       </c>
       <c r="G85" s="10" t="inlineStr">
@@ -2770,18 +2739,29 @@
     </row>
     <row r="86" ht="45" customHeight="1" s="12">
       <c r="A86" s="8" t="n"/>
-      <c r="B86" s="8" t="n"/>
-      <c r="C86" s="8" t="n"/>
-      <c r="D86" s="8" t="n"/>
+      <c r="B86" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>Actividad del Comensal:
+Historial de pedidos y reservas pasadas, para consulta y repetición rápida.</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>Comensal</t>
+        </is>
+      </c>
       <c r="E86" s="14" t="inlineStr">
         <is>
-          <t>HU22 - Ver detalle de reseñas de un restaurante (Comensal)
-Como comensal, quiero ver el listado completo de reseñas de un restaurante (autor, calificación, comentario, fecha), para revisar el detalle si el resumen de IA no me es suficiente.</t>
+          <t>HU20 - Historial de pedidos y reservas
+Como comensal, quiero ver el historial de mis pedidos y reservas pasadas, para llevar un registro de mi actividad y repetir un pedido anterior fácilmente.</t>
         </is>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
-          <t>Listado de reseñas ordenado por fecha, con calificación y comentario</t>
+          <t>Listado de pedidos y reservas pasadas, ordenado por fecha</t>
         </is>
       </c>
       <c r="G86" s="10" t="inlineStr">
@@ -2791,17 +2771,17 @@
       </c>
       <c r="H86" s="14" t="inlineStr">
         <is>
-          <t>Firestore (colección de reseñas); Jetpack Compose</t>
+          <t>Firestore (historial); Retrofit + corrutinas (backend propio); Jetpack Compose</t>
         </is>
       </c>
       <c r="I86" s="10" t="inlineStr">
         <is>
-          <t>Semana 11</t>
+          <t>Semana 13</t>
         </is>
       </c>
       <c r="J86" s="10" t="inlineStr">
         <is>
-          <t>Semana 12</t>
+          <t>Semana 14</t>
         </is>
       </c>
       <c r="K86" s="10" t="inlineStr">
@@ -2818,7 +2798,7 @@
       <c r="E87" s="8" t="n"/>
       <c r="F87" s="14" t="inlineStr">
         <is>
-          <t>Filtro por calificación (1 a 5 estrellas)</t>
+          <t>Detalle de cada pedido o reserva pasado (restaurante, ítems, estado final)</t>
         </is>
       </c>
       <c r="G87" s="10" t="inlineStr">
@@ -2834,12 +2814,12 @@
     <row r="88" ht="36" customHeight="1" s="12">
       <c r="A88" s="8" t="n"/>
       <c r="B88" s="8" t="n"/>
-      <c r="C88" s="8" t="n"/>
-      <c r="D88" s="8" t="n"/>
-      <c r="E88" s="8" t="n"/>
+      <c r="C88" s="9" t="n"/>
+      <c r="D88" s="9" t="n"/>
+      <c r="E88" s="9" t="n"/>
       <c r="F88" s="14" t="inlineStr">
         <is>
-          <t>Se muestra la respuesta del restaurante debajo de la reseña, si existe</t>
+          <t>Opción de “repetir pedido” que precarga el carrito con los mismos ítems; si incluía menú del día, se eligen entrada y segundo del menú de hoy</t>
         </is>
       </c>
       <c r="G88" s="10" t="inlineStr">
@@ -2847,20 +2827,34 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H88" s="8" t="n"/>
-      <c r="I88" s="8" t="n"/>
-      <c r="J88" s="8" t="n"/>
-      <c r="K88" s="8" t="n"/>
-    </row>
-    <row r="89" ht="36" customHeight="1" s="12">
+      <c r="H88" s="9" t="n"/>
+      <c r="I88" s="9" t="n"/>
+      <c r="J88" s="9" t="n"/>
+      <c r="K88" s="9" t="n"/>
+    </row>
+    <row r="89" ht="45" customHeight="1" s="12">
       <c r="A89" s="8" t="n"/>
       <c r="B89" s="8" t="n"/>
-      <c r="C89" s="8" t="n"/>
-      <c r="D89" s="8" t="n"/>
-      <c r="E89" s="9" t="n"/>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>Chatbot y Reseñas con IA:
+Atención conversacional para el comensal, y el sistema completo de reseñas: resumen y alerta con IA, visualización de detalle, y respuesta del restaurante.</t>
+        </is>
+      </c>
+      <c r="D89" s="10" t="inlineStr">
+        <is>
+          <t>Comensal / Restaurante / Backend</t>
+        </is>
+      </c>
+      <c r="E89" s="14" t="inlineStr">
+        <is>
+          <t>HU11 - Chatbot de atención con entrada por voz
+Como comensal, quiero consultar a un chatbot (por texto o por voz) sobre horarios, disponibilidad o el estado de mi reserva/pedido, para resolver dudas rápidas sin llamar al restaurante.</t>
+        </is>
+      </c>
       <c r="F89" s="14" t="inlineStr">
         <is>
-          <t>Reportar una reseña ajena con motivo (ofensiva, falsa, spam u otro); cada comensal puede reportarla una sola vez y la reseña pasa a la cola de moderación de HU25</t>
+          <t>Chat conversacional accesible desde la pantalla de un restaurante</t>
         </is>
       </c>
       <c r="G89" s="10" t="inlineStr">
@@ -2868,25 +2862,36 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H89" s="9" t="n"/>
-      <c r="I89" s="9" t="n"/>
-      <c r="J89" s="9" t="n"/>
-      <c r="K89" s="9" t="n"/>
-    </row>
-    <row r="90" ht="45" customHeight="1" s="12">
+      <c r="H89" s="14" t="inlineStr">
+        <is>
+          <t>SpeechRecognizer (entrada de voz); Gemini vía Firebase AI Logic, con los datos del local y del pedido o reserva leídos de Firestore; Jetpack Compose</t>
+        </is>
+      </c>
+      <c r="I89" s="10" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="J89" s="10" t="inlineStr">
+        <is>
+          <t>Semana 14</t>
+        </is>
+      </c>
+      <c r="K89" s="10" t="inlineStr">
+        <is>
+          <t>Camila Bada</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="36" customHeight="1" s="12">
       <c r="A90" s="8" t="n"/>
       <c r="B90" s="8" t="n"/>
       <c r="C90" s="8" t="n"/>
       <c r="D90" s="8" t="n"/>
-      <c r="E90" s="14" t="inlineStr">
-        <is>
-          <t>HU15 - Alerta de reseñas negativas (Restaurante)
-Como restaurante, quiero recibir una alerta cuando llega una reseña negativa, para poder responder o corregir el problema a tiempo.</t>
-        </is>
-      </c>
+      <c r="E90" s="8" t="n"/>
       <c r="F90" s="14" t="inlineStr">
         <is>
-          <t>Clasificación automática del sentimiento de cada reseña nueva (positivo/negativo/neutro)</t>
+          <t>Entrada por voz mediante reconocimiento de habla, como alternativa al texto</t>
         </is>
       </c>
       <c r="G90" s="10" t="inlineStr">
@@ -2894,26 +2899,10 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H90" s="14" t="inlineStr">
-        <is>
-          <t>Cloud Functions for Firebase (trigger en Firestore); API de un LLM; Firebase Cloud Messaging</t>
-        </is>
-      </c>
-      <c r="I90" s="10" t="inlineStr">
-        <is>
-          <t>Semana 11</t>
-        </is>
-      </c>
-      <c r="J90" s="10" t="inlineStr">
-        <is>
-          <t>Semana 12</t>
-        </is>
-      </c>
-      <c r="K90" s="10" t="inlineStr">
-        <is>
-          <t>Rodrigo Puente</t>
-        </is>
-      </c>
+      <c r="H90" s="8" t="n"/>
+      <c r="I90" s="8" t="n"/>
+      <c r="J90" s="8" t="n"/>
+      <c r="K90" s="8" t="n"/>
     </row>
     <row r="91" ht="36" customHeight="1" s="12">
       <c r="A91" s="8" t="n"/>
@@ -2923,7 +2912,7 @@
       <c r="E91" s="8" t="n"/>
       <c r="F91" s="14" t="inlineStr">
         <is>
-          <t>Extracción del motivo principal cuando la reseña es negativa</t>
+          <t>Respuestas sobre horarios, menú y disponibilidad de ese restaurante</t>
         </is>
       </c>
       <c r="G91" s="10" t="inlineStr">
@@ -2944,7 +2933,7 @@
       <c r="E92" s="9" t="n"/>
       <c r="F92" s="14" t="inlineStr">
         <is>
-          <t>Notificación push al restaurante ante una reseña clasificada como negativa</t>
+          <t>Consulta del estado de una reserva o pedido activo mediante el chat</t>
         </is>
       </c>
       <c r="G92" s="10" t="inlineStr">
@@ -2964,13 +2953,13 @@
       <c r="D93" s="8" t="n"/>
       <c r="E93" s="14" t="inlineStr">
         <is>
-          <t>HU21 - Gestión y respuesta a reseñas (Restaurante)
-Como restaurante, quiero ver todas mis reseñas recibidas y responder a cualquiera de ellas, para mostrar que atiendo la retroalimentación de mis comensales, no solo las negativas.</t>
+          <t>HU22 - Ver detalle de reseñas de un restaurante (Comensal)
+Como comensal, quiero ver el listado completo de reseñas de un restaurante (autor, calificación, comentario, fecha), para revisar el detalle si el resumen de IA no me es suficiente.</t>
         </is>
       </c>
       <c r="F93" s="14" t="inlineStr">
         <is>
-          <t>Listado completo de reseñas recibidas, no solo las negativas</t>
+          <t>Listado de reseñas ordenado por fecha, con calificación y comentario</t>
         </is>
       </c>
       <c r="G93" s="10" t="inlineStr">
@@ -2980,22 +2969,22 @@
       </c>
       <c r="H93" s="14" t="inlineStr">
         <is>
-          <t>Firestore (subcolección de respuestas); Firebase Cloud Messaging</t>
+          <t>Firestore (colección de reseñas); Jetpack Compose</t>
         </is>
       </c>
       <c r="I93" s="10" t="inlineStr">
         <is>
-          <t>Semana 11</t>
+          <t>Semana 13</t>
         </is>
       </c>
       <c r="J93" s="10" t="inlineStr">
         <is>
-          <t>Semana 12</t>
+          <t>Semana 13</t>
         </is>
       </c>
       <c r="K93" s="10" t="inlineStr">
         <is>
-          <t>Jose Chuque</t>
+          <t>Camila Bada</t>
         </is>
       </c>
     </row>
@@ -3007,7 +2996,7 @@
       <c r="E94" s="8" t="n"/>
       <c r="F94" s="14" t="inlineStr">
         <is>
-          <t>Responder públicamente a cualquier reseña</t>
+          <t>Filtro por calificación (1 a 5 estrellas)</t>
         </is>
       </c>
       <c r="G94" s="10" t="inlineStr">
@@ -3023,12 +3012,12 @@
     <row r="95" ht="36" customHeight="1" s="12">
       <c r="A95" s="8" t="n"/>
       <c r="B95" s="8" t="n"/>
-      <c r="C95" s="9" t="n"/>
-      <c r="D95" s="9" t="n"/>
-      <c r="E95" s="9" t="n"/>
+      <c r="C95" s="8" t="n"/>
+      <c r="D95" s="8" t="n"/>
+      <c r="E95" s="8" t="n"/>
       <c r="F95" s="14" t="inlineStr">
         <is>
-          <t>Notificación al comensal cuando su reseña recibe respuesta</t>
+          <t>Se muestra la respuesta del restaurante debajo de la reseña, si existe</t>
         </is>
       </c>
       <c r="G95" s="10" t="inlineStr">
@@ -3036,34 +3025,20 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H95" s="9" t="n"/>
-      <c r="I95" s="9" t="n"/>
-      <c r="J95" s="9" t="n"/>
-      <c r="K95" s="9" t="n"/>
-    </row>
-    <row r="96" ht="45" customHeight="1" s="12">
+      <c r="H95" s="8" t="n"/>
+      <c r="I95" s="8" t="n"/>
+      <c r="J95" s="8" t="n"/>
+      <c r="K95" s="8" t="n"/>
+    </row>
+    <row r="96" ht="36" customHeight="1" s="12">
       <c r="A96" s="8" t="n"/>
       <c r="B96" s="8" t="n"/>
-      <c r="C96" s="10" t="inlineStr">
-        <is>
-          <t>Moderación de la Plataforma (Administrador):
-Revisión y moderación de las reseñas del sistema.</t>
-        </is>
-      </c>
-      <c r="D96" s="10" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-      <c r="E96" s="14" t="inlineStr">
-        <is>
-          <t>HU25 - Moderación de reseñas
-Como administrador, quiero revisar y eliminar una reseña reportada como abusiva o falsa, para mantener la confianza del sistema de reseñas.</t>
-        </is>
-      </c>
+      <c r="C96" s="8" t="n"/>
+      <c r="D96" s="8" t="n"/>
+      <c r="E96" s="9" t="n"/>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>Listado de reseñas reportadas o marcadas para revisión</t>
+          <t>Reportar una reseña ajena con motivo (ofensiva, falsa, spam u otro); cada comensal puede reportarla una sola vez y la reseña pasa a la cola de moderación de HU25</t>
         </is>
       </c>
       <c r="G96" s="10" t="inlineStr">
@@ -3071,36 +3046,25 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H96" s="14" t="inlineStr">
-        <is>
-          <t>Firestore (listener de reseñas reportadas); Cloud Functions for Firebase</t>
-        </is>
-      </c>
-      <c r="I96" s="10" t="inlineStr">
-        <is>
-          <t>Semana 11</t>
-        </is>
-      </c>
-      <c r="J96" s="10" t="inlineStr">
-        <is>
-          <t>Semana 12</t>
-        </is>
-      </c>
-      <c r="K96" s="10" t="inlineStr">
-        <is>
-          <t>Camila Bada</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="36" customHeight="1" s="12">
+      <c r="H96" s="9" t="n"/>
+      <c r="I96" s="9" t="n"/>
+      <c r="J96" s="9" t="n"/>
+      <c r="K96" s="9" t="n"/>
+    </row>
+    <row r="97" ht="45" customHeight="1" s="12">
       <c r="A97" s="8" t="n"/>
       <c r="B97" s="8" t="n"/>
       <c r="C97" s="8" t="n"/>
       <c r="D97" s="8" t="n"/>
-      <c r="E97" s="8" t="n"/>
+      <c r="E97" s="14" t="inlineStr">
+        <is>
+          <t>HU21 - Gestión y respuesta a reseñas (Restaurante)
+Como restaurante, quiero ver todas mis reseñas recibidas y responder a cualquiera de ellas, para mostrar que atiendo la retroalimentación de mis comensales, no solo las negativas.</t>
+        </is>
+      </c>
       <c r="F97" s="14" t="inlineStr">
         <is>
-          <t>Eliminar una reseña clasificada como abusiva o falsa</t>
+          <t>Listado completo de reseñas recibidas, no solo las negativas</t>
         </is>
       </c>
       <c r="G97" s="10" t="inlineStr">
@@ -3108,20 +3072,36 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H97" s="8" t="n"/>
-      <c r="I97" s="8" t="n"/>
-      <c r="J97" s="8" t="n"/>
-      <c r="K97" s="8" t="n"/>
+      <c r="H97" s="14" t="inlineStr">
+        <is>
+          <t>Firestore (subcolección de respuestas); Firebase Cloud Messaging</t>
+        </is>
+      </c>
+      <c r="I97" s="10" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="J97" s="10" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="K97" s="10" t="inlineStr">
+        <is>
+          <t>Jose Chuque</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="36" customHeight="1" s="12">
       <c r="A98" s="8" t="n"/>
       <c r="B98" s="8" t="n"/>
-      <c r="C98" s="9" t="n"/>
-      <c r="D98" s="9" t="n"/>
-      <c r="E98" s="9" t="n"/>
+      <c r="C98" s="8" t="n"/>
+      <c r="D98" s="8" t="n"/>
+      <c r="E98" s="8" t="n"/>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>Registro de la acción de moderación realizada</t>
+          <t>Responder públicamente a cualquier reseña</t>
         </is>
       </c>
       <c r="G98" s="10" t="inlineStr">
@@ -3129,34 +3109,20 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H98" s="9" t="n"/>
-      <c r="I98" s="9" t="n"/>
-      <c r="J98" s="9" t="n"/>
-      <c r="K98" s="9" t="n"/>
-    </row>
-    <row r="99" ht="45" customHeight="1" s="12">
+      <c r="H98" s="8" t="n"/>
+      <c r="I98" s="8" t="n"/>
+      <c r="J98" s="8" t="n"/>
+      <c r="K98" s="8" t="n"/>
+    </row>
+    <row r="99" ht="36" customHeight="1" s="12">
       <c r="A99" s="8" t="n"/>
       <c r="B99" s="8" t="n"/>
-      <c r="C99" s="10" t="inlineStr">
-        <is>
-          <t>Dashboard de Restaurante y de Plataforma:
-Panel de indicadores del negocio para el restaurante, y panel agregado de la plataforma para el administrador.</t>
-        </is>
-      </c>
-      <c r="D99" s="10" t="inlineStr">
-        <is>
-          <t>Restaurante / Administrador</t>
-        </is>
-      </c>
-      <c r="E99" s="14" t="inlineStr">
-        <is>
-          <t>HU13 - Dashboard de restaurante
-Como restaurante, quiero ver un dashboard con mis ventas, platos más pedidos y calificación promedio, para entender cómo va mi negocio en la app.</t>
-        </is>
-      </c>
+      <c r="C99" s="9" t="n"/>
+      <c r="D99" s="9" t="n"/>
+      <c r="E99" s="9" t="n"/>
       <c r="F99" s="14" t="inlineStr">
         <is>
-          <t>Gráfico de ventas/pedidos por día o semana</t>
+          <t>Notificación al comensal cuando su reseña recibe respuesta</t>
         </is>
       </c>
       <c r="G99" s="10" t="inlineStr">
@@ -3164,36 +3130,34 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H99" s="14" t="inlineStr">
-        <is>
-          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de pedidos y calificaciones)</t>
-        </is>
-      </c>
-      <c r="I99" s="10" t="inlineStr">
-        <is>
-          <t>Semana 12</t>
-        </is>
-      </c>
-      <c r="J99" s="10" t="inlineStr">
-        <is>
-          <t>Semana 12</t>
-        </is>
-      </c>
-      <c r="K99" s="10" t="inlineStr">
-        <is>
-          <t>Jose Chuque</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="36" customHeight="1" s="12">
+      <c r="H99" s="9" t="n"/>
+      <c r="I99" s="9" t="n"/>
+      <c r="J99" s="9" t="n"/>
+      <c r="K99" s="9" t="n"/>
+    </row>
+    <row r="100" ht="45" customHeight="1" s="12">
       <c r="A100" s="8" t="n"/>
       <c r="B100" s="8" t="n"/>
-      <c r="C100" s="8" t="n"/>
-      <c r="D100" s="8" t="n"/>
-      <c r="E100" s="8" t="n"/>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>Moderación de la Plataforma (Administrador):
+Revisión y moderación de las reseñas del sistema.</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="E100" s="14" t="inlineStr">
+        <is>
+          <t>HU25 - Moderación de reseñas
+Como administrador, quiero revisar y eliminar una reseña reportada como abusiva o falsa, para mantener la confianza del sistema de reseñas.</t>
+        </is>
+      </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>Ranking de platos más pedidos</t>
+          <t>Listado de reseñas reportadas o marcadas para revisión</t>
         </is>
       </c>
       <c r="G100" s="10" t="inlineStr">
@@ -3201,20 +3165,36 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H100" s="8" t="n"/>
-      <c r="I100" s="8" t="n"/>
-      <c r="J100" s="8" t="n"/>
-      <c r="K100" s="8" t="n"/>
+      <c r="H100" s="14" t="inlineStr">
+        <is>
+          <t>Firestore (listener de reseñas reportadas); Cloud Functions for Firebase</t>
+        </is>
+      </c>
+      <c r="I100" s="10" t="inlineStr">
+        <is>
+          <t>Semana 11</t>
+        </is>
+      </c>
+      <c r="J100" s="10" t="inlineStr">
+        <is>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="K100" s="10" t="inlineStr">
+        <is>
+          <t>Jose Chuque</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="36" customHeight="1" s="12">
       <c r="A101" s="8" t="n"/>
       <c r="B101" s="8" t="n"/>
       <c r="C101" s="8" t="n"/>
       <c r="D101" s="8" t="n"/>
-      <c r="E101" s="9" t="n"/>
+      <c r="E101" s="8" t="n"/>
       <c r="F101" s="14" t="inlineStr">
         <is>
-          <t>Calificación promedio y su evolución en el tiempo</t>
+          <t>Eliminar una reseña clasificada como abusiva o falsa</t>
         </is>
       </c>
       <c r="G101" s="10" t="inlineStr">
@@ -3222,25 +3202,20 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H101" s="9" t="n"/>
-      <c r="I101" s="9" t="n"/>
-      <c r="J101" s="9" t="n"/>
-      <c r="K101" s="9" t="n"/>
-    </row>
-    <row r="102" ht="45" customHeight="1" s="12">
+      <c r="H101" s="8" t="n"/>
+      <c r="I101" s="8" t="n"/>
+      <c r="J101" s="8" t="n"/>
+      <c r="K101" s="8" t="n"/>
+    </row>
+    <row r="102" ht="36" customHeight="1" s="12">
       <c r="A102" s="8" t="n"/>
       <c r="B102" s="8" t="n"/>
-      <c r="C102" s="8" t="n"/>
-      <c r="D102" s="8" t="n"/>
-      <c r="E102" s="14" t="inlineStr">
-        <is>
-          <t>HU26 - Dashboard global (Administrador)
-Como administrador, quiero ver métricas agregadas de toda la plataforma (restaurantes activos, pedidos totales), para monitorear la salud del negocio.</t>
-        </is>
-      </c>
+      <c r="C102" s="9" t="n"/>
+      <c r="D102" s="9" t="n"/>
+      <c r="E102" s="9" t="n"/>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>Métricas agregadas de todos los restaurantes: restaurantes activos y pedidos totales</t>
+          <t>Registro de la acción de moderación realizada</t>
         </is>
       </c>
       <c r="G102" s="10" t="inlineStr">
@@ -3248,36 +3223,34 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H102" s="14" t="inlineStr">
-        <is>
-          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de locales y pedidos); Cloud Functions</t>
-        </is>
-      </c>
-      <c r="I102" s="10" t="inlineStr">
-        <is>
-          <t>Semana 12</t>
-        </is>
-      </c>
-      <c r="J102" s="10" t="inlineStr">
-        <is>
-          <t>Semana 12</t>
-        </is>
-      </c>
-      <c r="K102" s="10" t="inlineStr">
-        <is>
-          <t>Rodrigo Puente</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="36" customHeight="1" s="12">
+      <c r="H102" s="9" t="n"/>
+      <c r="I102" s="9" t="n"/>
+      <c r="J102" s="9" t="n"/>
+      <c r="K102" s="9" t="n"/>
+    </row>
+    <row r="103" ht="45" customHeight="1" s="12">
       <c r="A103" s="8" t="n"/>
       <c r="B103" s="8" t="n"/>
-      <c r="C103" s="8" t="n"/>
-      <c r="D103" s="8" t="n"/>
-      <c r="E103" s="8" t="n"/>
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard de Restaurante y de Plataforma:
+Panel de indicadores del negocio para el restaurante, y panel agregado de la plataforma para el administrador.</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>Restaurante / Administrador</t>
+        </is>
+      </c>
+      <c r="E103" s="14" t="inlineStr">
+        <is>
+          <t>HU13 - Dashboard de restaurante
+Como restaurante, quiero ver un dashboard con mis ventas, platos más pedidos y calificación promedio, para entender cómo va mi negocio en la app.</t>
+        </is>
+      </c>
       <c r="F103" s="14" t="inlineStr">
         <is>
-          <t>El dashboard obtiene las métricas con consultas de agregación de Firestore (count, sum), sin backend propio; lo que no se pueda agregar así lo calcula una Cloud Function</t>
+          <t>Gráfico de ventas/pedidos por día o semana</t>
         </is>
       </c>
       <c r="G103" s="10" t="inlineStr">
@@ -3285,20 +3258,36 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H103" s="8" t="n"/>
-      <c r="I103" s="8" t="n"/>
-      <c r="J103" s="8" t="n"/>
-      <c r="K103" s="8" t="n"/>
+      <c r="H103" s="14" t="inlineStr">
+        <is>
+          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de pedidos y calificaciones)</t>
+        </is>
+      </c>
+      <c r="I103" s="10" t="inlineStr">
+        <is>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="J103" s="10" t="inlineStr">
+        <is>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="K103" s="10" t="inlineStr">
+        <is>
+          <t>Jose Chuque</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="36" customHeight="1" s="12">
       <c r="A104" s="8" t="n"/>
-      <c r="B104" s="9" t="n"/>
-      <c r="C104" s="9" t="n"/>
-      <c r="D104" s="9" t="n"/>
-      <c r="E104" s="9" t="n"/>
+      <c r="B104" s="8" t="n"/>
+      <c r="C104" s="8" t="n"/>
+      <c r="D104" s="8" t="n"/>
+      <c r="E104" s="8" t="n"/>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>Gráfico de evolución de pedidos totales por semana</t>
+          <t>Ranking de platos más pedidos</t>
         </is>
       </c>
       <c r="G104" s="10" t="inlineStr">
@@ -3306,84 +3295,73 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H104" s="9" t="n"/>
-      <c r="I104" s="9" t="n"/>
-      <c r="J104" s="9" t="n"/>
-      <c r="K104" s="9" t="n"/>
-    </row>
-    <row r="105" ht="45" customHeight="1" s="12">
+      <c r="H104" s="8" t="n"/>
+      <c r="I104" s="8" t="n"/>
+      <c r="J104" s="8" t="n"/>
+      <c r="K104" s="8" t="n"/>
+    </row>
+    <row r="105" ht="36" customHeight="1" s="12">
       <c r="A105" s="8" t="n"/>
-      <c r="B105" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="C105" s="7" t="inlineStr">
-        <is>
-          <t>Seguridad, Pruebas y Despliegue:
-Asegurar, probar y publicar ambas aplicaciones.</t>
-        </is>
-      </c>
-      <c r="D105" s="7" t="inlineStr">
-        <is>
-          <t>Ambas</t>
-        </is>
-      </c>
-      <c r="E105" s="11" t="inlineStr">
-        <is>
-          <t>HU16 - Aseguramiento con OWASP Mobile
-Como equipo, queremos aplicar buenas prácticas de seguridad móvil OWASP, para proteger los datos de comensales y restaurantes en ambas apps.</t>
-        </is>
-      </c>
-      <c r="F105" s="11" t="inlineStr">
-        <is>
-          <t>Revisión de almacenamiento seguro de credenciales y tokens</t>
-        </is>
-      </c>
-      <c r="G105" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H105" s="11" t="inlineStr">
-        <is>
-          <t>OWASP MASVS/MSTG (checklist); ProGuard/R8; EncryptedSharedPreferences</t>
-        </is>
-      </c>
-      <c r="I105" s="7" t="inlineStr">
-        <is>
-          <t>Semana 13</t>
-        </is>
-      </c>
-      <c r="J105" s="7" t="inlineStr">
-        <is>
-          <t>Semana 13</t>
-        </is>
-      </c>
-      <c r="K105" s="7" t="inlineStr">
-        <is>
-          <t>Rodrigo Puente</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="36" customHeight="1" s="12">
+      <c r="B105" s="8" t="n"/>
+      <c r="C105" s="8" t="n"/>
+      <c r="D105" s="8" t="n"/>
+      <c r="E105" s="9" t="n"/>
+      <c r="F105" s="14" t="inlineStr">
+        <is>
+          <t>Calificación promedio y su evolución en el tiempo</t>
+        </is>
+      </c>
+      <c r="G105" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H105" s="9" t="n"/>
+      <c r="I105" s="9" t="n"/>
+      <c r="J105" s="9" t="n"/>
+      <c r="K105" s="9" t="n"/>
+    </row>
+    <row r="106" ht="45" customHeight="1" s="12">
       <c r="A106" s="8" t="n"/>
       <c r="B106" s="8" t="n"/>
       <c r="C106" s="8" t="n"/>
       <c r="D106" s="8" t="n"/>
-      <c r="E106" s="8" t="n"/>
-      <c r="F106" s="11" t="inlineStr">
-        <is>
-          <t>Ofuscación de código y protección contra ingeniería inversa</t>
-        </is>
-      </c>
-      <c r="G106" s="7" t="inlineStr">
-        <is>
-          <t>Sin Empezar</t>
-        </is>
-      </c>
-      <c r="H106" s="8" t="n"/>
-      <c r="I106" s="8" t="n"/>
-      <c r="J106" s="8" t="n"/>
-      <c r="K106" s="8" t="n"/>
+      <c r="E106" s="14" t="inlineStr">
+        <is>
+          <t>HU26 - Dashboard global (Administrador)
+Como administrador, quiero ver métricas agregadas de toda la plataforma (restaurantes activos, pedidos totales), para monitorear la salud del negocio.</t>
+        </is>
+      </c>
+      <c r="F106" s="14" t="inlineStr">
+        <is>
+          <t>Métricas agregadas de todos los restaurantes: restaurantes activos y pedidos totales</t>
+        </is>
+      </c>
+      <c r="G106" s="10" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H106" s="14" t="inlineStr">
+        <is>
+          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de locales y pedidos); Cloud Functions</t>
+        </is>
+      </c>
+      <c r="I106" s="10" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="J106" s="10" t="inlineStr">
+        <is>
+          <t>Semana 14</t>
+        </is>
+      </c>
+      <c r="K106" s="10" t="inlineStr">
+        <is>
+          <t>Rodrigo Puente</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="36" customHeight="1" s="12">
       <c r="A107" s="8" t="n"/>
@@ -3391,12 +3369,12 @@
       <c r="C107" s="8" t="n"/>
       <c r="D107" s="8" t="n"/>
       <c r="E107" s="8" t="n"/>
-      <c r="F107" s="11" t="inlineStr">
-        <is>
-          <t>Validación de comunicación segura (HTTPS/TLS) con el backend y Firebase</t>
-        </is>
-      </c>
-      <c r="G107" s="7" t="inlineStr">
+      <c r="F107" s="14" t="inlineStr">
+        <is>
+          <t>El dashboard obtiene las métricas con consultas de agregación de Firestore (count, sum), sin backend propio; lo que no se pueda agregar así lo calcula una Cloud Function</t>
+        </is>
+      </c>
+      <c r="G107" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3409,15 +3387,15 @@
     <row r="108" ht="36" customHeight="1" s="12">
       <c r="A108" s="8" t="n"/>
       <c r="B108" s="8" t="n"/>
-      <c r="C108" s="8" t="n"/>
-      <c r="D108" s="8" t="n"/>
+      <c r="C108" s="9" t="n"/>
+      <c r="D108" s="9" t="n"/>
       <c r="E108" s="9" t="n"/>
-      <c r="F108" s="11" t="inlineStr">
-        <is>
-          <t>Validación de que solo el rol administrador puede acceder a los endpoints y reglas de agregación global</t>
-        </is>
-      </c>
-      <c r="G108" s="7" t="inlineStr">
+      <c r="F108" s="14" t="inlineStr">
+        <is>
+          <t>Gráfico de evolución de pedidos totales por semana</t>
+        </is>
+      </c>
+      <c r="G108" s="10" t="inlineStr">
         <is>
           <t>Sin Empezar</t>
         </is>
@@ -3430,17 +3408,26 @@
     <row r="109" ht="45" customHeight="1" s="12">
       <c r="A109" s="8" t="n"/>
       <c r="B109" s="8" t="n"/>
-      <c r="C109" s="8" t="n"/>
-      <c r="D109" s="8" t="n"/>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad, Pruebas y Despliegue:
+Asegurar, probar y publicar ambas aplicaciones.</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="inlineStr">
+        <is>
+          <t>Ambas</t>
+        </is>
+      </c>
       <c r="E109" s="11" t="inlineStr">
         <is>
-          <t>HU17 - Pruebas y corrección de observaciones
-Como equipo, queremos probar ambas aplicaciones de forma integral y levantar las observaciones de los sprints anteriores, para asegurar la calidad antes del despliegue final.</t>
+          <t>HU16 - Aseguramiento con OWASP Mobile
+Como equipo, queremos aplicar buenas prácticas de seguridad móvil OWASP, para proteger los datos de comensales y restaurantes en ambas apps.</t>
         </is>
       </c>
       <c r="F109" s="11" t="inlineStr">
         <is>
-          <t>Pruebas unitarias de ViewModels y casos de uso principales en ambas apps</t>
+          <t>Revisión de almacenamiento seguro de credenciales y tokens</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
@@ -3450,17 +3437,17 @@
       </c>
       <c r="H109" s="11" t="inlineStr">
         <is>
-          <t>JUnit; Espresso / Compose Testing; Firebase Test Lab</t>
+          <t>OWASP MASVS/MSTG (checklist); ProGuard/R8; EncryptedSharedPreferences</t>
         </is>
       </c>
       <c r="I109" s="7" t="inlineStr">
         <is>
-          <t>Semana 14</t>
+          <t>Semana 13</t>
         </is>
       </c>
       <c r="J109" s="7" t="inlineStr">
         <is>
-          <t>Semana 14</t>
+          <t>Semana 13</t>
         </is>
       </c>
       <c r="K109" s="7" t="inlineStr">
@@ -3477,7 +3464,7 @@
       <c r="E110" s="8" t="n"/>
       <c r="F110" s="11" t="inlineStr">
         <is>
-          <t>Pruebas de UI de los flujos críticos (registro, pedido, reserva)</t>
+          <t>Ofuscación de código y protección contra ingeniería inversa</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
@@ -3498,7 +3485,7 @@
       <c r="E111" s="8" t="n"/>
       <c r="F111" s="11" t="inlineStr">
         <is>
-          <t>Ejecución en Firebase Test Lab en distintos dispositivos</t>
+          <t>Validación de comunicación segura (HTTPS/TLS) con el backend y Firebase</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">
@@ -3519,7 +3506,7 @@
       <c r="E112" s="9" t="n"/>
       <c r="F112" s="11" t="inlineStr">
         <is>
-          <t>Corrección de observaciones formuladas en la sustentación del 2do Sprint</t>
+          <t>Validación de que solo el rol administrador puede acceder a los endpoints y reglas de agregación global</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
@@ -3539,13 +3526,13 @@
       <c r="D113" s="8" t="n"/>
       <c r="E113" s="11" t="inlineStr">
         <is>
-          <t>HU18 - Despliegue en Google Play Store (2 apps)
-Como equipo, queremos publicar ambas aplicaciones en Google Play Store, para que estén disponibles públicamente al finalizar el curso.</t>
+          <t>HU17 - Pruebas y corrección de observaciones
+Como equipo, queremos probar ambas aplicaciones de forma integral y levantar las observaciones de los sprints anteriores, para asegurar la calidad antes del despliegue final.</t>
         </is>
       </c>
       <c r="F113" s="11" t="inlineStr">
         <is>
-          <t>Generación del bundle firmado (AAB) de cada app</t>
+          <t>Pruebas unitarias de ViewModels y casos de uso principales en ambas apps</t>
         </is>
       </c>
       <c r="G113" s="7" t="inlineStr">
@@ -3555,17 +3542,17 @@
       </c>
       <c r="H113" s="11" t="inlineStr">
         <is>
-          <t>Play App Signing; Google Play Console; Firebase App Distribution</t>
+          <t>JUnit; Espresso / Compose Testing; Firebase Test Lab</t>
         </is>
       </c>
       <c r="I113" s="7" t="inlineStr">
         <is>
-          <t>Semana 15</t>
+          <t>Semana 14</t>
         </is>
       </c>
       <c r="J113" s="7" t="inlineStr">
         <is>
-          <t>Semana 15</t>
+          <t>Semana 14</t>
         </is>
       </c>
       <c r="K113" s="7" t="inlineStr">
@@ -3582,7 +3569,7 @@
       <c r="E114" s="8" t="n"/>
       <c r="F114" s="11" t="inlineStr">
         <is>
-          <t>Configuración de la ficha de cada app en Play Console</t>
+          <t>Pruebas de UI de los flujos críticos (registro, pedido, reserva)</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
@@ -3603,7 +3590,7 @@
       <c r="E115" s="8" t="n"/>
       <c r="F115" s="11" t="inlineStr">
         <is>
-          <t>Distribución beta previa con Firebase App Distribution</t>
+          <t>Ejecución en Firebase Test Lab en distintos dispositivos</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
@@ -3617,14 +3604,14 @@
       <c r="K115" s="8" t="n"/>
     </row>
     <row r="116" ht="36" customHeight="1" s="12">
-      <c r="A116" s="9" t="n"/>
-      <c r="B116" s="9" t="n"/>
-      <c r="C116" s="9" t="n"/>
-      <c r="D116" s="9" t="n"/>
+      <c r="A116" s="8" t="n"/>
+      <c r="B116" s="8" t="n"/>
+      <c r="C116" s="8" t="n"/>
+      <c r="D116" s="8" t="n"/>
       <c r="E116" s="9" t="n"/>
       <c r="F116" s="11" t="inlineStr">
         <is>
-          <t>Publicación en producción de ambas apps en Google Play Store</t>
+          <t>Corrección de observaciones formuladas en la sustentación del 2do Sprint</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
@@ -3637,166 +3624,273 @@
       <c r="J116" s="9" t="n"/>
       <c r="K116" s="9" t="n"/>
     </row>
+    <row r="117" ht="45" customHeight="1" s="12">
+      <c r="A117" s="8" t="n"/>
+      <c r="B117" s="8" t="n"/>
+      <c r="C117" s="8" t="n"/>
+      <c r="D117" s="8" t="n"/>
+      <c r="E117" s="11" t="inlineStr">
+        <is>
+          <t>HU18 - Despliegue en Google Play Store (2 apps)
+Como equipo, queremos publicar ambas aplicaciones en Google Play Store, para que estén disponibles públicamente al finalizar el curso.</t>
+        </is>
+      </c>
+      <c r="F117" s="11" t="inlineStr">
+        <is>
+          <t>Generación del bundle firmado (AAB) de cada app</t>
+        </is>
+      </c>
+      <c r="G117" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H117" s="11" t="inlineStr">
+        <is>
+          <t>Play App Signing; Google Play Console; Firebase App Distribution</t>
+        </is>
+      </c>
+      <c r="I117" s="7" t="inlineStr">
+        <is>
+          <t>Semana 15</t>
+        </is>
+      </c>
+      <c r="J117" s="7" t="inlineStr">
+        <is>
+          <t>Semana 15</t>
+        </is>
+      </c>
+      <c r="K117" s="7" t="inlineStr">
+        <is>
+          <t>Rodrigo Puente</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="36" customHeight="1" s="12">
+      <c r="A118" s="8" t="n"/>
+      <c r="B118" s="8" t="n"/>
+      <c r="C118" s="8" t="n"/>
+      <c r="D118" s="8" t="n"/>
+      <c r="E118" s="8" t="n"/>
+      <c r="F118" s="11" t="inlineStr">
+        <is>
+          <t>Configuración de la ficha de cada app en Play Console</t>
+        </is>
+      </c>
+      <c r="G118" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H118" s="8" t="n"/>
+      <c r="I118" s="8" t="n"/>
+      <c r="J118" s="8" t="n"/>
+      <c r="K118" s="8" t="n"/>
+    </row>
+    <row r="119" ht="36" customHeight="1" s="12">
+      <c r="A119" s="8" t="n"/>
+      <c r="B119" s="8" t="n"/>
+      <c r="C119" s="8" t="n"/>
+      <c r="D119" s="8" t="n"/>
+      <c r="E119" s="8" t="n"/>
+      <c r="F119" s="11" t="inlineStr">
+        <is>
+          <t>Distribución beta previa con Firebase App Distribution</t>
+        </is>
+      </c>
+      <c r="G119" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H119" s="8" t="n"/>
+      <c r="I119" s="8" t="n"/>
+      <c r="J119" s="8" t="n"/>
+      <c r="K119" s="8" t="n"/>
+    </row>
+    <row r="120" ht="36" customHeight="1" s="12">
+      <c r="A120" s="9" t="n"/>
+      <c r="B120" s="9" t="n"/>
+      <c r="C120" s="9" t="n"/>
+      <c r="D120" s="9" t="n"/>
+      <c r="E120" s="9" t="n"/>
+      <c r="F120" s="11" t="inlineStr">
+        <is>
+          <t>Publicación en producción de ambas apps en Google Play Store</t>
+        </is>
+      </c>
+      <c r="G120" s="7" t="inlineStr">
+        <is>
+          <t>Sin Empezar</t>
+        </is>
+      </c>
+      <c r="H120" s="9" t="n"/>
+      <c r="I120" s="9" t="n"/>
+      <c r="J120" s="9" t="n"/>
+      <c r="K120" s="9" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="158">
-    <mergeCell ref="K80:K83"/>
-    <mergeCell ref="K96:K98"/>
-    <mergeCell ref="I48:I50"/>
-    <mergeCell ref="K48:K50"/>
+  <mergeCells count="160">
+    <mergeCell ref="B48:B85"/>
+    <mergeCell ref="H93:H96"/>
+    <mergeCell ref="K89:K92"/>
+    <mergeCell ref="J93:J96"/>
+    <mergeCell ref="H100:H102"/>
+    <mergeCell ref="E117:E120"/>
     <mergeCell ref="J25:J27"/>
     <mergeCell ref="H7:H11"/>
-    <mergeCell ref="D99:D104"/>
-    <mergeCell ref="J68:J71"/>
     <mergeCell ref="E7:E11"/>
+    <mergeCell ref="H54:H63"/>
+    <mergeCell ref="E97:E99"/>
+    <mergeCell ref="E106:E108"/>
+    <mergeCell ref="H86:H88"/>
     <mergeCell ref="J43:J47"/>
     <mergeCell ref="I38:I42"/>
     <mergeCell ref="E3:K3"/>
     <mergeCell ref="K38:K42"/>
-    <mergeCell ref="C48:C67"/>
-    <mergeCell ref="K105:K108"/>
+    <mergeCell ref="H117:H120"/>
     <mergeCell ref="H33:H37"/>
-    <mergeCell ref="D68:D76"/>
     <mergeCell ref="J33:J37"/>
-    <mergeCell ref="I90:I92"/>
-    <mergeCell ref="J72:J76"/>
+    <mergeCell ref="C72:C80"/>
+    <mergeCell ref="H81:H82"/>
+    <mergeCell ref="H103:H105"/>
+    <mergeCell ref="K54:K63"/>
+    <mergeCell ref="H97:H99"/>
+    <mergeCell ref="I93:I96"/>
+    <mergeCell ref="J97:J99"/>
     <mergeCell ref="K33:K37"/>
     <mergeCell ref="H28:H29"/>
     <mergeCell ref="E4:K4"/>
+    <mergeCell ref="D103:D108"/>
+    <mergeCell ref="E89:E92"/>
     <mergeCell ref="H19:H24"/>
+    <mergeCell ref="I48:I53"/>
+    <mergeCell ref="J109:J112"/>
     <mergeCell ref="E113:E116"/>
-    <mergeCell ref="J109:J112"/>
-    <mergeCell ref="I84:I85"/>
+    <mergeCell ref="C109:C120"/>
+    <mergeCell ref="I100:I102"/>
+    <mergeCell ref="K100:K102"/>
+    <mergeCell ref="I64:I71"/>
+    <mergeCell ref="J86:J88"/>
+    <mergeCell ref="I76:I80"/>
+    <mergeCell ref="H48:H53"/>
+    <mergeCell ref="K76:K80"/>
     <mergeCell ref="I109:I112"/>
-    <mergeCell ref="E99:E101"/>
-    <mergeCell ref="I60:I67"/>
     <mergeCell ref="I19:I24"/>
     <mergeCell ref="K19:K24"/>
-    <mergeCell ref="E68:E71"/>
-    <mergeCell ref="I102:I104"/>
-    <mergeCell ref="K102:K104"/>
-    <mergeCell ref="C80:C95"/>
     <mergeCell ref="E30:E32"/>
-    <mergeCell ref="K51:K59"/>
-    <mergeCell ref="D48:D67"/>
-    <mergeCell ref="E51:E59"/>
-    <mergeCell ref="E77:E79"/>
-    <mergeCell ref="I86:I89"/>
+    <mergeCell ref="J106:J108"/>
+    <mergeCell ref="K86:K88"/>
+    <mergeCell ref="E86:E88"/>
     <mergeCell ref="K12:K18"/>
-    <mergeCell ref="H99:H101"/>
-    <mergeCell ref="J90:J92"/>
-    <mergeCell ref="H68:H71"/>
+    <mergeCell ref="D72:D80"/>
+    <mergeCell ref="J48:J53"/>
     <mergeCell ref="K7:K11"/>
-    <mergeCell ref="C96:C98"/>
+    <mergeCell ref="K81:K82"/>
+    <mergeCell ref="C81:C85"/>
+    <mergeCell ref="C103:C108"/>
+    <mergeCell ref="J117:J120"/>
+    <mergeCell ref="K97:K99"/>
+    <mergeCell ref="J76:J80"/>
+    <mergeCell ref="D48:D71"/>
+    <mergeCell ref="I72:I75"/>
     <mergeCell ref="K109:K112"/>
+    <mergeCell ref="K72:K75"/>
+    <mergeCell ref="D109:D120"/>
     <mergeCell ref="C28:C32"/>
+    <mergeCell ref="J89:J92"/>
+    <mergeCell ref="H76:H80"/>
     <mergeCell ref="H109:H112"/>
-    <mergeCell ref="E80:E83"/>
-    <mergeCell ref="E96:E98"/>
-    <mergeCell ref="E60:E67"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="E72:E76"/>
+    <mergeCell ref="D89:D99"/>
+    <mergeCell ref="D100:D102"/>
     <mergeCell ref="J113:J116"/>
     <mergeCell ref="H25:H27"/>
-    <mergeCell ref="J51:J59"/>
-    <mergeCell ref="J77:J79"/>
-    <mergeCell ref="J99:J101"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="H80:H83"/>
-    <mergeCell ref="D80:D95"/>
+    <mergeCell ref="K48:K53"/>
+    <mergeCell ref="H72:H75"/>
+    <mergeCell ref="I106:I108"/>
     <mergeCell ref="K28:K29"/>
-    <mergeCell ref="C105:C116"/>
+    <mergeCell ref="K106:K108"/>
+    <mergeCell ref="D86:D88"/>
     <mergeCell ref="J30:J32"/>
+    <mergeCell ref="E81:E82"/>
     <mergeCell ref="I25:I27"/>
-    <mergeCell ref="I72:I76"/>
-    <mergeCell ref="K99:K101"/>
-    <mergeCell ref="I105:I108"/>
-    <mergeCell ref="E90:E92"/>
+    <mergeCell ref="E54:E63"/>
     <mergeCell ref="C7:C27"/>
-    <mergeCell ref="K68:K71"/>
-    <mergeCell ref="I93:I95"/>
-    <mergeCell ref="H72:H76"/>
+    <mergeCell ref="K93:K96"/>
+    <mergeCell ref="J72:J75"/>
+    <mergeCell ref="E93:E96"/>
     <mergeCell ref="I43:I47"/>
     <mergeCell ref="K43:K47"/>
-    <mergeCell ref="K77:K79"/>
-    <mergeCell ref="H96:H98"/>
+    <mergeCell ref="I83:I85"/>
+    <mergeCell ref="B86:B120"/>
     <mergeCell ref="I113:I116"/>
     <mergeCell ref="J7:J11"/>
-    <mergeCell ref="H90:H92"/>
     <mergeCell ref="I33:I37"/>
-    <mergeCell ref="H77:H79"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="E84:E85"/>
-    <mergeCell ref="B48:B104"/>
-    <mergeCell ref="J80:J83"/>
-    <mergeCell ref="J96:J98"/>
-    <mergeCell ref="J60:J67"/>
-    <mergeCell ref="J48:J50"/>
+    <mergeCell ref="E100:E102"/>
+    <mergeCell ref="E76:E80"/>
     <mergeCell ref="E28:E29"/>
+    <mergeCell ref="K103:K105"/>
     <mergeCell ref="K25:K27"/>
+    <mergeCell ref="C86:C88"/>
     <mergeCell ref="E19:E24"/>
-    <mergeCell ref="E102:E104"/>
-    <mergeCell ref="H84:H85"/>
-    <mergeCell ref="I51:I59"/>
-    <mergeCell ref="K60:K67"/>
+    <mergeCell ref="H64:H71"/>
     <mergeCell ref="E12:E18"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="C99:C104"/>
+    <mergeCell ref="I86:I88"/>
+    <mergeCell ref="I117:I120"/>
     <mergeCell ref="H43:H47"/>
-    <mergeCell ref="H60:H67"/>
-    <mergeCell ref="C68:C76"/>
-    <mergeCell ref="H102:H104"/>
-    <mergeCell ref="J102:J104"/>
+    <mergeCell ref="K117:K120"/>
+    <mergeCell ref="D81:D85"/>
+    <mergeCell ref="J54:J63"/>
     <mergeCell ref="I7:I11"/>
-    <mergeCell ref="D77:D79"/>
+    <mergeCell ref="I81:I82"/>
+    <mergeCell ref="I97:I99"/>
+    <mergeCell ref="J83:J85"/>
     <mergeCell ref="E109:E112"/>
     <mergeCell ref="E38:E42"/>
-    <mergeCell ref="I96:I98"/>
-    <mergeCell ref="K90:K92"/>
+    <mergeCell ref="C89:C99"/>
     <mergeCell ref="E2:K2"/>
+    <mergeCell ref="J81:J82"/>
+    <mergeCell ref="J103:J105"/>
     <mergeCell ref="B7:B47"/>
-    <mergeCell ref="J84:J85"/>
     <mergeCell ref="H113:H116"/>
+    <mergeCell ref="J100:J102"/>
     <mergeCell ref="C33:C47"/>
-    <mergeCell ref="H51:H59"/>
-    <mergeCell ref="A7:A116"/>
+    <mergeCell ref="J64:J71"/>
     <mergeCell ref="J28:J29"/>
+    <mergeCell ref="I89:I92"/>
     <mergeCell ref="D28:D32"/>
     <mergeCell ref="J19:J24"/>
-    <mergeCell ref="C77:C79"/>
+    <mergeCell ref="A7:A120"/>
     <mergeCell ref="I28:I29"/>
-    <mergeCell ref="K84:K85"/>
+    <mergeCell ref="H89:H92"/>
+    <mergeCell ref="E48:E53"/>
     <mergeCell ref="K113:K116"/>
-    <mergeCell ref="H48:H50"/>
+    <mergeCell ref="I54:I63"/>
     <mergeCell ref="E25:E27"/>
     <mergeCell ref="H30:H32"/>
+    <mergeCell ref="K64:K71"/>
     <mergeCell ref="H12:H18"/>
+    <mergeCell ref="E64:E71"/>
     <mergeCell ref="J12:J18"/>
-    <mergeCell ref="J86:J89"/>
-    <mergeCell ref="E105:E108"/>
-    <mergeCell ref="I99:I101"/>
-    <mergeCell ref="K93:K95"/>
-    <mergeCell ref="I68:I71"/>
-    <mergeCell ref="E93:E95"/>
-    <mergeCell ref="B105:B116"/>
+    <mergeCell ref="H106:H108"/>
+    <mergeCell ref="K83:K85"/>
     <mergeCell ref="E43:E47"/>
     <mergeCell ref="I30:I32"/>
-    <mergeCell ref="D105:D116"/>
+    <mergeCell ref="E83:E85"/>
     <mergeCell ref="K30:K32"/>
-    <mergeCell ref="K86:K89"/>
-    <mergeCell ref="I77:I79"/>
-    <mergeCell ref="D96:D98"/>
-    <mergeCell ref="H105:H108"/>
+    <mergeCell ref="C48:C71"/>
+    <mergeCell ref="E33:E37"/>
     <mergeCell ref="H38:H42"/>
-    <mergeCell ref="E33:E37"/>
     <mergeCell ref="J38:J42"/>
     <mergeCell ref="D7:D27"/>
     <mergeCell ref="D33:D47"/>
-    <mergeCell ref="H93:H95"/>
-    <mergeCell ref="J93:J95"/>
-    <mergeCell ref="K72:K76"/>
+    <mergeCell ref="C100:C102"/>
+    <mergeCell ref="H83:H85"/>
+    <mergeCell ref="E103:E105"/>
+    <mergeCell ref="I103:I105"/>
+    <mergeCell ref="E72:E75"/>
     <mergeCell ref="I12:I18"/>
-    <mergeCell ref="J105:J108"/>
-    <mergeCell ref="I80:I83"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[SCRUM-100] feat: cambia el estado del pedido desde la bandeja (listo, en camino, entregado)
</commit_message>
<xml_diff>
--- a/docs/SanMarkFood-Planificacion.xlsx
+++ b/docs/SanMarkFood-Planificacion.xlsx
@@ -2718,7 +2718,7 @@
     </row>
     <row r="85" ht="36" customHeight="1" s="12">
       <c r="A85" s="8" t="n"/>
-      <c r="B85" s="9" t="n"/>
+      <c r="B85" s="8" t="n"/>
       <c r="C85" s="8" t="n"/>
       <c r="D85" s="8" t="n"/>
       <c r="E85" s="9" t="n"/>
@@ -2739,29 +2739,27 @@
     </row>
     <row r="86" ht="45" customHeight="1" s="12">
       <c r="A86" s="8" t="n"/>
-      <c r="B86" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C86" s="10" t="inlineStr">
-        <is>
-          <t>Actividad del Comensal:
-Historial de pedidos y reservas pasadas, para consulta y repetición rápida.</t>
-        </is>
-      </c>
-      <c r="D86" s="10" t="inlineStr">
-        <is>
-          <t>Comensal</t>
+      <c r="B86" s="8" t="n"/>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard de Restaurante y de Plataforma:
+Panel de indicadores del negocio para el restaurante, y panel agregado de la plataforma para el administrador.</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>Restaurante / Administrador</t>
         </is>
       </c>
       <c r="E86" s="14" t="inlineStr">
         <is>
-          <t>HU20 - Historial de pedidos y reservas
-Como comensal, quiero ver el historial de mis pedidos y reservas pasadas, para llevar un registro de mi actividad y repetir un pedido anterior fácilmente.</t>
+          <t>HU26 - Dashboard global (Administrador)
+Como administrador, quiero ver métricas agregadas de toda la plataforma (restaurantes activos, pedidos totales), para monitorear la salud del negocio.</t>
         </is>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
-          <t>Listado de pedidos y reservas pasadas, ordenado por fecha</t>
+          <t>Métricas agregadas de todos los restaurantes: restaurantes activos y pedidos totales</t>
         </is>
       </c>
       <c r="G86" s="10" t="inlineStr">
@@ -2771,22 +2769,22 @@
       </c>
       <c r="H86" s="14" t="inlineStr">
         <is>
-          <t>Firestore (historial); Retrofit + corrutinas (backend propio); Jetpack Compose</t>
+          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de locales y pedidos); Cloud Functions</t>
         </is>
       </c>
       <c r="I86" s="10" t="inlineStr">
         <is>
-          <t>Semana 13</t>
+          <t>Semana 12</t>
         </is>
       </c>
       <c r="J86" s="10" t="inlineStr">
         <is>
-          <t>Semana 14</t>
+          <t>Semana 12</t>
         </is>
       </c>
       <c r="K86" s="10" t="inlineStr">
         <is>
-          <t>Camila Bada</t>
+          <t>Rodrigo Puente</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2796,7 @@
       <c r="E87" s="8" t="n"/>
       <c r="F87" s="14" t="inlineStr">
         <is>
-          <t>Detalle de cada pedido o reserva pasado (restaurante, ítems, estado final)</t>
+          <t>El dashboard obtiene las métricas con consultas de agregación de Firestore (count, sum), sin backend propio; lo que no se pueda agregar así lo calcula una Cloud Function</t>
         </is>
       </c>
       <c r="G87" s="10" t="inlineStr">
@@ -2813,13 +2811,13 @@
     </row>
     <row r="88" ht="36" customHeight="1" s="12">
       <c r="A88" s="8" t="n"/>
-      <c r="B88" s="8" t="n"/>
+      <c r="B88" s="9" t="n"/>
       <c r="C88" s="9" t="n"/>
       <c r="D88" s="9" t="n"/>
       <c r="E88" s="9" t="n"/>
       <c r="F88" s="14" t="inlineStr">
         <is>
-          <t>Opción de “repetir pedido” que precarga el carrito con los mismos ítems; si incluía menú del día, se eligen entrada y segundo del menú de hoy</t>
+          <t>Gráfico de evolución de pedidos totales por semana</t>
         </is>
       </c>
       <c r="G88" s="10" t="inlineStr">
@@ -2834,27 +2832,29 @@
     </row>
     <row r="89" ht="45" customHeight="1" s="12">
       <c r="A89" s="8" t="n"/>
-      <c r="B89" s="8" t="n"/>
+      <c r="B89" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>Chatbot y Reseñas con IA:
-Atención conversacional para el comensal, y el sistema completo de reseñas: resumen y alerta con IA, visualización de detalle, y respuesta del restaurante.</t>
+          <t>Actividad del Comensal:
+Historial de pedidos y reservas pasadas, para consulta y repetición rápida.</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>Comensal / Restaurante / Backend</t>
+          <t>Comensal</t>
         </is>
       </c>
       <c r="E89" s="14" t="inlineStr">
         <is>
-          <t>HU11 - Chatbot de atención con entrada por voz
-Como comensal, quiero consultar a un chatbot (por texto o por voz) sobre horarios, disponibilidad o el estado de mi reserva/pedido, para resolver dudas rápidas sin llamar al restaurante.</t>
+          <t>HU20 - Historial de pedidos y reservas
+Como comensal, quiero ver el historial de mis pedidos y reservas pasadas, para llevar un registro de mi actividad y repetir un pedido anterior fácilmente.</t>
         </is>
       </c>
       <c r="F89" s="14" t="inlineStr">
         <is>
-          <t>Chat conversacional accesible desde la pantalla de un restaurante</t>
+          <t>Listado de pedidos y reservas pasadas, ordenado por fecha</t>
         </is>
       </c>
       <c r="G89" s="10" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="H89" s="14" t="inlineStr">
         <is>
-          <t>SpeechRecognizer (entrada de voz); Gemini vía Firebase AI Logic, con los datos del local y del pedido o reserva leídos de Firestore; Jetpack Compose</t>
+          <t>Firestore (historial); Retrofit + corrutinas (backend propio); Jetpack Compose</t>
         </is>
       </c>
       <c r="I89" s="10" t="inlineStr">
@@ -2891,7 +2891,7 @@
       <c r="E90" s="8" t="n"/>
       <c r="F90" s="14" t="inlineStr">
         <is>
-          <t>Entrada por voz mediante reconocimiento de habla, como alternativa al texto</t>
+          <t>Detalle de cada pedido o reserva pasado (restaurante, ítems, estado final)</t>
         </is>
       </c>
       <c r="G90" s="10" t="inlineStr">
@@ -2907,12 +2907,12 @@
     <row r="91" ht="36" customHeight="1" s="12">
       <c r="A91" s="8" t="n"/>
       <c r="B91" s="8" t="n"/>
-      <c r="C91" s="8" t="n"/>
-      <c r="D91" s="8" t="n"/>
-      <c r="E91" s="8" t="n"/>
+      <c r="C91" s="9" t="n"/>
+      <c r="D91" s="9" t="n"/>
+      <c r="E91" s="9" t="n"/>
       <c r="F91" s="14" t="inlineStr">
         <is>
-          <t>Respuestas sobre horarios, menú y disponibilidad de ese restaurante</t>
+          <t>Opción de “repetir pedido” que precarga el carrito con los mismos ítems; si incluía menú del día, se eligen entrada y segundo del menú de hoy</t>
         </is>
       </c>
       <c r="G91" s="10" t="inlineStr">
@@ -2920,20 +2920,34 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H91" s="8" t="n"/>
-      <c r="I91" s="8" t="n"/>
-      <c r="J91" s="8" t="n"/>
-      <c r="K91" s="8" t="n"/>
-    </row>
-    <row r="92" ht="36" customHeight="1" s="12">
+      <c r="H91" s="9" t="n"/>
+      <c r="I91" s="9" t="n"/>
+      <c r="J91" s="9" t="n"/>
+      <c r="K91" s="9" t="n"/>
+    </row>
+    <row r="92" ht="45" customHeight="1" s="12">
       <c r="A92" s="8" t="n"/>
       <c r="B92" s="8" t="n"/>
-      <c r="C92" s="8" t="n"/>
-      <c r="D92" s="8" t="n"/>
-      <c r="E92" s="9" t="n"/>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>Chatbot y Reseñas con IA:
+Atención conversacional para el comensal, y el sistema completo de reseñas: resumen y alerta con IA, visualización de detalle, y respuesta del restaurante.</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="inlineStr">
+        <is>
+          <t>Comensal / Restaurante / Backend</t>
+        </is>
+      </c>
+      <c r="E92" s="14" t="inlineStr">
+        <is>
+          <t>HU11 - Chatbot de atención con entrada por voz
+Como comensal, quiero consultar a un chatbot (por texto o por voz) sobre horarios, disponibilidad o el estado de mi reserva/pedido, para resolver dudas rápidas sin llamar al restaurante.</t>
+        </is>
+      </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
-          <t>Consulta del estado de una reserva o pedido activo mediante el chat</t>
+          <t>Chat conversacional accesible desde la pantalla de un restaurante</t>
         </is>
       </c>
       <c r="G92" s="10" t="inlineStr">
@@ -2941,25 +2955,36 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H92" s="9" t="n"/>
-      <c r="I92" s="9" t="n"/>
-      <c r="J92" s="9" t="n"/>
-      <c r="K92" s="9" t="n"/>
-    </row>
-    <row r="93" ht="45" customHeight="1" s="12">
+      <c r="H92" s="14" t="inlineStr">
+        <is>
+          <t>SpeechRecognizer (entrada de voz); Gemini vía Firebase AI Logic, con los datos del local y del pedido o reserva leídos de Firestore; Jetpack Compose</t>
+        </is>
+      </c>
+      <c r="I92" s="10" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="J92" s="10" t="inlineStr">
+        <is>
+          <t>Semana 14</t>
+        </is>
+      </c>
+      <c r="K92" s="10" t="inlineStr">
+        <is>
+          <t>Camila Bada</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="36" customHeight="1" s="12">
       <c r="A93" s="8" t="n"/>
       <c r="B93" s="8" t="n"/>
       <c r="C93" s="8" t="n"/>
       <c r="D93" s="8" t="n"/>
-      <c r="E93" s="14" t="inlineStr">
-        <is>
-          <t>HU22 - Ver detalle de reseñas de un restaurante (Comensal)
-Como comensal, quiero ver el listado completo de reseñas de un restaurante (autor, calificación, comentario, fecha), para revisar el detalle si el resumen de IA no me es suficiente.</t>
-        </is>
-      </c>
+      <c r="E93" s="8" t="n"/>
       <c r="F93" s="14" t="inlineStr">
         <is>
-          <t>Listado de reseñas ordenado por fecha, con calificación y comentario</t>
+          <t>Entrada por voz mediante reconocimiento de habla, como alternativa al texto</t>
         </is>
       </c>
       <c r="G93" s="10" t="inlineStr">
@@ -2967,26 +2992,10 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H93" s="14" t="inlineStr">
-        <is>
-          <t>Firestore (colección de reseñas); Jetpack Compose</t>
-        </is>
-      </c>
-      <c r="I93" s="10" t="inlineStr">
-        <is>
-          <t>Semana 13</t>
-        </is>
-      </c>
-      <c r="J93" s="10" t="inlineStr">
-        <is>
-          <t>Semana 13</t>
-        </is>
-      </c>
-      <c r="K93" s="10" t="inlineStr">
-        <is>
-          <t>Camila Bada</t>
-        </is>
-      </c>
+      <c r="H93" s="8" t="n"/>
+      <c r="I93" s="8" t="n"/>
+      <c r="J93" s="8" t="n"/>
+      <c r="K93" s="8" t="n"/>
     </row>
     <row r="94" ht="36" customHeight="1" s="12">
       <c r="A94" s="8" t="n"/>
@@ -2996,7 +3005,7 @@
       <c r="E94" s="8" t="n"/>
       <c r="F94" s="14" t="inlineStr">
         <is>
-          <t>Filtro por calificación (1 a 5 estrellas)</t>
+          <t>Respuestas sobre horarios, menú y disponibilidad de ese restaurante</t>
         </is>
       </c>
       <c r="G94" s="10" t="inlineStr">
@@ -3014,10 +3023,10 @@
       <c r="B95" s="8" t="n"/>
       <c r="C95" s="8" t="n"/>
       <c r="D95" s="8" t="n"/>
-      <c r="E95" s="8" t="n"/>
+      <c r="E95" s="9" t="n"/>
       <c r="F95" s="14" t="inlineStr">
         <is>
-          <t>Se muestra la respuesta del restaurante debajo de la reseña, si existe</t>
+          <t>Consulta del estado de una reserva o pedido activo mediante el chat</t>
         </is>
       </c>
       <c r="G95" s="10" t="inlineStr">
@@ -3025,20 +3034,25 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H95" s="8" t="n"/>
-      <c r="I95" s="8" t="n"/>
-      <c r="J95" s="8" t="n"/>
-      <c r="K95" s="8" t="n"/>
-    </row>
-    <row r="96" ht="36" customHeight="1" s="12">
+      <c r="H95" s="9" t="n"/>
+      <c r="I95" s="9" t="n"/>
+      <c r="J95" s="9" t="n"/>
+      <c r="K95" s="9" t="n"/>
+    </row>
+    <row r="96" ht="45" customHeight="1" s="12">
       <c r="A96" s="8" t="n"/>
       <c r="B96" s="8" t="n"/>
       <c r="C96" s="8" t="n"/>
       <c r="D96" s="8" t="n"/>
-      <c r="E96" s="9" t="n"/>
+      <c r="E96" s="14" t="inlineStr">
+        <is>
+          <t>HU22 - Ver detalle de reseñas de un restaurante (Comensal)
+Como comensal, quiero ver el listado completo de reseñas de un restaurante (autor, calificación, comentario, fecha), para revisar el detalle si el resumen de IA no me es suficiente.</t>
+        </is>
+      </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>Reportar una reseña ajena con motivo (ofensiva, falsa, spam u otro); cada comensal puede reportarla una sola vez y la reseña pasa a la cola de moderación de HU25</t>
+          <t>Listado de reseñas ordenado por fecha, con calificación y comentario</t>
         </is>
       </c>
       <c r="G96" s="10" t="inlineStr">
@@ -3046,25 +3060,36 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H96" s="9" t="n"/>
-      <c r="I96" s="9" t="n"/>
-      <c r="J96" s="9" t="n"/>
-      <c r="K96" s="9" t="n"/>
-    </row>
-    <row r="97" ht="45" customHeight="1" s="12">
+      <c r="H96" s="14" t="inlineStr">
+        <is>
+          <t>Firestore (colección de reseñas); Jetpack Compose</t>
+        </is>
+      </c>
+      <c r="I96" s="10" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="J96" s="10" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="K96" s="10" t="inlineStr">
+        <is>
+          <t>Camila Bada</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="36" customHeight="1" s="12">
       <c r="A97" s="8" t="n"/>
       <c r="B97" s="8" t="n"/>
       <c r="C97" s="8" t="n"/>
       <c r="D97" s="8" t="n"/>
-      <c r="E97" s="14" t="inlineStr">
-        <is>
-          <t>HU21 - Gestión y respuesta a reseñas (Restaurante)
-Como restaurante, quiero ver todas mis reseñas recibidas y responder a cualquiera de ellas, para mostrar que atiendo la retroalimentación de mis comensales, no solo las negativas.</t>
-        </is>
-      </c>
+      <c r="E97" s="8" t="n"/>
       <c r="F97" s="14" t="inlineStr">
         <is>
-          <t>Listado completo de reseñas recibidas, no solo las negativas</t>
+          <t>Filtro por calificación (1 a 5 estrellas)</t>
         </is>
       </c>
       <c r="G97" s="10" t="inlineStr">
@@ -3072,26 +3097,10 @@
           <t>Sin Empezar</t>
         </is>
       </c>
-      <c r="H97" s="14" t="inlineStr">
-        <is>
-          <t>Firestore (subcolección de respuestas); Firebase Cloud Messaging</t>
-        </is>
-      </c>
-      <c r="I97" s="10" t="inlineStr">
-        <is>
-          <t>Semana 13</t>
-        </is>
-      </c>
-      <c r="J97" s="10" t="inlineStr">
-        <is>
-          <t>Semana 13</t>
-        </is>
-      </c>
-      <c r="K97" s="10" t="inlineStr">
-        <is>
-          <t>Jose Chuque</t>
-        </is>
-      </c>
+      <c r="H97" s="8" t="n"/>
+      <c r="I97" s="8" t="n"/>
+      <c r="J97" s="8" t="n"/>
+      <c r="K97" s="8" t="n"/>
     </row>
     <row r="98" ht="36" customHeight="1" s="12">
       <c r="A98" s="8" t="n"/>
@@ -3101,7 +3110,7 @@
       <c r="E98" s="8" t="n"/>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>Responder públicamente a cualquier reseña</t>
+          <t>Se muestra la respuesta del restaurante debajo de la reseña, si existe</t>
         </is>
       </c>
       <c r="G98" s="10" t="inlineStr">
@@ -3117,12 +3126,12 @@
     <row r="99" ht="36" customHeight="1" s="12">
       <c r="A99" s="8" t="n"/>
       <c r="B99" s="8" t="n"/>
-      <c r="C99" s="9" t="n"/>
-      <c r="D99" s="9" t="n"/>
+      <c r="C99" s="8" t="n"/>
+      <c r="D99" s="8" t="n"/>
       <c r="E99" s="9" t="n"/>
       <c r="F99" s="14" t="inlineStr">
         <is>
-          <t>Notificación al comensal cuando su reseña recibe respuesta</t>
+          <t>Reportar una reseña ajena con motivo (ofensiva, falsa, spam u otro); cada comensal puede reportarla una sola vez y la reseña pasa a la cola de moderación de HU25</t>
         </is>
       </c>
       <c r="G99" s="10" t="inlineStr">
@@ -3138,26 +3147,17 @@
     <row r="100" ht="45" customHeight="1" s="12">
       <c r="A100" s="8" t="n"/>
       <c r="B100" s="8" t="n"/>
-      <c r="C100" s="10" t="inlineStr">
-        <is>
-          <t>Moderación de la Plataforma (Administrador):
-Revisión y moderación de las reseñas del sistema.</t>
-        </is>
-      </c>
-      <c r="D100" s="10" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
+      <c r="C100" s="8" t="n"/>
+      <c r="D100" s="8" t="n"/>
       <c r="E100" s="14" t="inlineStr">
         <is>
-          <t>HU25 - Moderación de reseñas
-Como administrador, quiero revisar y eliminar una reseña reportada como abusiva o falsa, para mantener la confianza del sistema de reseñas.</t>
+          <t>HU21 - Gestión y respuesta a reseñas (Restaurante)
+Como restaurante, quiero ver todas mis reseñas recibidas y responder a cualquiera de ellas, para mostrar que atiendo la retroalimentación de mis comensales, no solo las negativas.</t>
         </is>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>Listado de reseñas reportadas o marcadas para revisión</t>
+          <t>Listado completo de reseñas recibidas, no solo las negativas</t>
         </is>
       </c>
       <c r="G100" s="10" t="inlineStr">
@@ -3167,17 +3167,17 @@
       </c>
       <c r="H100" s="14" t="inlineStr">
         <is>
-          <t>Firestore (listener de reseñas reportadas); Cloud Functions for Firebase</t>
+          <t>Firestore (subcolección de respuestas); Firebase Cloud Messaging</t>
         </is>
       </c>
       <c r="I100" s="10" t="inlineStr">
         <is>
-          <t>Semana 11</t>
+          <t>Semana 13</t>
         </is>
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>Semana 12</t>
+          <t>Semana 13</t>
         </is>
       </c>
       <c r="K100" s="10" t="inlineStr">
@@ -3194,7 +3194,7 @@
       <c r="E101" s="8" t="n"/>
       <c r="F101" s="14" t="inlineStr">
         <is>
-          <t>Eliminar una reseña clasificada como abusiva o falsa</t>
+          <t>Responder públicamente a cualquier reseña</t>
         </is>
       </c>
       <c r="G101" s="10" t="inlineStr">
@@ -3215,7 +3215,7 @@
       <c r="E102" s="9" t="n"/>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>Registro de la acción de moderación realizada</t>
+          <t>Notificación al comensal cuando su reseña recibe respuesta</t>
         </is>
       </c>
       <c r="G102" s="10" t="inlineStr">
@@ -3233,24 +3233,24 @@
       <c r="B103" s="8" t="n"/>
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>Dashboard de Restaurante y de Plataforma:
-Panel de indicadores del negocio para el restaurante, y panel agregado de la plataforma para el administrador.</t>
+          <t>Moderación de la Plataforma (Administrador):
+Revisión y moderación de las reseñas del sistema.</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>Restaurante / Administrador</t>
+          <t>Administrador</t>
         </is>
       </c>
       <c r="E103" s="14" t="inlineStr">
         <is>
-          <t>HU13 - Dashboard de restaurante
-Como restaurante, quiero ver un dashboard con mis ventas, platos más pedidos y calificación promedio, para entender cómo va mi negocio en la app.</t>
+          <t>HU25 - Moderación de reseñas
+Como administrador, quiero revisar y eliminar una reseña reportada como abusiva o falsa, para mantener la confianza del sistema de reseñas.</t>
         </is>
       </c>
       <c r="F103" s="14" t="inlineStr">
         <is>
-          <t>Gráfico de ventas/pedidos por día o semana</t>
+          <t>Listado de reseñas reportadas o marcadas para revisión</t>
         </is>
       </c>
       <c r="G103" s="10" t="inlineStr">
@@ -3260,12 +3260,12 @@
       </c>
       <c r="H103" s="14" t="inlineStr">
         <is>
-          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de pedidos y calificaciones)</t>
+          <t>Firestore (listener de reseñas reportadas); Cloud Functions for Firebase</t>
         </is>
       </c>
       <c r="I103" s="10" t="inlineStr">
         <is>
-          <t>Semana 12</t>
+          <t>Semana 11</t>
         </is>
       </c>
       <c r="J103" s="10" t="inlineStr">
@@ -3287,7 +3287,7 @@
       <c r="E104" s="8" t="n"/>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>Ranking de platos más pedidos</t>
+          <t>Eliminar una reseña clasificada como abusiva o falsa</t>
         </is>
       </c>
       <c r="G104" s="10" t="inlineStr">
@@ -3303,12 +3303,12 @@
     <row r="105" ht="36" customHeight="1" s="12">
       <c r="A105" s="8" t="n"/>
       <c r="B105" s="8" t="n"/>
-      <c r="C105" s="8" t="n"/>
-      <c r="D105" s="8" t="n"/>
+      <c r="C105" s="9" t="n"/>
+      <c r="D105" s="9" t="n"/>
       <c r="E105" s="9" t="n"/>
       <c r="F105" s="14" t="inlineStr">
         <is>
-          <t>Calificación promedio y su evolución en el tiempo</t>
+          <t>Registro de la acción de moderación realizada</t>
         </is>
       </c>
       <c r="G105" s="10" t="inlineStr">
@@ -3324,17 +3324,26 @@
     <row r="106" ht="45" customHeight="1" s="12">
       <c r="A106" s="8" t="n"/>
       <c r="B106" s="8" t="n"/>
-      <c r="C106" s="8" t="n"/>
-      <c r="D106" s="8" t="n"/>
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard de Restaurante y de Plataforma:
+Panel de indicadores del negocio para el restaurante, y panel agregado de la plataforma para el administrador.</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="inlineStr">
+        <is>
+          <t>Restaurante / Administrador</t>
+        </is>
+      </c>
       <c r="E106" s="14" t="inlineStr">
         <is>
-          <t>HU26 - Dashboard global (Administrador)
-Como administrador, quiero ver métricas agregadas de toda la plataforma (restaurantes activos, pedidos totales), para monitorear la salud del negocio.</t>
+          <t>HU13 - Dashboard de restaurante
+Como restaurante, quiero ver un dashboard con mis ventas, platos más pedidos y calificación promedio, para entender cómo va mi negocio en la app.</t>
         </is>
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
-          <t>Métricas agregadas de todos los restaurantes: restaurantes activos y pedidos totales</t>
+          <t>Gráfico de ventas/pedidos por día o semana</t>
         </is>
       </c>
       <c r="G106" s="10" t="inlineStr">
@@ -3344,22 +3353,22 @@
       </c>
       <c r="H106" s="14" t="inlineStr">
         <is>
-          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de locales y pedidos); Cloud Functions</t>
+          <t>MPAndroidChart o Vico (gráficos); Firestore (agregación de pedidos y calificaciones)</t>
         </is>
       </c>
       <c r="I106" s="10" t="inlineStr">
         <is>
-          <t>Semana 13</t>
+          <t>Semana 12</t>
         </is>
       </c>
       <c r="J106" s="10" t="inlineStr">
         <is>
-          <t>Semana 14</t>
+          <t>Semana 12</t>
         </is>
       </c>
       <c r="K106" s="10" t="inlineStr">
         <is>
-          <t>Rodrigo Puente</t>
+          <t>Jose Chuque</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3380,7 @@
       <c r="E107" s="8" t="n"/>
       <c r="F107" s="14" t="inlineStr">
         <is>
-          <t>El dashboard obtiene las métricas con consultas de agregación de Firestore (count, sum), sin backend propio; lo que no se pueda agregar así lo calcula una Cloud Function</t>
+          <t>Ranking de platos más pedidos</t>
         </is>
       </c>
       <c r="G107" s="10" t="inlineStr">
@@ -3392,7 +3401,7 @@
       <c r="E108" s="9" t="n"/>
       <c r="F108" s="14" t="inlineStr">
         <is>
-          <t>Gráfico de evolución de pedidos totales por semana</t>
+          <t>Calificación promedio y su evolución en el tiempo</t>
         </is>
       </c>
       <c r="G108" s="10" t="inlineStr">
@@ -3730,18 +3739,13 @@
       <c r="K120" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="160">
-    <mergeCell ref="B48:B85"/>
-    <mergeCell ref="H93:H96"/>
-    <mergeCell ref="K89:K92"/>
-    <mergeCell ref="J93:J96"/>
+  <mergeCells count="162">
     <mergeCell ref="H100:H102"/>
     <mergeCell ref="E117:E120"/>
     <mergeCell ref="J25:J27"/>
     <mergeCell ref="H7:H11"/>
     <mergeCell ref="E7:E11"/>
     <mergeCell ref="H54:H63"/>
-    <mergeCell ref="E97:E99"/>
     <mergeCell ref="E106:E108"/>
     <mergeCell ref="H86:H88"/>
     <mergeCell ref="J43:J47"/>
@@ -3752,23 +3756,23 @@
     <mergeCell ref="H33:H37"/>
     <mergeCell ref="J33:J37"/>
     <mergeCell ref="C72:C80"/>
+    <mergeCell ref="H103:H105"/>
+    <mergeCell ref="C89:C91"/>
     <mergeCell ref="H81:H82"/>
-    <mergeCell ref="H103:H105"/>
     <mergeCell ref="K54:K63"/>
-    <mergeCell ref="H97:H99"/>
-    <mergeCell ref="I93:I96"/>
-    <mergeCell ref="J97:J99"/>
+    <mergeCell ref="B48:B88"/>
     <mergeCell ref="K33:K37"/>
     <mergeCell ref="H28:H29"/>
     <mergeCell ref="E4:K4"/>
-    <mergeCell ref="D103:D108"/>
-    <mergeCell ref="E89:E92"/>
+    <mergeCell ref="H96:H99"/>
     <mergeCell ref="H19:H24"/>
     <mergeCell ref="I48:I53"/>
+    <mergeCell ref="H89:H91"/>
+    <mergeCell ref="E113:E116"/>
     <mergeCell ref="J109:J112"/>
-    <mergeCell ref="E113:E116"/>
     <mergeCell ref="C109:C120"/>
     <mergeCell ref="I100:I102"/>
+    <mergeCell ref="J96:J99"/>
     <mergeCell ref="K100:K102"/>
     <mergeCell ref="I64:I71"/>
     <mergeCell ref="J86:J88"/>
@@ -3776,33 +3780,37 @@
     <mergeCell ref="H48:H53"/>
     <mergeCell ref="K76:K80"/>
     <mergeCell ref="I109:I112"/>
+    <mergeCell ref="J89:J91"/>
     <mergeCell ref="I19:I24"/>
     <mergeCell ref="K19:K24"/>
+    <mergeCell ref="H92:H95"/>
+    <mergeCell ref="B89:B120"/>
     <mergeCell ref="E30:E32"/>
+    <mergeCell ref="E92:E95"/>
     <mergeCell ref="J106:J108"/>
     <mergeCell ref="K86:K88"/>
     <mergeCell ref="E86:E88"/>
     <mergeCell ref="K12:K18"/>
     <mergeCell ref="D72:D80"/>
-    <mergeCell ref="J48:J53"/>
     <mergeCell ref="K7:K11"/>
+    <mergeCell ref="J117:J120"/>
     <mergeCell ref="K81:K82"/>
     <mergeCell ref="C81:C85"/>
-    <mergeCell ref="C103:C108"/>
-    <mergeCell ref="J117:J120"/>
-    <mergeCell ref="K97:K99"/>
+    <mergeCell ref="C106:C108"/>
+    <mergeCell ref="J48:J53"/>
     <mergeCell ref="J76:J80"/>
     <mergeCell ref="D48:D71"/>
     <mergeCell ref="I72:I75"/>
     <mergeCell ref="K109:K112"/>
     <mergeCell ref="K72:K75"/>
     <mergeCell ref="D109:D120"/>
+    <mergeCell ref="I96:I99"/>
     <mergeCell ref="C28:C32"/>
-    <mergeCell ref="J89:J92"/>
+    <mergeCell ref="K96:K99"/>
     <mergeCell ref="H76:H80"/>
     <mergeCell ref="H109:H112"/>
-    <mergeCell ref="D89:D99"/>
-    <mergeCell ref="D100:D102"/>
+    <mergeCell ref="I89:I91"/>
+    <mergeCell ref="K89:K91"/>
     <mergeCell ref="J113:J116"/>
     <mergeCell ref="H25:H27"/>
     <mergeCell ref="K48:K53"/>
@@ -3812,21 +3820,24 @@
     <mergeCell ref="K106:K108"/>
     <mergeCell ref="D86:D88"/>
     <mergeCell ref="J30:J32"/>
+    <mergeCell ref="C92:C102"/>
+    <mergeCell ref="I25:I27"/>
     <mergeCell ref="E81:E82"/>
-    <mergeCell ref="I25:I27"/>
+    <mergeCell ref="J92:J95"/>
+    <mergeCell ref="C7:C27"/>
+    <mergeCell ref="D103:D105"/>
     <mergeCell ref="E54:E63"/>
-    <mergeCell ref="C7:C27"/>
-    <mergeCell ref="K93:K96"/>
     <mergeCell ref="J72:J75"/>
-    <mergeCell ref="E93:E96"/>
+    <mergeCell ref="D106:D108"/>
     <mergeCell ref="I43:I47"/>
     <mergeCell ref="K43:K47"/>
+    <mergeCell ref="K92:K95"/>
     <mergeCell ref="I83:I85"/>
-    <mergeCell ref="B86:B120"/>
     <mergeCell ref="I113:I116"/>
     <mergeCell ref="J7:J11"/>
     <mergeCell ref="I33:I37"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D89:D91"/>
     <mergeCell ref="E100:E102"/>
     <mergeCell ref="E76:E80"/>
     <mergeCell ref="E28:E29"/>
@@ -3841,34 +3852,32 @@
     <mergeCell ref="H43:H47"/>
     <mergeCell ref="K117:K120"/>
     <mergeCell ref="D81:D85"/>
+    <mergeCell ref="I7:I11"/>
     <mergeCell ref="J54:J63"/>
-    <mergeCell ref="I7:I11"/>
     <mergeCell ref="I81:I82"/>
-    <mergeCell ref="I97:I99"/>
     <mergeCell ref="J83:J85"/>
     <mergeCell ref="E109:E112"/>
     <mergeCell ref="E38:E42"/>
-    <mergeCell ref="C89:C99"/>
+    <mergeCell ref="E96:E99"/>
     <mergeCell ref="E2:K2"/>
     <mergeCell ref="J81:J82"/>
     <mergeCell ref="J103:J105"/>
+    <mergeCell ref="E89:E91"/>
     <mergeCell ref="B7:B47"/>
     <mergeCell ref="H113:H116"/>
     <mergeCell ref="J100:J102"/>
     <mergeCell ref="C33:C47"/>
     <mergeCell ref="J64:J71"/>
     <mergeCell ref="J28:J29"/>
-    <mergeCell ref="I89:I92"/>
     <mergeCell ref="D28:D32"/>
     <mergeCell ref="J19:J24"/>
     <mergeCell ref="A7:A120"/>
     <mergeCell ref="I28:I29"/>
-    <mergeCell ref="H89:H92"/>
     <mergeCell ref="E48:E53"/>
     <mergeCell ref="K113:K116"/>
-    <mergeCell ref="I54:I63"/>
     <mergeCell ref="E25:E27"/>
     <mergeCell ref="H30:H32"/>
+    <mergeCell ref="I54:I63"/>
     <mergeCell ref="K64:K71"/>
     <mergeCell ref="H12:H18"/>
     <mergeCell ref="E64:E71"/>
@@ -3880,12 +3889,14 @@
     <mergeCell ref="E83:E85"/>
     <mergeCell ref="K30:K32"/>
     <mergeCell ref="C48:C71"/>
+    <mergeCell ref="D92:D102"/>
+    <mergeCell ref="I92:I95"/>
     <mergeCell ref="E33:E37"/>
     <mergeCell ref="H38:H42"/>
     <mergeCell ref="J38:J42"/>
     <mergeCell ref="D7:D27"/>
+    <mergeCell ref="C103:C105"/>
     <mergeCell ref="D33:D47"/>
-    <mergeCell ref="C100:C102"/>
     <mergeCell ref="H83:H85"/>
     <mergeCell ref="E103:E105"/>
     <mergeCell ref="I103:I105"/>

</xml_diff>